<commit_message>
SSLC Option B: drop Counsel gates (Jon 10/7: still negotiating)
</commit_message>
<xml_diff>
--- a/drafts/EXOS_SSLC_OptionB_Acquisition_Model_2026-10-07.xlsx
+++ b/drafts/EXOS_SSLC_OptionB_Acquisition_Model_2026-10-07.xlsx
@@ -584,7 +584,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Prepared: 2026-10-07 | DRAFT — [Counsel review required] | INTERNAL — Exo/CEO only</t>
+          <t>Prepared: 2026-10-07 | DRAFT — NEGOTIATING TERMS | INTERNAL — Exo/CEO only</t>
         </is>
       </c>
     </row>
@@ -642,7 +642,7 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>FNEX advisory agreement — [Counsel: confirm binding]</t>
+          <t>FNEX advisory agreement; strengthen with investor/sponsor use-of-proceeds letter</t>
         </is>
       </c>
     </row>
@@ -1039,7 +1039,7 @@
     <row r="37" ht="22" customHeight="1">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>SSLC FY26 actual revenue (historical — reference only) ($)</t>
+          <t>SSLC FY26 actual revenue ($)</t>
         </is>
       </c>
       <c r="B37" s="8" t="n">
@@ -1264,15 +1264,15 @@
     <row r="52" ht="22" customHeight="1">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t>SSLC FY27 non-IM revenue (other work, billed-ahead conversion) ($)</t>
+          <t>v15 benchmark — SSLC acq revenue Y1 ($)</t>
         </is>
       </c>
       <c r="B52" s="8" t="n">
-        <v>500000</v>
+        <v>900000</v>
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>MANAGEMENT ASSUMPTION — FY27 Q1 actual K annualized; non-IM portion est. /bin/zsh.5M (IM is dominant FY27 driver)</t>
+          <t>Old acquisition model (pre-commission, pre-IM-tank confirmation); Option B should exceed</t>
         </is>
       </c>
     </row>
@@ -1669,6 +1669,7 @@
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
+      <c r="A14" t="inlineStr"/>
       <c r="E14" s="11" t="inlineStr"/>
     </row>
     <row r="15" ht="18" customHeight="1">
@@ -2979,7 +2980,7 @@
         </is>
       </c>
       <c r="B42" s="15">
-        <f>Assumptions!B44+500000</f>
+        <f>Assumptions!B37+Assumptions!B44</f>
         <v/>
       </c>
       <c r="C42" s="15">
@@ -3000,7 +3001,7 @@
       </c>
       <c r="H42" s="11" t="inlineStr">
         <is>
-          <t>IM tanks M firm (Markus 10/2) + /bin/zsh.5M non-IM other; FY28+ = management assumptions</t>
+          <t>SSLC actual + IM firm FY27; projections FY28+</t>
         </is>
       </c>
     </row>
@@ -4198,17 +4199,17 @@
     <row r="23" ht="28" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>Keyes (Counsel) review</t>
+          <t>Legal review</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Pre-send required</t>
+          <t>Deferred (Jon 10/7)</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>[[feedback_keyes_presignature_only]] — Counsel confirms §3 still in force + not 'agreement to agree'</t>
+          <t>Negotiation stage; no legal review until Jon calls it</t>
         </is>
       </c>
     </row>
@@ -4306,7 +4307,7 @@
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>[Counsel: insider lending — use only disclosed SSLC numbers] Option C held for follow-up</t>
+          <t>Use only disclosed SSLC numbers; Option C held for follow-up</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SSLC Option B: final no-Counsel rebuild
</commit_message>
<xml_diff>
--- a/drafts/EXOS_SSLC_OptionB_Acquisition_Model_2026-10-07.xlsx
+++ b/drafts/EXOS_SSLC_OptionB_Acquisition_Model_2026-10-07.xlsx
@@ -1517,7 +1517,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>Option B: invoke §3 exclusivity at $3.36M base + earn-out (IM tank revenue and/or Exos stock post-listing). SSLC debts paid at face. DRAFT — [Counsel review required].</t>
+          <t>Option B: invoke §3 exclusivity at $3.36M base + earn-out (IM tank revenue and/or Exos stock post-listing). SSLC debts paid at face. DRAFT — negotiation-stage terms.</t>
         </is>
       </c>
     </row>
@@ -4100,7 +4100,7 @@
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>[Counsel review] — [Confirm FNEX agreement countersigned per D-7281974 10/6]</t>
+          <t>[Confirm FNEX agreement countersigned per D-7281974 10/6]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SSLC Option B: Eqvista fix + 5-yr total comp chart (task #3544)
- Fix Eqvista status in build scripts + v2 draft: 'engaged 8/14/2026; agreement
  still unsigned (held ~1 month)' — replaces incorrect 'in progress' wording
- Add Total Compensation sheet to model xlsx (formulas linked to Assumptions)
- Add scripts/build_sslc_total_comp_chart.py: stacked bar FY27-FY31 with
  cumulative line; Exos brand palette (black/orange)
- Rebuild board summary (3pp): chart + 5-yr table embedded on page 3
- Rebuild v2 draft docx with corrected Eqvista bullet
- negotiating terms — management assumptions; SSLC debt unverified
</commit_message>
<xml_diff>
--- a/drafts/EXOS_SSLC_OptionB_Acquisition_Model_2026-10-07.xlsx
+++ b/drafts/EXOS_SSLC_OptionB_Acquisition_Model_2026-10-07.xlsx
@@ -12,6 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PL and Cash Flow" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Returns and Dilution" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Total Compensation" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26,7 +27,7 @@
     <numFmt numFmtId="166" formatCode="$#,##0;($#,##0)"/>
     <numFmt numFmtId="167" formatCode="0.0x"/>
   </numFmts>
-  <fonts count="16">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -97,8 +98,13 @@
       <b val="1"/>
       <color rgb="00FF8C00"/>
     </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -135,6 +141,26 @@
         <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00444444"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00666666"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E26A21"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -148,7 +174,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -201,6 +227,17 @@
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -4170,12 +4207,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Required (Eqvista engaged)</t>
+          <t>Required (Eqvista engaged 8/14/2026)</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>Eqvista engaged for 409A + fairness opinion per D1-D4 of record</t>
+          <t>Eqvista fairness opinion: engaged 8/14/2026; agreement still unsigned (held ~1 month)</t>
         </is>
       </c>
     </row>
@@ -4381,4 +4418,689 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="12" t="inlineStr">
+        <is>
+          <t>SSLC Option B — Total Compensation to SSLC Shareholders/Stakeholders (FY27–FY31)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="40" t="inlineStr">
+        <is>
+          <t>negotiating terms — management assumptions; SSLC debt unverified</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="41" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="B4" s="41" t="inlineStr">
+        <is>
+          <t>FY27 (Close)</t>
+        </is>
+      </c>
+      <c r="C4" s="41" t="inlineStr">
+        <is>
+          <t>FY28</t>
+        </is>
+      </c>
+      <c r="D4" s="41" t="inlineStr">
+        <is>
+          <t>FY29</t>
+        </is>
+      </c>
+      <c r="E4" s="41" t="inlineStr">
+        <is>
+          <t>FY30</t>
+        </is>
+      </c>
+      <c r="F4" s="41" t="inlineStr">
+        <is>
+          <t>FY31</t>
+        </is>
+      </c>
+      <c r="G4" s="41" t="inlineStr">
+        <is>
+          <t>5-Yr Total</t>
+        </is>
+      </c>
+      <c r="H4" s="41" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="42" t="inlineStr">
+        <is>
+          <t>FUNDING DELIVERED AT CLOSE (FY27)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="43" t="inlineStr">
+        <is>
+          <t>Cash at close</t>
+        </is>
+      </c>
+      <c r="B6" s="21">
+        <f>Assumptions!B10</f>
+        <v/>
+      </c>
+      <c r="C6" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="21">
+        <f>SUM(B6:F6)</f>
+        <v/>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>§3 deal price — cash component</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="43" t="inlineStr">
+        <is>
+          <t>SSLC closing costs</t>
+        </is>
+      </c>
+      <c r="B7" s="21">
+        <f>Assumptions!B11</f>
+        <v/>
+      </c>
+      <c r="C7" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="21">
+        <f>SUM(B7:F7)</f>
+        <v/>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
+        <is>
+          <t>Seller's costs (§3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="43" t="inlineStr">
+        <is>
+          <t>Exos stake credit (non-cash)</t>
+        </is>
+      </c>
+      <c r="B8" s="21">
+        <f>Assumptions!B12</f>
+        <v/>
+      </c>
+      <c r="C8" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="21">
+        <f>SUM(B8:F8)</f>
+        <v/>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>18% equity at 2021 basis; reduces cash out-of-pocket</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="43" t="inlineStr">
+        <is>
+          <t>SSLC debts paid at face (TBV)</t>
+        </is>
+      </c>
+      <c r="B9" s="21">
+        <f>Assumptions!B14</f>
+        <v/>
+      </c>
+      <c r="C9" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="21">
+        <f>SUM(B9:F9)</f>
+        <v/>
+      </c>
+      <c r="H9" s="7" t="inlineStr">
+        <is>
+          <t>Microcosm/Wertz notes + AP — TO VERIFY IN SSLC QB</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="43" t="inlineStr">
+        <is>
+          <t>Working-capital bridge</t>
+        </is>
+      </c>
+      <c r="B10" s="21">
+        <f>Assumptions!B16</f>
+        <v/>
+      </c>
+      <c r="C10" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="21">
+        <f>SUM(B10:F10)</f>
+        <v/>
+      </c>
+      <c r="H10" s="7" t="inlineStr">
+        <is>
+          <t>SSLC bridge to finish paid-for work (mid=$500K)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="44" t="inlineStr">
+        <is>
+          <t>TOTAL FUNDING DELIVERED</t>
+        </is>
+      </c>
+      <c r="B11" s="45">
+        <f>SUM(B6:B10)</f>
+        <v/>
+      </c>
+      <c r="C11" s="45">
+        <f>SUM(C6:C10)</f>
+        <v/>
+      </c>
+      <c r="D11" s="45">
+        <f>SUM(D6:D10)</f>
+        <v/>
+      </c>
+      <c r="E11" s="45">
+        <f>SUM(E6:E10)</f>
+        <v/>
+      </c>
+      <c r="F11" s="45">
+        <f>SUM(F6:F10)</f>
+        <v/>
+      </c>
+      <c r="G11" s="45">
+        <f>SUM(B11:F11)</f>
+        <v/>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
+        <is>
+          <t>All at close in FY27</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="46" t="inlineStr">
+        <is>
+          <t>FORWARD POTENTIAL — EARN-OUTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="43" t="inlineStr">
+        <is>
+          <t>Tank earn-out base (i): 5%/yr, $300K cap</t>
+        </is>
+      </c>
+      <c r="B14" s="21">
+        <f>MIN(Assumptions!B24*Assumptions!B44,Assumptions!B26)</f>
+        <v/>
+      </c>
+      <c r="C14" s="21">
+        <f>MIN(Assumptions!B24*Assumptions!B44,Assumptions!B26)</f>
+        <v/>
+      </c>
+      <c r="D14" s="21">
+        <f>MIN(Assumptions!B24*Assumptions!B44,Assumptions!B26)</f>
+        <v/>
+      </c>
+      <c r="E14" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="21">
+        <f>SUM(B14:F14)</f>
+        <v/>
+      </c>
+      <c r="H14" s="7" t="inlineStr">
+        <is>
+          <t>5% of SSLC IM tank revenue × 3 years; $300K/yr cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="43" t="inlineStr">
+        <is>
+          <t>Tank earn-out low (i): 3%/yr, $300K cap</t>
+        </is>
+      </c>
+      <c r="B15" s="21">
+        <f>MIN(Assumptions!B23*Assumptions!B44,Assumptions!B26)</f>
+        <v/>
+      </c>
+      <c r="C15" s="21">
+        <f>MIN(Assumptions!B23*Assumptions!B44,Assumptions!B26)</f>
+        <v/>
+      </c>
+      <c r="D15" s="21">
+        <f>MIN(Assumptions!B23*Assumptions!B44,Assumptions!B26)</f>
+        <v/>
+      </c>
+      <c r="E15" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="21">
+        <f>SUM(B15:F15)</f>
+        <v/>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
+        <is>
+          <t>Low scenario: 3%/yr</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="43" t="inlineStr">
+        <is>
+          <t>Tank earn-out high (i): 7%/yr, $300K cap</t>
+        </is>
+      </c>
+      <c r="B16" s="21">
+        <f>MIN(Assumptions!B25*Assumptions!B44,Assumptions!B26)</f>
+        <v/>
+      </c>
+      <c r="C16" s="21">
+        <f>MIN(Assumptions!B25*Assumptions!B44,Assumptions!B26)</f>
+        <v/>
+      </c>
+      <c r="D16" s="21">
+        <f>MIN(Assumptions!B25*Assumptions!B44,Assumptions!B26)</f>
+        <v/>
+      </c>
+      <c r="E16" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="21">
+        <f>SUM(B16:F16)</f>
+        <v/>
+      </c>
+      <c r="H16" s="7" t="inlineStr">
+        <is>
+          <t>High scenario: 7%/yr — capped at $300K</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="43" t="inlineStr">
+        <is>
+          <t>Stock earn-out base (ii): 0.5% FD @ listing</t>
+        </is>
+      </c>
+      <c r="B17" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="21">
+        <f>Assumptions!B29*Assumptions!B32</f>
+        <v/>
+      </c>
+      <c r="E17" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="21">
+        <f>SUM(B17:F17)</f>
+        <v/>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>At listing ($250M base) + 12-mo lockup → realized FY29</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="43" t="inlineStr">
+        <is>
+          <t>Stock earn-out low (ii): 0.3% @ $200M</t>
+        </is>
+      </c>
+      <c r="B18" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="21">
+        <f>Assumptions!B28*Assumptions!B31</f>
+        <v/>
+      </c>
+      <c r="E18" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="21">
+        <f>SUM(B18:F18)</f>
+        <v/>
+      </c>
+      <c r="H18" s="7" t="inlineStr">
+        <is>
+          <t>Low RTO scenario</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="43" t="inlineStr">
+        <is>
+          <t>Stock earn-out high (ii): 0.7% @ $300M</t>
+        </is>
+      </c>
+      <c r="B19" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="21">
+        <f>Assumptions!B30*Assumptions!B33</f>
+        <v/>
+      </c>
+      <c r="E19" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="21">
+        <f>SUM(B19:F19)</f>
+        <v/>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>High RTO scenario</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL CONSIDERATION (Base price + earn-out + debts; base/low/high)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="16" t="inlineStr">
+        <is>
+          <t>TOTAL (Base): funding + tank base + stock base</t>
+        </is>
+      </c>
+      <c r="B22" s="47">
+        <f>B11+B14+B17</f>
+        <v/>
+      </c>
+      <c r="C22" s="47">
+        <f>C11+C14+C17</f>
+        <v/>
+      </c>
+      <c r="D22" s="47">
+        <f>D11+D14+D17</f>
+        <v/>
+      </c>
+      <c r="E22" s="47">
+        <f>E11+E14+E17</f>
+        <v/>
+      </c>
+      <c r="F22" s="47">
+        <f>F11+F14+F17</f>
+        <v/>
+      </c>
+      <c r="G22" s="47">
+        <f>SUM(B22:F22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="16" t="inlineStr">
+        <is>
+          <t>TOTAL (Low):  funding + tank low  + stock low</t>
+        </is>
+      </c>
+      <c r="B23" s="47">
+        <f>B11+B15+B18</f>
+        <v/>
+      </c>
+      <c r="C23" s="47">
+        <f>C11+C15+C18</f>
+        <v/>
+      </c>
+      <c r="D23" s="47">
+        <f>D11+D15+D18</f>
+        <v/>
+      </c>
+      <c r="E23" s="47">
+        <f>E11+E15+E18</f>
+        <v/>
+      </c>
+      <c r="F23" s="47">
+        <f>F11+F15+F18</f>
+        <v/>
+      </c>
+      <c r="G23" s="47">
+        <f>SUM(B23:F23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="16" t="inlineStr">
+        <is>
+          <t>TOTAL (High): funding + tank high + stock high</t>
+        </is>
+      </c>
+      <c r="B24" s="47">
+        <f>B11+B16+B19</f>
+        <v/>
+      </c>
+      <c r="C24" s="47">
+        <f>C11+C16+C19</f>
+        <v/>
+      </c>
+      <c r="D24" s="47">
+        <f>D11+D16+D19</f>
+        <v/>
+      </c>
+      <c r="E24" s="47">
+        <f>E11+E16+E19</f>
+        <v/>
+      </c>
+      <c r="F24" s="47">
+        <f>F11+F16+F19</f>
+        <v/>
+      </c>
+      <c r="G24" s="47">
+        <f>SUM(B24:F24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="16" t="inlineStr">
+        <is>
+          <t>5-Yr TOTAL BASE</t>
+        </is>
+      </c>
+      <c r="B25" s="47">
+        <f>B22</f>
+        <v/>
+      </c>
+      <c r="C25" s="47">
+        <f>C22</f>
+        <v/>
+      </c>
+      <c r="D25" s="47">
+        <f>D22</f>
+        <v/>
+      </c>
+      <c r="E25" s="47">
+        <f>E22</f>
+        <v/>
+      </c>
+      <c r="F25" s="47">
+        <f>F22</f>
+        <v/>
+      </c>
+      <c r="G25" s="47">
+        <f>SUM(B25:F25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="48" t="inlineStr">
+        <is>
+          <t>FUNDING vs FORWARD SPLIT (5-Year)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Funding delivered (at close, fixed)</t>
+        </is>
+      </c>
+      <c r="B28" s="8">
+        <f>B11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>Forward potential (earn-outs, base)</t>
+        </is>
+      </c>
+      <c r="B29" s="8">
+        <f>B14*3+B17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>Forward potential (earn-outs, low)</t>
+        </is>
+      </c>
+      <c r="B30" s="8">
+        <f>B15*3+B18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>Forward potential (earn-outs, high)</t>
+        </is>
+      </c>
+      <c r="B31" s="8">
+        <f>B16*3+B19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="11" t="inlineStr">
+        <is>
+          <t>Chart: see drafts/SSLC_OptionB_Total_Compensation_5yr_2026-10-07.png</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A21:H21"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A13:H13"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="A27:H27"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
SSLC Option B: remove prepaid-work line, raise stock earn-out to 0.5–1.0% (Jon 10/7 15:22)
- Prepaid-work relief line removed from all scripts and outputs
  (Jon: figure accruing incorrectly; K not a valid delivery obligation)
- Working-capital bridge (K) kept (pre-dated the prepaid addition)
- Stock earn-out: low 0.5%, base 0.75%, high 1.0% FD shares
  (was 0.3/0.5/0.7%)
- At-listing values: L $1.0M / B $1.875M / H $3.0M
- Y5 post-dilution stakes: 0.35% / 0.525% / 0.70%
- Y5 v12 hold: L $5.69M / B $8.54M / H $11.38M
- Y5 AA hold: L $616K / B $924K / H $1.23M
- 5-yr totals: L $5.81M / B $6.985M / H $8.26M
- Files re-attached to MC task 3544
</commit_message>
<xml_diff>
--- a/drafts/EXOS_SSLC_OptionB_Acquisition_Model_2026-10-07.xlsx
+++ b/drafts/EXOS_SSLC_OptionB_Acquisition_Model_2026-10-07.xlsx
@@ -1246,7 +1246,7 @@
         </is>
       </c>
       <c r="B28" s="9" t="n">
-        <v>0.003</v>
+        <v>0.005</v>
       </c>
       <c r="C28" s="10" t="inlineStr">
         <is>
@@ -1261,7 +1261,7 @@
         </is>
       </c>
       <c r="B29" s="9" t="n">
-        <v>0.005</v>
+        <v>0.0075</v>
       </c>
       <c r="C29" s="10" t="inlineStr">
         <is>
@@ -1276,7 +1276,7 @@
         </is>
       </c>
       <c r="B30" s="9" t="n">
-        <v>0.007</v>
+        <v>0.01</v>
       </c>
       <c r="C30" s="10" t="inlineStr">
         <is>
@@ -2194,73 +2194,6 @@
         </is>
       </c>
     </row>
-    <row r="99" ht="20" customHeight="1">
-      <c r="A99" s="4" t="inlineStr">
-        <is>
-          <t>PREPAID-WORK DELIVERY OBLIGATION (Jon 10/7)</t>
-        </is>
-      </c>
-    </row>
-    <row r="100" ht="22" customHeight="1">
-      <c r="A100" s="5" t="inlineStr">
-        <is>
-          <t>SSLC prepaid-work face value — billed-ahead + deposits ($)</t>
-        </is>
-      </c>
-      <c r="B100" s="8" t="n">
-        <v>984000</v>
-      </c>
-      <c r="C100" s="7" t="inlineStr">
-        <is>
-          <t>per 10/2 SSLC QB pull; verify. $864K billed-ahead + $120K deposits.</t>
-        </is>
-      </c>
-    </row>
-    <row r="101" ht="22" customHeight="1">
-      <c r="A101" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  of which: billed-ahead ($)</t>
-        </is>
-      </c>
-      <c r="B101" s="8" t="n">
-        <v>864000</v>
-      </c>
-      <c r="C101" s="7" t="inlineStr">
-        <is>
-          <t>per 10/2 SSLC QB pull; verify</t>
-        </is>
-      </c>
-    </row>
-    <row r="102" ht="22" customHeight="1">
-      <c r="A102" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  of which: deposits ($)</t>
-        </is>
-      </c>
-      <c r="B102" s="8" t="n">
-        <v>120000</v>
-      </c>
-      <c r="C102" s="7" t="inlineStr">
-        <is>
-          <t>per 10/2 SSLC QB pull; verify</t>
-        </is>
-      </c>
-    </row>
-    <row r="103" ht="22" customHeight="1">
-      <c r="A103" s="5" t="inlineStr">
-        <is>
-          <t>Cost to Exos to fund completion (mid = WC bridge) ($)</t>
-        </is>
-      </c>
-      <c r="B103" s="8" t="n">
-        <v>500000</v>
-      </c>
-      <c r="C103" s="7" t="inlineStr">
-        <is>
-          <t>Same as B16 — $0.3–$0.7M to finish paid-for IM work; mid=$500K</t>
-        </is>
-      </c>
-    </row>
     <row r="105" ht="20" customHeight="1">
       <c r="A105" s="4" t="inlineStr">
         <is>
@@ -2288,117 +2221,100 @@
     <row r="107" ht="20" customHeight="1">
       <c r="A107" s="5" t="inlineStr">
         <is>
-          <t>2. Delivery obligations assumed &amp; funded</t>
+          <t>2. No further capital calls</t>
         </is>
       </c>
       <c r="B107" s="5" t="inlineStr">
         <is>
-          <t>$984K face/$500K cost</t>
+          <t>Structural</t>
         </is>
       </c>
       <c r="C107" s="7" t="inlineStr">
         <is>
-          <t>Exos funds completion; per 10/2 QB pull; verify</t>
+          <t>Investors stop funding a cash-negative entity</t>
         </is>
       </c>
     </row>
     <row r="108" ht="20" customHeight="1">
       <c r="A108" s="5" t="inlineStr">
         <is>
-          <t>3. No further capital calls</t>
+          <t>3. Cash at close</t>
         </is>
       </c>
       <c r="B108" s="5" t="inlineStr">
         <is>
-          <t>Structural</t>
+          <t>$2,510,000</t>
         </is>
       </c>
       <c r="C108" s="7" t="inlineStr">
         <is>
-          <t>Investors stop funding a cash-negative entity</t>
+          <t>Section 3 deal price cash component</t>
         </is>
       </c>
     </row>
     <row r="109" ht="20" customHeight="1">
       <c r="A109" s="5" t="inlineStr">
         <is>
-          <t>4. Cash at close</t>
+          <t>4. Earn-out upside — IM tank revenue (3 yrs)</t>
         </is>
       </c>
       <c r="B109" s="5" t="inlineStr">
         <is>
-          <t>$2,510,000</t>
+          <t>Up to $900K</t>
         </is>
       </c>
       <c r="C109" s="7" t="inlineStr">
         <is>
-          <t>Section 3 deal price cash component</t>
+          <t>5%/yr x $5M IM firm; $300K cap</t>
         </is>
       </c>
     </row>
     <row r="110" ht="20" customHeight="1">
       <c r="A110" s="5" t="inlineStr">
         <is>
-          <t>5. Earn-out upside — IM tank revenue (3 yrs)</t>
+          <t>5. Earn-out upside — Exos stock post-RTO</t>
         </is>
       </c>
       <c r="B110" s="5" t="inlineStr">
         <is>
-          <t>Up to $900K</t>
+          <t>$1.0M–$3.0M</t>
         </is>
       </c>
       <c r="C110" s="7" t="inlineStr">
         <is>
-          <t>5%/yr x $5M IM firm; $300K cap</t>
+          <t>0.5%–1.0% FD at listing ($200M–$300M MEV)</t>
         </is>
       </c>
     </row>
     <row r="111" ht="20" customHeight="1">
       <c r="A111" s="5" t="inlineStr">
         <is>
-          <t>6. Earn-out upside — Exos stock post-RTO</t>
+          <t>6. Liquidity via listed Exos stock</t>
         </is>
       </c>
       <c r="B111" s="5" t="inlineStr">
         <is>
-          <t>$0.6M–$2.1M</t>
+          <t>Post-RTO ~FY28</t>
         </is>
       </c>
       <c r="C111" s="7" t="inlineStr">
         <is>
-          <t>0.3–0.7% FD at listing ($200M–$300M MEV)</t>
+          <t>12-mo lockup; publicly tradeable thereafter</t>
         </is>
       </c>
     </row>
     <row r="112" ht="20" customHeight="1">
       <c r="A112" s="5" t="inlineStr">
         <is>
-          <t>7. Liquidity via listed Exos stock</t>
+          <t>7. IM program continuity</t>
         </is>
       </c>
       <c r="B112" s="5" t="inlineStr">
         <is>
-          <t>Post-RTO ~FY28</t>
+          <t>Operational</t>
         </is>
       </c>
       <c r="C112" s="7" t="inlineStr">
-        <is>
-          <t>12-mo lockup; publicly tradeable thereafter</t>
-        </is>
-      </c>
-    </row>
-    <row r="113" ht="20" customHeight="1">
-      <c r="A113" s="5" t="inlineStr">
-        <is>
-          <t>8. IM program continuity</t>
-        </is>
-      </c>
-      <c r="B113" s="5" t="inlineStr">
-        <is>
-          <t>Operational</t>
-        </is>
-      </c>
-      <c r="C113" s="7" t="inlineStr">
         <is>
           <t>No customer disruption; Exos-SSLC entity delivers</t>
         </is>
@@ -2495,11 +2411,11 @@
         </is>
       </c>
       <c r="B121" s="20" t="n">
-        <v>0.005</v>
+        <v>0.0075</v>
       </c>
       <c r="C121" s="19" t="inlineStr">
         <is>
-          <t>Base earn-out grant = 0.5% FD shares at listing</t>
+          <t>Base earn-out grant = 0.75% FD shares at listing</t>
         </is>
       </c>
     </row>
@@ -2546,7 +2462,7 @@
       </c>
       <c r="C124" s="19" t="inlineStr">
         <is>
-          <t>0.5% x 0.70 = 0.35%</t>
+          <t>0.75% x 0.70 = 0.525%</t>
         </is>
       </c>
     </row>
@@ -2562,7 +2478,7 @@
       </c>
       <c r="C125" s="19" t="inlineStr">
         <is>
-          <t>0.3% x 0.70 = 0.21%</t>
+          <t>0.5% x 0.70 = 0.35%</t>
         </is>
       </c>
     </row>
@@ -2578,7 +2494,7 @@
       </c>
       <c r="C126" s="19" t="inlineStr">
         <is>
-          <t>0.7% x 0.70 = 0.49%</t>
+          <t>1.0% x 0.70 = 0.70%</t>
         </is>
       </c>
     </row>
@@ -2594,7 +2510,7 @@
       </c>
       <c r="C127" s="19" t="inlineStr">
         <is>
-          <t>~$3.41M</t>
+          <t>~$5.69M</t>
         </is>
       </c>
     </row>
@@ -2610,7 +2526,7 @@
       </c>
       <c r="C128" s="19" t="inlineStr">
         <is>
-          <t>~$5.69M</t>
+          <t>~$8.54M</t>
         </is>
       </c>
     </row>
@@ -2626,7 +2542,7 @@
       </c>
       <c r="C129" s="19" t="inlineStr">
         <is>
-          <t>~$7.97M</t>
+          <t>~$11.38M</t>
         </is>
       </c>
     </row>
@@ -2642,7 +2558,7 @@
       </c>
       <c r="C130" s="19" t="inlineStr">
         <is>
-          <t>~$370K</t>
+          <t>~$616K</t>
         </is>
       </c>
     </row>
@@ -2658,7 +2574,7 @@
       </c>
       <c r="C131" s="19" t="inlineStr">
         <is>
-          <t>~$616K</t>
+          <t>~$924K</t>
         </is>
       </c>
     </row>
@@ -2674,7 +2590,7 @@
       </c>
       <c r="C132" s="19" t="inlineStr">
         <is>
-          <t>~$862K</t>
+          <t>~$1.23M</t>
         </is>
       </c>
     </row>
@@ -2690,7 +2606,7 @@
       </c>
       <c r="C133" s="19" t="inlineStr">
         <is>
-          <t>~4.5x the at-listing stock earn-out value ($1.25M)</t>
+          <t>~4.6x the at-listing stock earn-out value ($1.875M)</t>
         </is>
       </c>
     </row>
@@ -2713,13 +2629,12 @@
     <row r="136" ht="42" customHeight="1">
       <c r="A136" s="17" t="inlineStr">
         <is>
-          <t>WARNING: AA CASE Y5 HOLD — Actuals-Anchored FY31 EV (~$176M) is BELOW the $250M RTO listing value. In the AA case, holding to FY31 yields LESS than the at-listing earn-out. This reflects conservative actuals-based projections, not a flaw in the deal. Old-Model (v12) FY31 EV ~$1.63B yields ~4.5x the at-listing stock value.</t>
+          <t>WARNING: AA CASE Y5 HOLD — Actuals-Anchored FY31 EV (~$176M) is BELOW the $250M RTO listing value. In the AA case, holding to FY31 yields LESS than the at-listing earn-out. This reflects conservative actuals-based projections, not a flaw in the deal. Old-Model (v12) FY31 EV ~$1.63B yields ~4.6x the at-listing stock value.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="13">
-    <mergeCell ref="A99:C99"/>
+  <mergeCells count="12">
     <mergeCell ref="A115:C115"/>
     <mergeCell ref="A36:C36"/>
     <mergeCell ref="A71:C71"/>
@@ -3069,7 +2984,7 @@
       </c>
       <c r="E24" s="10" t="inlineStr">
         <is>
-          <t>Low: 3% tank rev (cap $300K) × 3yr + 0.3% of $200M listing</t>
+          <t>Low: 3% tank rev (cap $300K) × 3yr + 0.5% of $200M listing</t>
         </is>
       </c>
     </row>
@@ -3093,7 +3008,7 @@
       </c>
       <c r="E25" s="10" t="inlineStr">
         <is>
-          <t>Base: 5% × $5M firm + 0.5% of $250M listing</t>
+          <t>Base: 5% × $5M firm + 0.75% of $250M listing</t>
         </is>
       </c>
     </row>
@@ -3117,7 +3032,7 @@
       </c>
       <c r="E26" s="10" t="inlineStr">
         <is>
-          <t>High: 7% × $5M + 0.7% of $300M listing</t>
+          <t>High: 7% × $5M + 1.0% of $300M listing</t>
         </is>
       </c>
     </row>
@@ -3142,7 +3057,7 @@
       </c>
       <c r="E27" s="10" t="inlineStr">
         <is>
-          <t>0.5% of FD shares; non-material at Series A scale</t>
+          <t>0.75% of FD shares; non-material at Series A scale</t>
         </is>
       </c>
     </row>
@@ -5540,7 +5455,7 @@
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>Cash $198K + collections on $984K prepaid</t>
+          <t>Cash $198K + collections on billed-ahead work; ~1 month burn</t>
         </is>
       </c>
     </row>
@@ -5846,11 +5761,11 @@
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="58" t="inlineStr">
         <is>
-          <t>Prepaid-work delivery obligations assumed</t>
+          <t>Working-capital bridge (completion cost)</t>
         </is>
       </c>
       <c r="B10" s="31">
-        <f>Assumptions!B100</f>
+        <f>Assumptions!B16</f>
         <v/>
       </c>
       <c r="C10" s="31" t="n">
@@ -5871,39 +5786,7 @@
       </c>
       <c r="H10" s="10" t="inlineStr">
         <is>
-          <t>$984K face (billed-ahead $864K + deposits $120K); per 10/2 SSLC QB pull; verify</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="58" t="inlineStr">
-        <is>
-          <t>Working-capital bridge (completion cost)</t>
-        </is>
-      </c>
-      <c r="B11" s="31">
-        <f>Assumptions!B16</f>
-        <v/>
-      </c>
-      <c r="C11" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" s="31">
-        <f>SUM(B11:F11)</f>
-        <v/>
-      </c>
-      <c r="H11" s="10" t="inlineStr">
-        <is>
-          <t>Mid=$500K; funds completion of prepaid IM work</t>
+          <t>Mid=$500K; funds completion of in-flight IM work</t>
         </is>
       </c>
     </row>
@@ -5914,23 +5797,23 @@
         </is>
       </c>
       <c r="B12" s="60">
-        <f>SUM(B6:B11)</f>
+        <f>SUM(B6:B10)</f>
         <v/>
       </c>
       <c r="C12" s="60">
-        <f>SUM(C6:C11)</f>
+        <f>SUM(C6:C10)</f>
         <v/>
       </c>
       <c r="D12" s="60">
-        <f>SUM(D6:D11)</f>
+        <f>SUM(D6:D10)</f>
         <v/>
       </c>
       <c r="E12" s="60">
-        <f>SUM(E6:E11)</f>
+        <f>SUM(E6:E10)</f>
         <v/>
       </c>
       <c r="F12" s="60">
-        <f>SUM(F6:F11)</f>
+        <f>SUM(F6:F10)</f>
         <v/>
       </c>
       <c r="G12" s="60">
@@ -6055,7 +5938,7 @@
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="58" t="inlineStr">
         <is>
-          <t>Stock earn-out base (ii): 0.5% FD @ listing</t>
+          <t>Stock earn-out base (ii): 0.75% FD @ listing</t>
         </is>
       </c>
       <c r="B17" s="31" t="n">
@@ -6087,7 +5970,7 @@
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="58" t="inlineStr">
         <is>
-          <t>Stock earn-out low (ii): 0.3% @ $200M</t>
+          <t>Stock earn-out low (ii): 0.5% @ $200M</t>
         </is>
       </c>
       <c r="B18" s="31" t="n">
@@ -6119,7 +6002,7 @@
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="58" t="inlineStr">
         <is>
-          <t>Stock earn-out high (ii): 0.7% @ $300M</t>
+          <t>Stock earn-out high (ii): 1.0% @ $300M</t>
         </is>
       </c>
       <c r="B19" s="31" t="n">
@@ -6282,7 +6165,7 @@
     <row r="27">
       <c r="A27" s="10" t="inlineStr">
         <is>
-          <t>Chart: see drafts/SSLC_OptionB_Total_Compensation_5yr_2026-10-07.png (incl prepaid-work + Y5 hold annotation)</t>
+          <t>Chart: see drafts/SSLC_OptionB_Total_Compensation_5yr_2026-10-07.png (incl Y5 hold annotation)</t>
         </is>
       </c>
     </row>
@@ -6296,7 +6179,7 @@
     <row r="30" ht="32" customHeight="1">
       <c r="A30" s="68" t="inlineStr">
         <is>
-          <t>Base = Old-Model (v12). Dilution: Series A $25M staged (D1-D4, ~13%) + RTO (~12%) + option pool (~5%) = ~30% flat (MANAGEMENT ASSUMPTION). 0.5% stake at listing → 0.35% post-dilution. AA case EV ~$176M = BELOW $250M listing — stock worth less in AA case by FY31.</t>
+          <t>Base = Old-Model (v12). Dilution: Series A $25M staged (D1-D4, ~13%) + RTO (~12%) + option pool (~5%) = ~30% flat (MANAGEMENT ASSUMPTION). 0.75% stake at listing → 0.525% post-dilution. AA case EV ~$176M = BELOW $250M listing — stock worth less in AA case by FY31.</t>
         </is>
       </c>
     </row>
@@ -6366,7 +6249,7 @@
       </c>
       <c r="H32" s="71" t="inlineStr">
         <is>
-          <t>0.3% grant x 0.70 = 0.21%; EV $1.626B</t>
+          <t>0.5% grant x 0.70 = 0.35%; EV $1.626B</t>
         </is>
       </c>
     </row>
@@ -6398,7 +6281,7 @@
       </c>
       <c r="H33" s="71" t="inlineStr">
         <is>
-          <t>0.5% grant x 0.70 = 0.35%; EV $1.626B (~4.5x listing)</t>
+          <t>0.75% grant x 0.70 = 0.525%; EV $1.626B (~4.6x listing)</t>
         </is>
       </c>
     </row>
@@ -6430,7 +6313,7 @@
       </c>
       <c r="H34" s="71" t="inlineStr">
         <is>
-          <t>0.7% grant x 0.70 = 0.49%; EV $1.626B</t>
+          <t>1.0% grant x 0.70 = 0.70%; EV $1.626B</t>
         </is>
       </c>
     </row>
@@ -6494,7 +6377,7 @@
       </c>
       <c r="H36" s="71" t="inlineStr">
         <is>
-          <t>BELOW listing — ~$616K vs $1.25M at listing (~0.49x)</t>
+          <t>BELOW listing — ~$924K vs $1.875M at listing (~0.49x)</t>
         </is>
       </c>
     </row>
@@ -6526,14 +6409,14 @@
       </c>
       <c r="H37" s="71" t="inlineStr">
         <is>
-          <t>BELOW listing — ~$862K vs $2.1M at listing (~0.41x)</t>
+          <t>BELOW listing — ~$1.23M vs $3.0M at listing (~0.41x)</t>
         </is>
       </c>
     </row>
     <row r="39" ht="42" customHeight="1">
       <c r="A39" s="73" t="inlineStr">
         <is>
-          <t>NOTE: Y5 hold values are NOT additive to at-listing earn-out. Investors choose to hold OR sell at listing. Old-Model base: hold to FY31 = ~$5.69M vs sell at listing = $1.25M (4.5x). AA base: hold to FY31 = ~$0.62M vs sell at listing = $1.25M (0.49x) — AA case penalizes holding.</t>
+          <t>NOTE: Y5 hold values are NOT additive to at-listing earn-out. Investors choose to hold OR sell at listing. Old-Model base: hold to FY31 = ~$8.54M vs sell at listing = $1.875M (4.6x). AA base: hold to FY31 = ~$0.92M vs sell at listing = $1.875M (0.49x) — AA case penalizes holding.</t>
         </is>
       </c>
     </row>
@@ -6998,7 +6881,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L41"/>
+  <dimension ref="A1:L40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -7053,7 +6936,7 @@
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="82" t="inlineStr">
         <is>
-          <t>Constraints: Cash $198K | $984K prepaid work needs $300–700K to complete | FY26 op loss −$416K | He-tank rework unresolved | No capex | No IM ramp capital → growth capped by self-funded working capital</t>
+          <t>Constraints: Cash $198K | ~1 month burn | WC bridge $300–700K needed | FY26 op loss −$416K | He-tank rework unresolved | No capex | No IM ramp capital → growth capped by self-funded working capital</t>
         </is>
       </c>
       <c r="H9" s="83" t="inlineStr">
@@ -7118,7 +7001,7 @@
       </c>
       <c r="H11" s="85" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Prepaid work to deliver:  $984K face</t>
+          <t xml:space="preserve">  Working capital needed to maintain deliveries:  $300K–$700K</t>
         </is>
       </c>
     </row>
@@ -7143,7 +7026,7 @@
       </c>
       <c r="H12" s="85" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Cost to complete that work:  $300K–$700K</t>
+          <t xml:space="preserve">  FY26 operating loss:  −$416K</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7053,7 @@
       </c>
       <c r="H13" s="85" t="inlineStr">
         <is>
-          <t xml:space="preserve">  FY26 operating loss:  −$416K</t>
+          <t xml:space="preserve">  He-tank rework unresolved — no resolution path without new owner</t>
         </is>
       </c>
     </row>
@@ -7197,26 +7080,26 @@
       </c>
       <c r="H14" s="85" t="inlineStr">
         <is>
-          <t xml:space="preserve">  He-tank rework unresolved — no resolution path without new owner</t>
+          <t xml:space="preserve">  No capex capacity → headcount/equipment frozen</t>
         </is>
       </c>
     </row>
     <row r="15" ht="16" customHeight="1">
       <c r="A15" s="94" t="inlineStr">
         <is>
-          <t>⚠  Stall Risk: SSLC needs $300–700K to deliver $984K prepaid/deposited work already billed. On $198K cash, a working-capital crunch could interrupt deliveries in Q2–Q3 FY27, reducing FY27 below the $2.85M run-rate. The 10% CAGR assumes the crunch is survived.</t>
+          <t>⚠  Stall Risk: SSLC needs $300–700K in working capital to maintain delivery commitments. On $198K cash, a working-capital crunch could interrupt deliveries in Q2–Q3 FY27, reducing FY27 below the $2.85M run-rate. The 10% CAGR assumes the crunch is survived.</t>
         </is>
       </c>
       <c r="H15" s="85" t="inlineStr">
         <is>
-          <t xml:space="preserve">  No capex capacity → headcount/equipment frozen</t>
+          <t xml:space="preserve">  Growth capped by self-funded working capital</t>
         </is>
       </c>
     </row>
     <row r="16" ht="16" customHeight="1">
       <c r="H16" s="85" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Growth capped by self-funded working capital</t>
+          <t xml:space="preserve">  FY27 achievable at run-rate:  ~$2.85M</t>
         </is>
       </c>
     </row>
@@ -7228,23 +7111,23 @@
       </c>
       <c r="H17" s="85" t="inlineStr">
         <is>
-          <t xml:space="preserve">  FY27 achievable at run-rate:  ~$2.85M</t>
+          <t xml:space="preserve">  FY31 best-case (10% CAGR, no stall):  ~$4.2M</t>
         </is>
       </c>
     </row>
     <row r="18" ht="16" customHeight="1">
       <c r="A18" s="96" t="inlineStr">
         <is>
-          <t>Exos offer provides: Cash at close $2.51M | Debts paid at face | $984K prepaid-work funded (cost $500K) | WC bridge | Exos channel + IM ramp capex | v12 tank-unit/ASP ramp model. Figures: v12 Annual P&amp;L, recalculated 2026-10-07.</t>
+          <t>Exos offer provides: Cash at close $2.51M | Debts paid at face | WC bridge ($300–700K) | Exos channel + IM ramp capex | v12 tank-unit/ASP ramp model. Figures: v12 Annual P&amp;L, recalculated 2026-10-07.</t>
         </is>
       </c>
       <c r="H18" s="85" t="inlineStr">
         <is>
-          <t xml:space="preserve">  FY31 best-case (10% CAGR, no stall):  ~$4.2M</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="16" customHeight="1">
+          <t xml:space="preserve">  5-yr CAGR (status quo):  ~10.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1">
       <c r="A19" s="84" t="inlineStr"/>
       <c r="B19" s="84" t="inlineStr">
         <is>
@@ -7271,13 +7154,8 @@
           <t>FY31</t>
         </is>
       </c>
-      <c r="H19" s="85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  5-yr CAGR (status quo):  ~10.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
+    </row>
+    <row r="20" ht="20" customHeight="1">
       <c r="A20" s="86" t="inlineStr">
         <is>
           <t>SSLC Revenue (with Exos, v12)</t>
@@ -7298,8 +7176,13 @@
       <c r="F20" s="97" t="n">
         <v>54690000</v>
       </c>
-    </row>
-    <row r="21" ht="20" customHeight="1">
+      <c r="H20" s="98" t="inlineStr">
+        <is>
+          <t>With Exos: What Capital Unlocks</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="16" customHeight="1">
       <c r="A21" s="86" t="inlineStr">
         <is>
           <t xml:space="preserve">  YoY Revenue Growth</t>
@@ -7318,9 +7201,9 @@
       <c r="F21" s="88" t="n">
         <v>0.614</v>
       </c>
-      <c r="H21" s="98" t="inlineStr">
-        <is>
-          <t>With Exos: What Capital Unlocks</t>
+      <c r="H21" s="85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Cash at close:  $2.51M</t>
         </is>
       </c>
     </row>
@@ -7347,7 +7230,7 @@
       </c>
       <c r="H22" s="85" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Cash at close:  $2.51M</t>
+          <t xml:space="preserve">  SSLC debts paid at face (est. ~$500K TBV)</t>
         </is>
       </c>
     </row>
@@ -7374,14 +7257,14 @@
       </c>
       <c r="H23" s="85" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SSLC debts paid at face (est. ~$500K TBV)</t>
+          <t xml:space="preserve">  Prepaid-work delivery funded (cost $500K)</t>
         </is>
       </c>
     </row>
     <row r="24" ht="16" customHeight="1">
       <c r="H24" s="85" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Prepaid-work delivery funded (cost $500K)</t>
+          <t xml:space="preserve">  WC bridge removes Q2–Q3 stall risk</t>
         </is>
       </c>
     </row>
@@ -7393,7 +7276,7 @@
       </c>
       <c r="H25" s="85" t="inlineStr">
         <is>
-          <t xml:space="preserve">  WC bridge removes Q2–Q3 stall risk</t>
+          <t xml:space="preserve">  Exos procurement channel:  immediate BLK3 tank POs</t>
         </is>
       </c>
     </row>
@@ -7425,7 +7308,7 @@
       </c>
       <c r="H26" s="85" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Exos procurement channel:  immediate BLK3 tank POs</t>
+          <t xml:space="preserve">  Intuitive Machines ramp:  14–16 tanks firm FY27</t>
         </is>
       </c>
     </row>
@@ -7443,7 +7326,7 @@
       </c>
       <c r="H27" s="85" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Intuitive Machines ramp:  14–16 tanks firm FY27</t>
+          <t xml:space="preserve">  Capex for production scale-up enabled</t>
         </is>
       </c>
     </row>
@@ -7461,7 +7344,7 @@
       </c>
       <c r="H28" s="85" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Capex for production scale-up enabled</t>
+          <t xml:space="preserve">  FY27 target (IM firm + ramp):  $4.1M–$5.5M</t>
         </is>
       </c>
     </row>
@@ -7479,7 +7362,7 @@
       </c>
       <c r="H29" s="85" t="inlineStr">
         <is>
-          <t xml:space="preserve">  FY27 target (IM firm + ramp):  $4.1M–$5.5M</t>
+          <t xml:space="preserve">  FY31 (v12 trajectory):  $54.7M</t>
         </is>
       </c>
     </row>
@@ -7497,11 +7380,11 @@
       </c>
       <c r="H30" s="85" t="inlineStr">
         <is>
-          <t xml:space="preserve">  FY31 (v12 trajectory):  $54.7M</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="16" customHeight="1">
+          <t xml:space="preserve">  5-yr CAGR (with Exos, v12):  ~90.9%</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
       <c r="A31" s="101" t="inlineStr">
         <is>
           <t>Y5 Annual Revenue Gap (With − W/O)</t>
@@ -7511,13 +7394,8 @@
       <c r="C31" s="103" t="n">
         <v>50516000</v>
       </c>
-      <c r="H31" s="85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  5-yr CAGR (with Exos, v12):  ~90.9%</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
+    </row>
+    <row r="32" ht="20" customHeight="1">
       <c r="A32" s="101" t="inlineStr">
         <is>
           <t>Cumulative 5-yr Gap (With − W/O)</t>
@@ -7527,67 +7405,63 @@
       <c r="C32" s="103" t="n">
         <v>103187000</v>
       </c>
-    </row>
-    <row r="33" ht="20" customHeight="1">
-      <c r="H33" s="107" t="inlineStr">
+      <c r="H32" s="107" t="inlineStr">
         <is>
           <t>The Doubling Requirement</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="16" customHeight="1">
+      <c r="H33" s="85" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  FY27 $5M target − Q1 $713K actual = $4,287K remaining</t>
         </is>
       </c>
     </row>
     <row r="34" ht="16" customHeight="1">
       <c r="H34" s="85" t="inlineStr">
         <is>
-          <t xml:space="preserve">  FY27 $5M target − Q1 $713K actual = $4,287K remaining</t>
+          <t xml:space="preserve">  Over 3 quarters (Q2–Q4) = $1,429K/qtr required</t>
         </is>
       </c>
     </row>
     <row r="35" ht="16" customHeight="1">
       <c r="H35" s="85" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Over 3 quarters (Q2–Q4) = $1,429K/qtr required</t>
+          <t xml:space="preserve">  vs. Q1 $713K actual = 2.0× immediate ramp</t>
         </is>
       </c>
     </row>
     <row r="36" ht="16" customHeight="1">
       <c r="H36" s="85" t="inlineStr">
         <is>
-          <t xml:space="preserve">  vs. Q1 $713K actual = 2.0× immediate ramp</t>
+          <t xml:space="preserve">  Only funded if Exos capital bridges the working-capital gap</t>
         </is>
       </c>
     </row>
     <row r="37" ht="16" customHeight="1">
       <c r="H37" s="85" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Only funded if Exos capital bridges the working-capital gap</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="16" customHeight="1">
-      <c r="H38" s="85" t="inlineStr">
-        <is>
           <t xml:space="preserve">  Without capital → Q2–Q4 stays ≈ $713K/qtr = $2.85M FY27</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="28" customHeight="1">
-      <c r="A41" s="108" t="inlineStr">
+    <row r="40" ht="28" customHeight="1">
+      <c r="A40" s="108" t="inlineStr">
         <is>
           <t>Management Assumptions — all projections forward of FY27 Q1 actual ($713K) are management estimates, not independently audited. Without-Exos CAGR assumes no working-capital stall; stall scenarios produce lower figures. With-Exos CAGR uses v12 SSLC tank-unit/ASP/COGS drivers, not independently audited. DRAFT, 2026-10-07.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="39">
+  <mergeCells count="38">
     <mergeCell ref="H30:L30"/>
     <mergeCell ref="H26:L26"/>
     <mergeCell ref="H29:L29"/>
     <mergeCell ref="H35:L35"/>
-    <mergeCell ref="A41:L41"/>
-    <mergeCell ref="H38:L38"/>
+    <mergeCell ref="H20:L20"/>
     <mergeCell ref="H10:L10"/>
     <mergeCell ref="A18:F18"/>
-    <mergeCell ref="H31:L31"/>
     <mergeCell ref="H34:L34"/>
     <mergeCell ref="H9:L9"/>
     <mergeCell ref="A2:L2"/>
@@ -7600,10 +7474,11 @@
     <mergeCell ref="H11:L11"/>
     <mergeCell ref="H16:L16"/>
     <mergeCell ref="A9:F9"/>
+    <mergeCell ref="H32:L32"/>
     <mergeCell ref="H28:L28"/>
     <mergeCell ref="A4:L6"/>
+    <mergeCell ref="A40:L40"/>
     <mergeCell ref="H13:L13"/>
-    <mergeCell ref="H19:L19"/>
     <mergeCell ref="H37:L37"/>
     <mergeCell ref="H22:L22"/>
     <mergeCell ref="A15:F15"/>

</xml_diff>

<commit_message>
SSLC Option B: John 10/7 15:22-15:28 terms — table format, HIGH ~$10M, 5yr tank+milestones, principals' lockup, $5.1M trigger, name fix
</commit_message>
<xml_diff>
--- a/drafts/EXOS_SSLC_OptionB_Acquisition_Model_2026-10-07.xlsx
+++ b/drafts/EXOS_SSLC_OptionB_Acquisition_Model_2026-10-07.xlsx
@@ -23,14 +23,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="$#,##0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="$#,##0;($#,##0)"/>
     <numFmt numFmtId="167" formatCode="0.0x"/>
     <numFmt numFmtId="168" formatCode="0.00x"/>
+    <numFmt numFmtId="169" formatCode="&quot;$&quot;#,##0"/>
   </numFmts>
-  <fonts count="31">
+  <fonts count="35">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -172,8 +173,28 @@
     <font>
       <sz val="9.5"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="19">
+  <fills count="25">
     <fill>
       <patternFill/>
     </fill>
@@ -265,8 +286,38 @@
         <fgColor rgb="00BF8F00"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001E3A5F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DBEAFE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D1FAE5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F3F4F6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00BBF7D0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF3C7"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -302,11 +353,124 @@
         <color rgb="00CCCCCC"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="00BF8F00"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00BF8F00"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="00BF8F00"/>
+      </right>
+      <top style="medium">
+        <color rgb="00BF8F00"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="00BF8F00"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00BF8F00"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="00BF8F00"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="00BF8F00"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="00BF8F00"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="00BF8F00"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="109">
+  <cellXfs count="135">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -516,6 +680,36 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="31" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="32" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="32" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="32" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="33" fillId="20" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="32" fillId="20" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="32" fillId="20" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="32" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="33" fillId="21" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="33" fillId="21" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="33" fillId="22" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="33" fillId="22" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="33" fillId="23" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="33" fillId="23" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="34" fillId="24" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -940,7 +1134,7 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>Executed — Jon Quinn &amp; Jim Wertz</t>
+          <t>Executed — John Quinn &amp; Jim Wertz</t>
         </is>
       </c>
     </row>
@@ -1078,7 +1272,7 @@
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Jon decision 10/2; not re-proposed</t>
+          <t>John decision 10/2; not re-proposed</t>
         </is>
       </c>
     </row>
@@ -1231,11 +1425,11 @@
         </is>
       </c>
       <c r="B27" s="6" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C27" s="10" t="inlineStr">
         <is>
-          <t>Management assumption — unverified</t>
+          <t>Management assumption — unverified; FY27–FY31</t>
         </is>
       </c>
     </row>
@@ -1332,7 +1526,7 @@
     <row r="34" ht="22" customHeight="1">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>Earn-out ii — lockup period (months)</t>
+          <t>Earn-out ii — lockup (principals' terms)</t>
         </is>
       </c>
       <c r="B34" s="6" t="n">
@@ -1340,7 +1534,7 @@
       </c>
       <c r="C34" s="10" t="inlineStr">
         <is>
-          <t>Standard post-listing lockup</t>
+          <t>Same lockup terms as Exos principals (modeled ~12 months)</t>
         </is>
       </c>
     </row>
@@ -1362,7 +1556,7 @@
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>SSLC QB FY26 actuals (Jon 10/2 QB pull)</t>
+          <t>SSLC QB FY26 actuals (John 10/2 QB pull)</t>
         </is>
       </c>
     </row>
@@ -1407,7 +1601,7 @@
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>SSLC QB FY27 Q1 (Sep not yet closed, Jon 10/2)</t>
+          <t>SSLC QB FY27 Q1 (Sep not yet closed, John 10/2)</t>
         </is>
       </c>
     </row>
@@ -1452,7 +1646,7 @@
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>23.6% per Jon 10/2 board meeting</t>
+          <t>23.6% per John 10/2 board meeting</t>
         </is>
       </c>
     </row>
@@ -1467,7 +1661,7 @@
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>Markus Rufer confirmed ~$5M firm for 2027, 14–16 tanks (Jon 10/2)</t>
+          <t>Markus Rufer confirmed ~$5M firm for 2027, 14–16 tanks (John 10/2)</t>
         </is>
       </c>
     </row>
@@ -2197,7 +2391,7 @@
     <row r="105" ht="20" customHeight="1">
       <c r="A105" s="4" t="inlineStr">
         <is>
-          <t>BENEFITS TO SSLC INVESTORS (Jon 10/7)</t>
+          <t>BENEFITS TO SSLC INVESTORS (John 10/7)</t>
         </is>
       </c>
     </row>
@@ -2255,66 +2449,83 @@
     <row r="109" ht="20" customHeight="1">
       <c r="A109" s="5" t="inlineStr">
         <is>
-          <t>4. Earn-out upside — IM tank revenue (3 yrs)</t>
+          <t>4. Earn-out upside — IM tank revenue (5 yrs, FY27–FY31)</t>
         </is>
       </c>
       <c r="B109" s="5" t="inlineStr">
         <is>
-          <t>Up to $900K</t>
+          <t>Up to $1.5M</t>
         </is>
       </c>
       <c r="C109" s="7" t="inlineStr">
         <is>
-          <t>5%/yr x $5M IM firm; $300K cap</t>
+          <t>5%/yr x $5M IM firm; $300K cap; 5-year term</t>
         </is>
       </c>
     </row>
     <row r="110" ht="20" customHeight="1">
       <c r="A110" s="5" t="inlineStr">
         <is>
-          <t>5. Earn-out upside — Exos stock post-RTO</t>
+          <t>5. Milestone earn-outs (up to 5 goals)</t>
         </is>
       </c>
       <c r="B110" s="5" t="inlineStr">
         <is>
-          <t>$1.0M–$3.0M</t>
+          <t>Up to $1.1M</t>
         </is>
       </c>
       <c r="C110" s="7" t="inlineStr">
         <is>
-          <t>0.5%–1.0% FD at listing ($200M–$300M MEV)</t>
+          <t>Goal-based: $5.1M rev, OTV contract, $10M/$20M rev, BLK3 qual</t>
         </is>
       </c>
     </row>
     <row r="111" ht="20" customHeight="1">
       <c r="A111" s="5" t="inlineStr">
         <is>
-          <t>6. Liquidity via listed Exos stock</t>
+          <t>6. Earn-out upside — Exos stock post-RTO</t>
         </is>
       </c>
       <c r="B111" s="5" t="inlineStr">
         <is>
-          <t>Post-RTO ~FY28</t>
+          <t>$1.0M–$3.0M</t>
         </is>
       </c>
       <c r="C111" s="7" t="inlineStr">
         <is>
-          <t>12-mo lockup; publicly tradeable thereafter</t>
+          <t>0.5%–1.0% FD at listing ($200M–$300M MEV)</t>
         </is>
       </c>
     </row>
     <row r="112" ht="20" customHeight="1">
       <c r="A112" s="5" t="inlineStr">
         <is>
-          <t>7. IM program continuity</t>
+          <t>7. Liquidity via listed Exos stock</t>
         </is>
       </c>
       <c r="B112" s="5" t="inlineStr">
         <is>
+          <t>Post-RTO ~FY28</t>
+        </is>
+      </c>
+      <c r="C112" s="7" t="inlineStr">
+        <is>
+          <t>Principals' lockup terms; publicly tradeable thereafter</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="20" customHeight="1">
+      <c r="A113" s="5" t="inlineStr">
+        <is>
+          <t>8. IM program continuity</t>
+        </is>
+      </c>
+      <c r="B113" s="5" t="inlineStr">
+        <is>
           <t>Operational</t>
         </is>
       </c>
-      <c r="C112" s="7" t="inlineStr">
+      <c r="C113" s="7" t="inlineStr">
         <is>
           <t>No customer disruption; Exos-SSLC entity delivers</t>
         </is>
@@ -2323,7 +2534,7 @@
     <row r="115" ht="20" customHeight="1">
       <c r="A115" s="12" t="inlineStr">
         <is>
-          <t>HOLD TO YEAR 5 — ASSUMPTIONS (Jon 10/7)</t>
+          <t>HOLD TO YEAR 5 — ASSUMPTIONS (John 10/7)</t>
         </is>
       </c>
     </row>
@@ -2945,22 +3156,22 @@
       </c>
       <c r="B23" s="29" t="inlineStr">
         <is>
-          <t>% of SSLC IM tank revenue, annual cap, 3-year term</t>
+          <t>% of SSLC IM tank revenue, annual cap, 5-year term (FY27–FY31)</t>
         </is>
       </c>
       <c r="C23" s="29" t="inlineStr">
         <is>
-          <t>Exos common stock at listing (% of FD shares); 12-mo lockup</t>
+          <t>Exos common stock at listing (% of FD shares); principals' lockup</t>
         </is>
       </c>
       <c r="D23" s="29" t="inlineStr">
         <is>
-          <t>Both i + ii</t>
+          <t>Both i + ii + milestone earn-outs</t>
         </is>
       </c>
       <c r="E23" s="10" t="inlineStr">
         <is>
-          <t>Gives SSLC sellers upside from IM growth AND Exos growth</t>
+          <t>Gives SSLC sellers upside from IM growth AND Exos growth AND milestones</t>
         </is>
       </c>
     </row>
@@ -2984,7 +3195,7 @@
       </c>
       <c r="E24" s="10" t="inlineStr">
         <is>
-          <t>Low: 3% tank rev (cap $300K) × 3yr + 0.5% of $200M listing</t>
+          <t>Low: 3% tank rev (cap $300K) × 5yr + 0.5% of $200M listing + milestone 1 only</t>
         </is>
       </c>
     </row>
@@ -3008,7 +3219,7 @@
       </c>
       <c r="E25" s="10" t="inlineStr">
         <is>
-          <t>Base: 5% × $5M firm + 0.75% of $250M listing</t>
+          <t>Base: 5% × $5M firm × 5yr + 0.75% of $250M listing + milestones 1-3</t>
         </is>
       </c>
     </row>
@@ -3032,7 +3243,7 @@
       </c>
       <c r="E26" s="10" t="inlineStr">
         <is>
-          <t>High: 7% × $5M + 1.0% of $300M listing</t>
+          <t>High: 7% × $5M (cap $300K) × 5yr + 1.0% of $300M listing + all 5 milestones → ~$10M</t>
         </is>
       </c>
     </row>
@@ -3069,12 +3280,12 @@
       </c>
       <c r="B28" s="29" t="inlineStr">
         <is>
-          <t>Annual payments, 3 years</t>
+          <t>Annual payments, 5 years (FY27–FY31)</t>
         </is>
       </c>
       <c r="C28" s="29" t="inlineStr">
         <is>
-          <t>12-month lockup post-listing</t>
+          <t>Same lockup terms as Exos principals (modeled ~12 months)</t>
         </is>
       </c>
       <c r="D28" s="29" t="inlineStr">
@@ -3082,7 +3293,11 @@
           <t>Each tranche per its own schedule</t>
         </is>
       </c>
-      <c r="E28" s="10" t="inlineStr"/>
+      <c r="E28" s="10" t="inlineStr">
+        <is>
+          <t>Principals' lockup; realization timing modeled ~12 months post-listing</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="22" t="inlineStr">
@@ -5115,7 +5330,7 @@
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>SSLC stays OUT of RTO perimeter (Jon 10/2)</t>
+          <t>SSLC stays OUT of RTO perimeter (John 10/2)</t>
         </is>
       </c>
     </row>
@@ -5313,7 +5528,7 @@
     <row r="20" ht="28" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Jon sits on BOTH boards</t>
+          <t>John sits on BOTH boards</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -5323,7 +5538,7 @@
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>Jon must RECUSE from SSLC vote; send as Exos CEO only</t>
+          <t>John must RECUSE from SSLC vote; send as Exos CEO only</t>
         </is>
       </c>
     </row>
@@ -5357,7 +5572,7 @@
       </c>
       <c r="C22" s="7" t="inlineStr">
         <is>
-          <t>Markus Rufer and Bob; Jon abstains</t>
+          <t>Markus Rufer and Bob; John abstains</t>
         </is>
       </c>
     </row>
@@ -5369,12 +5584,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Deferred (Jon 10/7)</t>
+          <t>Deferred (John 10/7)</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>Negotiation stage; no legal review until Jon calls it</t>
+          <t>Negotiation stage; no legal review until John calls it</t>
         </is>
       </c>
     </row>
@@ -5554,7 +5769,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -5827,540 +6042,494 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="61" t="inlineStr">
-        <is>
-          <t>FORWARD POTENTIAL — EARN-OUTS (same in both cases; driven by IM firm revenue)</t>
+      <c r="A13" s="109" t="inlineStr">
+        <is>
+          <t>FORWARD POTENTIAL — EARN-OUTS (negotiating terms — management assumptions)</t>
         </is>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="58" t="inlineStr">
-        <is>
-          <t>Tank earn-out base (i): 5%/yr, $300K cap</t>
-        </is>
-      </c>
-      <c r="B14" s="31">
-        <f>MIN(Assumptions!B24*Assumptions!B44,Assumptions!B26)</f>
-        <v/>
-      </c>
-      <c r="C14" s="31">
-        <f>MIN(Assumptions!B24*Assumptions!B44,Assumptions!B26)</f>
-        <v/>
-      </c>
-      <c r="D14" s="31">
-        <f>MIN(Assumptions!B24*Assumptions!B44,Assumptions!B26)</f>
-        <v/>
-      </c>
-      <c r="E14" s="31" t="n">
+      <c r="A14" s="110" t="inlineStr">
+        <is>
+          <t>Tank earn-out BASE (5%/yr × avg $4M rev, cap $250K/yr)</t>
+        </is>
+      </c>
+      <c r="B14" s="111" t="n">
+        <v>200000</v>
+      </c>
+      <c r="C14" s="111" t="n">
+        <v>200000</v>
+      </c>
+      <c r="D14" s="111" t="n">
+        <v>200000</v>
+      </c>
+      <c r="E14" s="111" t="n">
+        <v>200000</v>
+      </c>
+      <c r="F14" s="111" t="n">
+        <v>200000</v>
+      </c>
+      <c r="G14" s="112">
+        <f>SUM(B14:F14)</f>
+        <v/>
+      </c>
+      <c r="H14" s="113" t="inlineStr">
+        <is>
+          <t>5%×~$4M SSLC/IM rev; cap $250K/yr; FY27-31; total $1,000K</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="110" t="inlineStr">
+        <is>
+          <t>Tank earn-out LOW (IM demand does not materialize)</t>
+        </is>
+      </c>
+      <c r="B15" s="111" t="n">
         <v>0</v>
       </c>
-      <c r="F14" s="31" t="n">
+      <c r="C15" s="111" t="n">
         <v>0</v>
       </c>
-      <c r="G14" s="31">
-        <f>SUM(B14:F14)</f>
-        <v/>
-      </c>
-      <c r="H14" s="10" t="inlineStr">
-        <is>
-          <t>5% × $5M firm IM ramp × 3 years; $300K/yr cap</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="58" t="inlineStr">
-        <is>
-          <t>Tank earn-out low (i): 3%/yr</t>
-        </is>
-      </c>
-      <c r="B15" s="31">
-        <f>MIN(Assumptions!B23*Assumptions!B44,Assumptions!B26)</f>
-        <v/>
-      </c>
-      <c r="C15" s="31">
-        <f>MIN(Assumptions!B23*Assumptions!B44,Assumptions!B26)</f>
-        <v/>
-      </c>
-      <c r="D15" s="31">
-        <f>MIN(Assumptions!B23*Assumptions!B44,Assumptions!B26)</f>
-        <v/>
-      </c>
-      <c r="E15" s="31" t="n">
+      <c r="D15" s="111" t="n">
         <v>0</v>
       </c>
-      <c r="F15" s="31" t="n">
+      <c r="E15" s="111" t="n">
         <v>0</v>
       </c>
-      <c r="G15" s="31">
+      <c r="F15" s="111" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="112">
         <f>SUM(B15:F15)</f>
         <v/>
       </c>
-      <c r="H15" s="10" t="inlineStr">
-        <is>
-          <t>Low scenario</t>
+      <c r="H15" s="113" t="inlineStr">
+        <is>
+          <t>Low scenario — $0</t>
         </is>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="58" t="inlineStr">
-        <is>
-          <t>Tank earn-out high (i): 7%/yr</t>
-        </is>
-      </c>
-      <c r="B16" s="31">
-        <f>MIN(Assumptions!B25*Assumptions!B44,Assumptions!B26)</f>
-        <v/>
-      </c>
-      <c r="C16" s="31">
-        <f>MIN(Assumptions!B25*Assumptions!B44,Assumptions!B26)</f>
-        <v/>
-      </c>
-      <c r="D16" s="31">
-        <f>MIN(Assumptions!B25*Assumptions!B44,Assumptions!B26)</f>
-        <v/>
-      </c>
-      <c r="E16" s="31" t="n">
+      <c r="A16" s="110" t="inlineStr">
+        <is>
+          <t>Tank earn-out HIGH (5%/yr × $5M rev, at $250K/yr cap)</t>
+        </is>
+      </c>
+      <c r="B16" s="111" t="n">
+        <v>250000</v>
+      </c>
+      <c r="C16" s="111" t="n">
+        <v>250000</v>
+      </c>
+      <c r="D16" s="111" t="n">
+        <v>250000</v>
+      </c>
+      <c r="E16" s="111" t="n">
+        <v>250000</v>
+      </c>
+      <c r="F16" s="111" t="n">
+        <v>250000</v>
+      </c>
+      <c r="G16" s="112">
+        <f>SUM(B16:F16)</f>
+        <v/>
+      </c>
+      <c r="H16" s="113" t="inlineStr">
+        <is>
+          <t>5%×$5M/yr; cap $250K; FY27-31; total $1,250K</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="114" t="inlineStr">
+        <is>
+          <t>MILESTONE EARN-OUTS — pays ONLY when trigger is verified (negotiating terms)</t>
+        </is>
+      </c>
+      <c r="B17" s="31" t="n"/>
+      <c r="C17" s="31" t="n"/>
+      <c r="D17" s="31" t="n"/>
+      <c r="E17" s="31" t="n"/>
+      <c r="F17" s="31" t="n"/>
+      <c r="G17" s="31" t="n"/>
+      <c r="H17" s="10" t="n"/>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  M1: SSLC FY27 $5M revenue on schedule</t>
+        </is>
+      </c>
+      <c r="B18" s="116" t="n"/>
+      <c r="C18" s="117" t="n">
+        <v>200000</v>
+      </c>
+      <c r="D18" s="116" t="n"/>
+      <c r="E18" s="116" t="n"/>
+      <c r="F18" s="116" t="n"/>
+      <c r="G18" s="116">
+        <f>SUM(B18:F18)</f>
+        <v/>
+      </c>
+      <c r="H18" s="115" t="inlineStr">
+        <is>
+          <t>BASE+HIGH; pays FY28 Q1; $200K</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  M2: Nebula/OTV production contract signed</t>
+        </is>
+      </c>
+      <c r="B19" s="116" t="n"/>
+      <c r="C19" s="116" t="n"/>
+      <c r="D19" s="117" t="n">
+        <v>300000</v>
+      </c>
+      <c r="E19" s="116" t="n"/>
+      <c r="F19" s="116" t="n"/>
+      <c r="G19" s="116">
+        <f>SUM(B19:F19)</f>
+        <v/>
+      </c>
+      <c r="H19" s="115" t="inlineStr">
+        <is>
+          <t>BASE+HIGH; pays at signing (est. FY29); $300K</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  M3: SSLC annual revenue ≥$10M</t>
+        </is>
+      </c>
+      <c r="B20" s="116" t="n"/>
+      <c r="C20" s="116" t="n"/>
+      <c r="D20" s="117" t="n">
+        <v>300000</v>
+      </c>
+      <c r="E20" s="116" t="n"/>
+      <c r="F20" s="116" t="n"/>
+      <c r="G20" s="116">
+        <f>SUM(B20:F20)</f>
+        <v/>
+      </c>
+      <c r="H20" s="115" t="inlineStr">
+        <is>
+          <t>HIGH only; est. FY29; $300K</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  M4: SSLC annual revenue ≥$20M</t>
+        </is>
+      </c>
+      <c r="B21" s="116" t="n"/>
+      <c r="C21" s="116" t="n"/>
+      <c r="D21" s="116" t="n"/>
+      <c r="E21" s="116" t="n"/>
+      <c r="F21" s="117" t="n">
+        <v>400000</v>
+      </c>
+      <c r="G21" s="116">
+        <f>SUM(B21:F21)</f>
+        <v/>
+      </c>
+      <c r="H21" s="115" t="inlineStr">
+        <is>
+          <t>HIGH only; est. FY31; $400K</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="115" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  M5: BLK3 tank qualification complete</t>
+        </is>
+      </c>
+      <c r="B22" s="116" t="n"/>
+      <c r="C22" s="117" t="n">
+        <v>150000</v>
+      </c>
+      <c r="D22" s="116" t="n"/>
+      <c r="E22" s="116" t="n"/>
+      <c r="F22" s="116" t="n"/>
+      <c r="G22" s="116">
+        <f>SUM(B22:F22)</f>
+        <v/>
+      </c>
+      <c r="H22" s="115" t="inlineStr">
+        <is>
+          <t>BASE+HIGH; est. FY28; $150K</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="113" t="inlineStr">
+        <is>
+          <t>Stock earn-out BASE (0.75% FD × $250M RTO)</t>
+        </is>
+      </c>
+      <c r="B23" s="111" t="n">
         <v>0</v>
       </c>
-      <c r="F16" s="31" t="n">
+      <c r="C23" s="111" t="n">
         <v>0</v>
       </c>
-      <c r="G16" s="31">
-        <f>SUM(B16:F16)</f>
-        <v/>
-      </c>
-      <c r="H16" s="10" t="inlineStr">
-        <is>
-          <t>High — capped at $300K</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="58" t="inlineStr">
-        <is>
-          <t>Stock earn-out base (ii): 0.75% FD @ listing</t>
-        </is>
-      </c>
-      <c r="B17" s="31" t="n">
+      <c r="D23" s="111" t="n">
+        <v>1875000</v>
+      </c>
+      <c r="E23" s="111" t="n">
         <v>0</v>
       </c>
-      <c r="C17" s="31" t="n">
+      <c r="F23" s="111" t="n">
         <v>0</v>
       </c>
-      <c r="D17" s="31">
-        <f>Assumptions!B29*Assumptions!B32</f>
-        <v/>
-      </c>
-      <c r="E17" s="31" t="n">
+      <c r="G23" s="113">
+        <f>SUM(B23:F23)</f>
+        <v/>
+      </c>
+      <c r="H23" s="113" t="inlineStr">
+        <is>
+          <t>12-mo lockup after ~FY28 listing; realized FY29</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="113" t="inlineStr">
+        <is>
+          <t>Stock earn-out LOW  (0.5% × $200M)</t>
+        </is>
+      </c>
+      <c r="B24" s="111" t="n">
         <v>0</v>
       </c>
-      <c r="F17" s="31" t="n">
+      <c r="C24" s="111" t="n">
         <v>0</v>
       </c>
-      <c r="G17" s="31">
-        <f>SUM(B17:F17)</f>
-        <v/>
-      </c>
-      <c r="H17" s="10" t="inlineStr">
-        <is>
-          <t>At $250M listing; realized FY29 post lockup</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="58" t="inlineStr">
-        <is>
-          <t>Stock earn-out low (ii): 0.5% @ $200M</t>
-        </is>
-      </c>
-      <c r="B18" s="31" t="n">
+      <c r="D24" s="111" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="E24" s="111" t="n">
         <v>0</v>
       </c>
-      <c r="C18" s="31" t="n">
+      <c r="F24" s="111" t="n">
         <v>0</v>
       </c>
-      <c r="D18" s="31">
-        <f>Assumptions!B28*Assumptions!B31</f>
-        <v/>
-      </c>
-      <c r="E18" s="31" t="n">
+      <c r="G24" s="113">
+        <f>SUM(B24:F24)</f>
+        <v/>
+      </c>
+      <c r="H24" s="113" t="inlineStr">
+        <is>
+          <t>Low RTO</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="118" t="inlineStr">
+        <is>
+          <t>Stock earn-out HIGH (1.0% × $300M)</t>
+        </is>
+      </c>
+      <c r="B25" s="111" t="n">
         <v>0</v>
       </c>
-      <c r="F18" s="31" t="n">
+      <c r="C25" s="111" t="n">
         <v>0</v>
       </c>
-      <c r="G18" s="31">
-        <f>SUM(B18:F18)</f>
-        <v/>
-      </c>
-      <c r="H18" s="10" t="inlineStr">
-        <is>
-          <t>Low RTO</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="58" t="inlineStr">
-        <is>
-          <t>Stock earn-out high (ii): 1.0% @ $300M</t>
-        </is>
-      </c>
-      <c r="B19" s="31" t="n">
+      <c r="D25" s="111" t="n">
+        <v>3000000</v>
+      </c>
+      <c r="E25" s="111" t="n">
         <v>0</v>
       </c>
-      <c r="C19" s="31" t="n">
+      <c r="F25" s="111" t="n">
         <v>0</v>
       </c>
-      <c r="D19" s="31">
-        <f>Assumptions!B30*Assumptions!B33</f>
-        <v/>
-      </c>
-      <c r="E19" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="F19" s="31" t="n">
-        <v>0</v>
-      </c>
-      <c r="G19" s="31">
-        <f>SUM(B19:F19)</f>
-        <v/>
-      </c>
-      <c r="H19" s="10" t="inlineStr">
+      <c r="G25" s="113">
+        <f>SUM(B25:F25)</f>
+        <v/>
+      </c>
+      <c r="H25" s="113" t="inlineStr">
         <is>
           <t>High RTO</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="12" t="inlineStr">
-        <is>
-          <t>TOTAL CONSIDERATION — OLD-MODEL CASE (v12) BASE | Actuals-Anchored as Sensitivity</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="26" t="inlineStr">
-        <is>
-          <t>OLD-MODEL BASE: funding + tank base + stock base</t>
-        </is>
-      </c>
-      <c r="B22" s="62">
-        <f>B12+B14+B17</f>
-        <v/>
-      </c>
-      <c r="C22" s="62">
-        <f>C12+C14+C17</f>
-        <v/>
-      </c>
-      <c r="D22" s="62">
-        <f>D12+D14+D17</f>
-        <v/>
-      </c>
-      <c r="E22" s="62">
-        <f>E12+E14+E17</f>
-        <v/>
-      </c>
-      <c r="F22" s="62">
-        <f>F12+F14+F17</f>
-        <v/>
-      </c>
-      <c r="G22" s="62">
-        <f>SUM(B22:F22)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="63" t="inlineStr">
-        <is>
-          <t>OLD-MODEL LOW:  funding + tank low + stock low</t>
-        </is>
-      </c>
-      <c r="B23" s="64">
-        <f>B12+B15+B18</f>
-        <v/>
-      </c>
-      <c r="C23" s="64">
-        <f>C12+C15+C18</f>
-        <v/>
-      </c>
-      <c r="D23" s="64">
-        <f>D12+D15+D18</f>
-        <v/>
-      </c>
-      <c r="E23" s="64">
-        <f>E12+E15+E18</f>
-        <v/>
-      </c>
-      <c r="F23" s="64">
-        <f>F12+F15+F18</f>
-        <v/>
-      </c>
-      <c r="G23" s="64">
-        <f>SUM(B23:F23)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24" ht="20" customHeight="1">
-      <c r="A24" s="65" t="inlineStr">
-        <is>
-          <t>OLD-MODEL HIGH: funding + tank high + stock high</t>
-        </is>
-      </c>
-      <c r="B24" s="66">
-        <f>B12+B16+B19</f>
-        <v/>
-      </c>
-      <c r="C24" s="66">
-        <f>C12+C16+C19</f>
-        <v/>
-      </c>
-      <c r="D24" s="66">
-        <f>D12+D16+D19</f>
-        <v/>
-      </c>
-      <c r="E24" s="66">
-        <f>E12+E16+E19</f>
-        <v/>
-      </c>
-      <c r="F24" s="66">
-        <f>F12+F16+F19</f>
-        <v/>
-      </c>
-      <c r="G24" s="66">
-        <f>SUM(B24:F24)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="24" t="inlineStr">
-        <is>
-          <t>AA SENSITIVITY BASE: funding + tank base + stock base</t>
-        </is>
-      </c>
-      <c r="B25" s="67">
-        <f>B12+B14+B17</f>
-        <v/>
-      </c>
-      <c r="C25" s="67">
-        <f>C12+C14+C17</f>
-        <v/>
-      </c>
-      <c r="D25" s="67">
-        <f>D12+D14+D17</f>
-        <v/>
-      </c>
-      <c r="E25" s="67">
-        <f>E12+E14+E17</f>
-        <v/>
-      </c>
-      <c r="F25" s="67">
-        <f>F12+F14+F17</f>
-        <v/>
-      </c>
-      <c r="G25" s="67">
-        <f>SUM(B25:F25)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="10" t="inlineStr">
-        <is>
-          <t>Chart: see drafts/SSLC_OptionB_Total_Compensation_5yr_2026-10-07.png (incl Y5 hold annotation)</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="12" t="inlineStr">
-        <is>
-          <t>HOLD TO YEAR 5 — Forward Potential if SSLC Investors Hold Exos Shares to FY31 (Jon 10/7)</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="32" customHeight="1">
-      <c r="A30" s="68" t="inlineStr">
-        <is>
-          <t>Base = Old-Model (v12). Dilution: Series A $25M staged (D1-D4, ~13%) + RTO (~12%) + option pool (~5%) = ~30% flat (MANAGEMENT ASSUMPTION). 0.75% stake at listing → 0.525% post-dilution. AA case EV ~$176M = BELOW $250M listing — stock worth less in AA case by FY31.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="22" customHeight="1">
-      <c r="A31" s="69" t="inlineStr">
-        <is>
-          <t>Scenario</t>
-        </is>
-      </c>
-      <c r="B31" s="69" t="inlineStr">
-        <is>
-          <t>FY31 EV</t>
-        </is>
-      </c>
-      <c r="C31" s="69" t="inlineStr">
-        <is>
-          <t>Post-dil stake</t>
-        </is>
-      </c>
-      <c r="D31" s="69" t="inlineStr">
-        <is>
-          <t>FY31 share value</t>
-        </is>
-      </c>
-      <c r="E31" s="69" t="inlineStr">
-        <is>
-          <t>At-listing value</t>
-        </is>
-      </c>
-      <c r="F31" s="69" t="inlineStr">
-        <is>
-          <t>Multiple vs listing</t>
-        </is>
-      </c>
-      <c r="G31" s="69" t="inlineStr"/>
-      <c r="H31" s="69" t="inlineStr">
-        <is>
-          <t>Notes</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="29" t="inlineStr">
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="26" t="n"/>
+      <c r="B26" s="62" t="n"/>
+      <c r="C26" s="62" t="n"/>
+      <c r="D26" s="62" t="n"/>
+      <c r="E26" s="62" t="n"/>
+      <c r="F26" s="62" t="n"/>
+      <c r="G26" s="62" t="n"/>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="119" t="inlineStr">
+        <is>
+          <t>TOTAL OFFER VALUE — BASE</t>
+        </is>
+      </c>
+      <c r="B27" s="120">
+        <f>B12+B14+B18+B19+B22+B23</f>
+        <v/>
+      </c>
+      <c r="C27" s="120">
+        <f>C12+C14+C18+C19+C22+C23</f>
+        <v/>
+      </c>
+      <c r="D27" s="120">
+        <f>D12+D14+D18+D19+D22+D23</f>
+        <v/>
+      </c>
+      <c r="E27" s="120">
+        <f>E12+E14+E18+E19+E22+E23</f>
+        <v/>
+      </c>
+      <c r="F27" s="120">
+        <f>F12+F14+F18+F19+F22+F23</f>
+        <v/>
+      </c>
+      <c r="G27" s="120">
+        <f>SUM(B27:F27)</f>
+        <v/>
+      </c>
+      <c r="H27" s="119" t="inlineStr">
+        <is>
+          <t>~$7.9M target</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="121" t="inlineStr">
+        <is>
+          <t>TOTAL OFFER VALUE — LOW  (no WC, no earn-outs, min stock)</t>
+        </is>
+      </c>
+      <c r="B28" s="122">
+        <f>B6+B7+B8+B9+B24</f>
+        <v/>
+      </c>
+      <c r="C28" s="122">
+        <f>C6+C7+C8+C9+C24</f>
+        <v/>
+      </c>
+      <c r="D28" s="122">
+        <f>D6+D7+D8+D9+D24</f>
+        <v/>
+      </c>
+      <c r="E28" s="122">
+        <f>E6+E7+E8+E9+E24</f>
+        <v/>
+      </c>
+      <c r="F28" s="122">
+        <f>F6+F7+F8+F9+F24</f>
+        <v/>
+      </c>
+      <c r="G28" s="122">
+        <f>SUM(B28:F28)</f>
+        <v/>
+      </c>
+      <c r="H28" s="121" t="inlineStr">
+        <is>
+          <t>~$4.9M target</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="123" t="inlineStr">
+        <is>
+          <t>TOTAL OFFER VALUE — HIGH (all milestones + tank high + stock high)</t>
+        </is>
+      </c>
+      <c r="B29" s="124">
+        <f>B12+B16+B18+B19+B20+B21+B22+B25</f>
+        <v/>
+      </c>
+      <c r="C29" s="124">
+        <f>C12+C16+C18+C19+C20+C21+C22+C25</f>
+        <v/>
+      </c>
+      <c r="D29" s="124">
+        <f>D12+D16+D18+D19+D20+D21+D22+D25</f>
+        <v/>
+      </c>
+      <c r="E29" s="124">
+        <f>E12+E16+E18+E19+E20+E21+E22+E25</f>
+        <v/>
+      </c>
+      <c r="F29" s="124">
+        <f>F12+F16+F18+F19+F20+F21+F22+F25</f>
+        <v/>
+      </c>
+      <c r="G29" s="124">
+        <f>SUM(B29:F29)</f>
+        <v/>
+      </c>
+      <c r="H29" s="123" t="inlineStr">
+        <is>
+          <t>~$10.0M target</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="125" t="inlineStr">
+        <is>
+          <t>Memo: Exos stock held to FY31 (NOT additive)</t>
+        </is>
+      </c>
+      <c r="B30" s="125" t="n"/>
+      <c r="C30" s="125" t="n"/>
+      <c r="D30" s="125" t="n"/>
+      <c r="E30" s="125" t="n"/>
+      <c r="F30" s="125" t="n"/>
+      <c r="G30" s="125" t="n"/>
+      <c r="H30" s="125" t="inlineStr">
+        <is>
+          <t>16×EV/EBITDA v12; ~30% dilution; L$5.7M/B$8.5M/H$11.4M — mgmt assumption</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="10" t="n"/>
+    </row>
+    <row r="32"/>
+    <row r="33">
+      <c r="A33" s="12" t="n"/>
+    </row>
+    <row r="34" ht="32" customHeight="1">
+      <c r="A34" s="68" t="n"/>
+    </row>
+    <row r="35" ht="22" customHeight="1">
+      <c r="A35" s="69" t="n"/>
+      <c r="B35" s="69" t="n"/>
+      <c r="C35" s="69" t="n"/>
+      <c r="D35" s="69" t="n"/>
+      <c r="E35" s="69" t="n"/>
+      <c r="F35" s="69" t="n"/>
+      <c r="G35" s="69" t="n"/>
+      <c r="H35" s="69" t="n"/>
+    </row>
+    <row r="36" ht="18" customHeight="1">
+      <c r="A36" s="29" t="inlineStr">
         <is>
           <t>Old-Model — Low</t>
         </is>
       </c>
-      <c r="B32" s="31">
+      <c r="B36" s="31">
         <f>Assumptions!B118</f>
         <v/>
       </c>
-      <c r="C32" s="54">
+      <c r="C36" s="54">
         <f>Assumptions!B125</f>
-        <v/>
-      </c>
-      <c r="D32" s="31">
-        <f>B32*C32</f>
-        <v/>
-      </c>
-      <c r="E32" s="31">
-        <f>Assumptions!B28*Assumptions!B31</f>
-        <v/>
-      </c>
-      <c r="F32" s="70">
-        <f>D32/E32</f>
-        <v/>
-      </c>
-      <c r="H32" s="71" t="inlineStr">
-        <is>
-          <t>0.5% grant x 0.70 = 0.35%; EV $1.626B</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="29" t="inlineStr">
-        <is>
-          <t>Old-Model — Base</t>
-        </is>
-      </c>
-      <c r="B33" s="31">
-        <f>Assumptions!B118</f>
-        <v/>
-      </c>
-      <c r="C33" s="54">
-        <f>Assumptions!B124</f>
-        <v/>
-      </c>
-      <c r="D33" s="31">
-        <f>B33*C33</f>
-        <v/>
-      </c>
-      <c r="E33" s="31">
-        <f>Assumptions!B29*Assumptions!B32</f>
-        <v/>
-      </c>
-      <c r="F33" s="70">
-        <f>D33/E33</f>
-        <v/>
-      </c>
-      <c r="H33" s="71" t="inlineStr">
-        <is>
-          <t>0.75% grant x 0.70 = 0.525%; EV $1.626B (~4.6x listing)</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="29" t="inlineStr">
-        <is>
-          <t>Old-Model — High</t>
-        </is>
-      </c>
-      <c r="B34" s="31">
-        <f>Assumptions!B118</f>
-        <v/>
-      </c>
-      <c r="C34" s="54">
-        <f>Assumptions!B126</f>
-        <v/>
-      </c>
-      <c r="D34" s="31">
-        <f>B34*C34</f>
-        <v/>
-      </c>
-      <c r="E34" s="31">
-        <f>Assumptions!B30*Assumptions!B33</f>
-        <v/>
-      </c>
-      <c r="F34" s="70">
-        <f>D34/E34</f>
-        <v/>
-      </c>
-      <c r="H34" s="71" t="inlineStr">
-        <is>
-          <t>1.0% grant x 0.70 = 0.70%; EV $1.626B</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="72" t="inlineStr">
-        <is>
-          <t>AA — Low</t>
-        </is>
-      </c>
-      <c r="B35" s="31">
-        <f>Assumptions!B120</f>
-        <v/>
-      </c>
-      <c r="C35" s="54">
-        <f>Assumptions!B125</f>
-        <v/>
-      </c>
-      <c r="D35" s="31">
-        <f>B35*C35</f>
-        <v/>
-      </c>
-      <c r="E35" s="31">
-        <f>Assumptions!B28*Assumptions!B31</f>
-        <v/>
-      </c>
-      <c r="F35" s="70">
-        <f>D35/E35</f>
-        <v/>
-      </c>
-      <c r="H35" s="71" t="inlineStr">
-        <is>
-          <t>BELOW listing value — AA FY31 EV ~$176M &lt; $250M MEV</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="72" t="inlineStr">
-        <is>
-          <t>AA — Base</t>
-        </is>
-      </c>
-      <c r="B36" s="31">
-        <f>Assumptions!B120</f>
-        <v/>
-      </c>
-      <c r="C36" s="54">
-        <f>Assumptions!B124</f>
         <v/>
       </c>
       <c r="D36" s="31">
@@ -6368,7 +6537,7 @@
         <v/>
       </c>
       <c r="E36" s="31">
-        <f>Assumptions!B29*Assumptions!B32</f>
+        <f>Assumptions!B28*Assumptions!B31</f>
         <v/>
       </c>
       <c r="F36" s="70">
@@ -6377,22 +6546,22 @@
       </c>
       <c r="H36" s="71" t="inlineStr">
         <is>
-          <t>BELOW listing — ~$924K vs $1.875M at listing (~0.49x)</t>
+          <t>0.5% grant x 0.70 = 0.35%; EV $1.626B</t>
         </is>
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="72" t="inlineStr">
-        <is>
-          <t>AA — High</t>
+      <c r="A37" s="29" t="inlineStr">
+        <is>
+          <t>Old-Model — Base</t>
         </is>
       </c>
       <c r="B37" s="31">
-        <f>Assumptions!B120</f>
+        <f>Assumptions!B118</f>
         <v/>
       </c>
       <c r="C37" s="54">
-        <f>Assumptions!B126</f>
+        <f>Assumptions!B124</f>
         <v/>
       </c>
       <c r="D37" s="31">
@@ -6400,7 +6569,7 @@
         <v/>
       </c>
       <c r="E37" s="31">
-        <f>Assumptions!B30*Assumptions!B33</f>
+        <f>Assumptions!B29*Assumptions!B32</f>
         <v/>
       </c>
       <c r="F37" s="70">
@@ -6409,28 +6578,151 @@
       </c>
       <c r="H37" s="71" t="inlineStr">
         <is>
+          <t>0.75% grant x 0.70 = 0.525%; EV $1.626B (~4.6x listing)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="18" customHeight="1">
+      <c r="A38" s="29" t="inlineStr">
+        <is>
+          <t>Old-Model — High</t>
+        </is>
+      </c>
+      <c r="B38" s="31">
+        <f>Assumptions!B118</f>
+        <v/>
+      </c>
+      <c r="C38" s="54">
+        <f>Assumptions!B126</f>
+        <v/>
+      </c>
+      <c r="D38" s="31">
+        <f>B38*C38</f>
+        <v/>
+      </c>
+      <c r="E38" s="31">
+        <f>Assumptions!B30*Assumptions!B33</f>
+        <v/>
+      </c>
+      <c r="F38" s="70">
+        <f>D38/E38</f>
+        <v/>
+      </c>
+      <c r="H38" s="71" t="inlineStr">
+        <is>
+          <t>1.0% grant x 0.70 = 0.70%; EV $1.626B</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="72" t="inlineStr">
+        <is>
+          <t>AA — Low</t>
+        </is>
+      </c>
+      <c r="B39" s="31">
+        <f>Assumptions!B120</f>
+        <v/>
+      </c>
+      <c r="C39" s="54">
+        <f>Assumptions!B125</f>
+        <v/>
+      </c>
+      <c r="D39" s="31">
+        <f>B39*C39</f>
+        <v/>
+      </c>
+      <c r="E39" s="31">
+        <f>Assumptions!B28*Assumptions!B31</f>
+        <v/>
+      </c>
+      <c r="F39" s="70">
+        <f>D39/E39</f>
+        <v/>
+      </c>
+      <c r="H39" s="71" t="inlineStr">
+        <is>
+          <t>BELOW listing value — AA FY31 EV ~$176M &lt; $250M MEV</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="72" t="inlineStr">
+        <is>
+          <t>AA — Base</t>
+        </is>
+      </c>
+      <c r="B40" s="31">
+        <f>Assumptions!B120</f>
+        <v/>
+      </c>
+      <c r="C40" s="54">
+        <f>Assumptions!B124</f>
+        <v/>
+      </c>
+      <c r="D40" s="31">
+        <f>B40*C40</f>
+        <v/>
+      </c>
+      <c r="E40" s="31">
+        <f>Assumptions!B29*Assumptions!B32</f>
+        <v/>
+      </c>
+      <c r="F40" s="70">
+        <f>D40/E40</f>
+        <v/>
+      </c>
+      <c r="H40" s="71" t="inlineStr">
+        <is>
+          <t>BELOW listing — ~$924K vs $1.875M at listing (~0.49x)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="18" customHeight="1">
+      <c r="A41" s="72" t="inlineStr">
+        <is>
+          <t>AA — High</t>
+        </is>
+      </c>
+      <c r="B41" s="31">
+        <f>Assumptions!B120</f>
+        <v/>
+      </c>
+      <c r="C41" s="54">
+        <f>Assumptions!B126</f>
+        <v/>
+      </c>
+      <c r="D41" s="31">
+        <f>B41*C41</f>
+        <v/>
+      </c>
+      <c r="E41" s="31">
+        <f>Assumptions!B30*Assumptions!B33</f>
+        <v/>
+      </c>
+      <c r="F41" s="70">
+        <f>D41/E41</f>
+        <v/>
+      </c>
+      <c r="H41" s="71" t="inlineStr">
+        <is>
           <t>BELOW listing — ~$1.23M vs $3.0M at listing (~0.41x)</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="42" customHeight="1">
-      <c r="A39" s="73" t="inlineStr">
+    <row r="43" ht="42" customHeight="1">
+      <c r="A43" s="73" t="inlineStr">
         <is>
           <t>NOTE: Y5 hold values are NOT additive to at-listing earn-out. Investors choose to hold OR sell at listing. Old-Model base: hold to FY31 = ~$8.54M vs sell at listing = $1.875M (4.6x). AA base: hold to FY31 = ~$0.92M vs sell at listing = $1.875M (0.49x) — AA case penalizes holding.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="4">
     <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A21:H21"/>
-    <mergeCell ref="A30:H30"/>
-    <mergeCell ref="A39:H39"/>
-    <mergeCell ref="A29:H29"/>
+    <mergeCell ref="A43:H43"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A13:H13"/>
     <mergeCell ref="A5:H5"/>
-    <mergeCell ref="A27:H27"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6915,12 +7207,39 @@
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="79" t="inlineStr">
         <is>
-          <t>KEY FACT:  Reaching $5M in FY27 requires averaging $1.43M/quarter for Q2–Q4  ($5,000K − $713K Q1 actual ÷ 3 quarters = $1,429K/qtr)  —  exactly 2.0× the most recent quarter's $713K  —  starting immediately.  Without Exos capital to fund working capital and IM ramp, that doubling is not achievable on SSLC's $198K cash position.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="22" customHeight="1"/>
-    <row r="6" ht="22" customHeight="1"/>
+          <t>KEY FACT:  Reaching $5.1M in FY27 requires averaging $1.46M/quarter for Q2–Q4  ($5,100K − $713K Q1 actual ÷ 3 quarters = $1,462K/qtr)  —  approximately 2.05× the most recent quarter's $713K  —  starting immediately.  Without Exos capital to fund working capital and IM ramp, that doubling is not achievable on SSLC's $198K cash position.</t>
+        </is>
+      </c>
+      <c r="B4" s="126" t="n"/>
+      <c r="C4" s="126" t="n"/>
+      <c r="D4" s="126" t="n"/>
+      <c r="E4" s="126" t="n"/>
+      <c r="F4" s="126" t="n"/>
+      <c r="G4" s="126" t="n"/>
+      <c r="H4" s="126" t="n"/>
+      <c r="I4" s="126" t="n"/>
+      <c r="J4" s="126" t="n"/>
+      <c r="K4" s="126" t="n"/>
+      <c r="L4" s="127" t="n"/>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="128" t="n"/>
+      <c r="L5" s="129" t="n"/>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="130" t="n"/>
+      <c r="B6" s="131" t="n"/>
+      <c r="C6" s="131" t="n"/>
+      <c r="D6" s="131" t="n"/>
+      <c r="E6" s="131" t="n"/>
+      <c r="F6" s="131" t="n"/>
+      <c r="G6" s="131" t="n"/>
+      <c r="H6" s="131" t="n"/>
+      <c r="I6" s="131" t="n"/>
+      <c r="J6" s="131" t="n"/>
+      <c r="K6" s="131" t="n"/>
+      <c r="L6" s="132" t="n"/>
+    </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="80" t="inlineStr">
         <is>
@@ -6977,6 +7296,10 @@
           <t xml:space="preserve">  Cash on hand (10/2/26):  $198K</t>
         </is>
       </c>
+      <c r="I10" s="133" t="n"/>
+      <c r="J10" s="133" t="n"/>
+      <c r="K10" s="133" t="n"/>
+      <c r="L10" s="134" t="n"/>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="86" t="inlineStr">
@@ -7004,6 +7327,10 @@
           <t xml:space="preserve">  Working capital needed to maintain deliveries:  $300K–$700K</t>
         </is>
       </c>
+      <c r="I11" s="133" t="n"/>
+      <c r="J11" s="133" t="n"/>
+      <c r="K11" s="133" t="n"/>
+      <c r="L11" s="134" t="n"/>
     </row>
     <row r="12" ht="16" customHeight="1">
       <c r="A12" s="86" t="inlineStr">
@@ -7029,6 +7356,10 @@
           <t xml:space="preserve">  FY26 operating loss:  −$416K</t>
         </is>
       </c>
+      <c r="I12" s="133" t="n"/>
+      <c r="J12" s="133" t="n"/>
+      <c r="K12" s="133" t="n"/>
+      <c r="L12" s="134" t="n"/>
     </row>
     <row r="13" ht="16" customHeight="1">
       <c r="A13" s="86" t="inlineStr">
@@ -7056,6 +7387,10 @@
           <t xml:space="preserve">  He-tank rework unresolved — no resolution path without new owner</t>
         </is>
       </c>
+      <c r="I13" s="133" t="n"/>
+      <c r="J13" s="133" t="n"/>
+      <c r="K13" s="133" t="n"/>
+      <c r="L13" s="134" t="n"/>
     </row>
     <row r="14" ht="16" customHeight="1">
       <c r="A14" s="86" t="inlineStr">
@@ -7083,6 +7418,10 @@
           <t xml:space="preserve">  No capex capacity → headcount/equipment frozen</t>
         </is>
       </c>
+      <c r="I14" s="133" t="n"/>
+      <c r="J14" s="133" t="n"/>
+      <c r="K14" s="133" t="n"/>
+      <c r="L14" s="134" t="n"/>
     </row>
     <row r="15" ht="16" customHeight="1">
       <c r="A15" s="94" t="inlineStr">
@@ -7095,6 +7434,10 @@
           <t xml:space="preserve">  Growth capped by self-funded working capital</t>
         </is>
       </c>
+      <c r="I15" s="133" t="n"/>
+      <c r="J15" s="133" t="n"/>
+      <c r="K15" s="133" t="n"/>
+      <c r="L15" s="134" t="n"/>
     </row>
     <row r="16" ht="16" customHeight="1">
       <c r="H16" s="85" t="inlineStr">
@@ -7102,6 +7445,10 @@
           <t xml:space="preserve">  FY27 achievable at run-rate:  ~$2.85M</t>
         </is>
       </c>
+      <c r="I16" s="133" t="n"/>
+      <c r="J16" s="133" t="n"/>
+      <c r="K16" s="133" t="n"/>
+      <c r="L16" s="134" t="n"/>
     </row>
     <row r="17" ht="16" customHeight="1">
       <c r="A17" s="95" t="inlineStr">
@@ -7114,6 +7461,10 @@
           <t xml:space="preserve">  FY31 best-case (10% CAGR, no stall):  ~$4.2M</t>
         </is>
       </c>
+      <c r="I17" s="133" t="n"/>
+      <c r="J17" s="133" t="n"/>
+      <c r="K17" s="133" t="n"/>
+      <c r="L17" s="134" t="n"/>
     </row>
     <row r="18" ht="16" customHeight="1">
       <c r="A18" s="96" t="inlineStr">
@@ -7126,6 +7477,10 @@
           <t xml:space="preserve">  5-yr CAGR (status quo):  ~10.0%</t>
         </is>
       </c>
+      <c r="I18" s="133" t="n"/>
+      <c r="J18" s="133" t="n"/>
+      <c r="K18" s="133" t="n"/>
+      <c r="L18" s="134" t="n"/>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="84" t="inlineStr"/>
@@ -7206,6 +7561,10 @@
           <t xml:space="preserve">  Cash at close:  $2.51M</t>
         </is>
       </c>
+      <c r="I21" s="133" t="n"/>
+      <c r="J21" s="133" t="n"/>
+      <c r="K21" s="133" t="n"/>
+      <c r="L21" s="134" t="n"/>
     </row>
     <row r="22" ht="16" customHeight="1">
       <c r="A22" s="86" t="inlineStr">
@@ -7233,6 +7592,10 @@
           <t xml:space="preserve">  SSLC debts paid at face (est. ~$500K TBV)</t>
         </is>
       </c>
+      <c r="I22" s="133" t="n"/>
+      <c r="J22" s="133" t="n"/>
+      <c r="K22" s="133" t="n"/>
+      <c r="L22" s="134" t="n"/>
     </row>
     <row r="23" ht="16" customHeight="1">
       <c r="A23" s="86" t="inlineStr">
@@ -7260,6 +7623,10 @@
           <t xml:space="preserve">  Prepaid-work delivery funded (cost $500K)</t>
         </is>
       </c>
+      <c r="I23" s="133" t="n"/>
+      <c r="J23" s="133" t="n"/>
+      <c r="K23" s="133" t="n"/>
+      <c r="L23" s="134" t="n"/>
     </row>
     <row r="24" ht="16" customHeight="1">
       <c r="H24" s="85" t="inlineStr">
@@ -7267,6 +7634,10 @@
           <t xml:space="preserve">  WC bridge removes Q2–Q3 stall risk</t>
         </is>
       </c>
+      <c r="I24" s="133" t="n"/>
+      <c r="J24" s="133" t="n"/>
+      <c r="K24" s="133" t="n"/>
+      <c r="L24" s="134" t="n"/>
     </row>
     <row r="25" ht="16" customHeight="1">
       <c r="A25" s="81" t="inlineStr">
@@ -7279,6 +7650,10 @@
           <t xml:space="preserve">  Exos procurement channel:  immediate BLK3 tank POs</t>
         </is>
       </c>
+      <c r="I25" s="133" t="n"/>
+      <c r="J25" s="133" t="n"/>
+      <c r="K25" s="133" t="n"/>
+      <c r="L25" s="134" t="n"/>
     </row>
     <row r="26" ht="16" customHeight="1">
       <c r="A26" s="84" t="inlineStr">
@@ -7311,6 +7686,10 @@
           <t xml:space="preserve">  Intuitive Machines ramp:  14–16 tanks firm FY27</t>
         </is>
       </c>
+      <c r="I26" s="133" t="n"/>
+      <c r="J26" s="133" t="n"/>
+      <c r="K26" s="133" t="n"/>
+      <c r="L26" s="134" t="n"/>
     </row>
     <row r="27" ht="16" customHeight="1">
       <c r="A27" s="101" t="inlineStr">
@@ -7329,6 +7708,10 @@
           <t xml:space="preserve">  Capex for production scale-up enabled</t>
         </is>
       </c>
+      <c r="I27" s="133" t="n"/>
+      <c r="J27" s="133" t="n"/>
+      <c r="K27" s="133" t="n"/>
+      <c r="L27" s="134" t="n"/>
     </row>
     <row r="28" ht="16" customHeight="1">
       <c r="A28" s="101" t="inlineStr">
@@ -7347,6 +7730,10 @@
           <t xml:space="preserve">  FY27 target (IM firm + ramp):  $4.1M–$5.5M</t>
         </is>
       </c>
+      <c r="I28" s="133" t="n"/>
+      <c r="J28" s="133" t="n"/>
+      <c r="K28" s="133" t="n"/>
+      <c r="L28" s="134" t="n"/>
     </row>
     <row r="29" ht="16" customHeight="1">
       <c r="A29" s="101" t="inlineStr">
@@ -7365,6 +7752,10 @@
           <t xml:space="preserve">  FY31 (v12 trajectory):  $54.7M</t>
         </is>
       </c>
+      <c r="I29" s="133" t="n"/>
+      <c r="J29" s="133" t="n"/>
+      <c r="K29" s="133" t="n"/>
+      <c r="L29" s="134" t="n"/>
     </row>
     <row r="30" ht="16" customHeight="1">
       <c r="A30" s="101" t="inlineStr">
@@ -7383,6 +7774,10 @@
           <t xml:space="preserve">  5-yr CAGR (with Exos, v12):  ~90.9%</t>
         </is>
       </c>
+      <c r="I30" s="133" t="n"/>
+      <c r="J30" s="133" t="n"/>
+      <c r="K30" s="133" t="n"/>
+      <c r="L30" s="134" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="101" t="inlineStr">
@@ -7414,23 +7809,35 @@
     <row r="33" ht="16" customHeight="1">
       <c r="H33" s="85" t="inlineStr">
         <is>
-          <t xml:space="preserve">  FY27 $5M target − Q1 $713K actual = $4,287K remaining</t>
-        </is>
-      </c>
+          <t xml:space="preserve">  FY27 $5.1M target − Q1 $713K actual = $4,387K remaining</t>
+        </is>
+      </c>
+      <c r="I33" s="133" t="n"/>
+      <c r="J33" s="133" t="n"/>
+      <c r="K33" s="133" t="n"/>
+      <c r="L33" s="134" t="n"/>
     </row>
     <row r="34" ht="16" customHeight="1">
       <c r="H34" s="85" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Over 3 quarters (Q2–Q4) = $1,429K/qtr required</t>
-        </is>
-      </c>
+          <t xml:space="preserve">  Over 3 quarters (Q2–Q4) = $1,462K/qtr required</t>
+        </is>
+      </c>
+      <c r="I34" s="133" t="n"/>
+      <c r="J34" s="133" t="n"/>
+      <c r="K34" s="133" t="n"/>
+      <c r="L34" s="134" t="n"/>
     </row>
     <row r="35" ht="16" customHeight="1">
       <c r="H35" s="85" t="inlineStr">
         <is>
-          <t xml:space="preserve">  vs. Q1 $713K actual = 2.0× immediate ramp</t>
-        </is>
-      </c>
+          <t xml:space="preserve">  vs. Q1 $713K actual = 2.05× immediate ramp</t>
+        </is>
+      </c>
+      <c r="I35" s="133" t="n"/>
+      <c r="J35" s="133" t="n"/>
+      <c r="K35" s="133" t="n"/>
+      <c r="L35" s="134" t="n"/>
     </row>
     <row r="36" ht="16" customHeight="1">
       <c r="H36" s="85" t="inlineStr">
@@ -7438,6 +7845,10 @@
           <t xml:space="preserve">  Only funded if Exos capital bridges the working-capital gap</t>
         </is>
       </c>
+      <c r="I36" s="133" t="n"/>
+      <c r="J36" s="133" t="n"/>
+      <c r="K36" s="133" t="n"/>
+      <c r="L36" s="134" t="n"/>
     </row>
     <row r="37" ht="16" customHeight="1">
       <c r="H37" s="85" t="inlineStr">
@@ -7445,6 +7856,10 @@
           <t xml:space="preserve">  Without capital → Q2–Q4 stays ≈ $713K/qtr = $2.85M FY27</t>
         </is>
       </c>
+      <c r="I37" s="133" t="n"/>
+      <c r="J37" s="133" t="n"/>
+      <c r="K37" s="133" t="n"/>
+      <c r="L37" s="134" t="n"/>
     </row>
     <row r="40" ht="28" customHeight="1">
       <c r="A40" s="108" t="inlineStr">

</xml_diff>

<commit_message>
SSLC Option B: reconcile summary/chart/model/draft to one structure (6.3/8.1/10.0M)
</commit_message>
<xml_diff>
--- a/drafts/EXOS_SSLC_OptionB_Acquisition_Model_2026-10-07.xlsx
+++ b/drafts/EXOS_SSLC_OptionB_Acquisition_Model_2026-10-07.xlsx
@@ -23,15 +23,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="$#,##0"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="$#,##0;($#,##0)"/>
     <numFmt numFmtId="167" formatCode="0.0x"/>
     <numFmt numFmtId="168" formatCode="0.00x"/>
-    <numFmt numFmtId="169" formatCode="&quot;$&quot;#,##0"/>
   </numFmts>
-  <fonts count="35">
+  <fonts count="31">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -173,28 +172,8 @@
     <font>
       <sz val="9.5"/>
     </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <i val="1"/>
-      <sz val="9"/>
-    </font>
   </fonts>
-  <fills count="25">
+  <fills count="19">
     <fill>
       <patternFill/>
     </fill>
@@ -286,38 +265,8 @@
         <fgColor rgb="00BF8F00"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001E3A5F"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00DBEAFE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00D1FAE5"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F3F4F6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00BBF7D0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FEF3C7"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="14">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -353,124 +302,11 @@
         <color rgb="00CCCCCC"/>
       </bottom>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00CCCCCC"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00CCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="00CCCCCC"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00CCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00CCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00CCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="00CCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00CCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color rgb="00BF8F00"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="00BF8F00"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color rgb="00BF8F00"/>
-      </right>
-      <top style="medium">
-        <color rgb="00BF8F00"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color rgb="00BF8F00"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="00BF8F00"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color rgb="00BF8F00"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color rgb="00BF8F00"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color rgb="00BF8F00"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color rgb="00BF8F00"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="135">
+  <cellXfs count="109">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -680,36 +516,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="31" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="32" fillId="12" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="169" fontId="32" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="32" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="33" fillId="20" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="32" fillId="20" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="32" fillId="20" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="169" fontId="32" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="33" fillId="21" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="33" fillId="21" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="33" fillId="22" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="33" fillId="22" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="33" fillId="23" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="33" fillId="23" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="34" fillId="24" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -6042,481 +5848,498 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="109" t="inlineStr">
-        <is>
-          <t>FORWARD POTENTIAL — EARN-OUTS (negotiating terms — management assumptions)</t>
+      <c r="A13" s="61" t="inlineStr">
+        <is>
+          <t>FORWARD POTENTIAL — EARN-OUTS (same in both cases; driven by IM firm revenue)</t>
         </is>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="110" t="inlineStr">
-        <is>
-          <t>Tank earn-out BASE (5%/yr × avg $4M rev, cap $250K/yr)</t>
-        </is>
-      </c>
-      <c r="B14" s="111" t="n">
+      <c r="A14" s="58" t="inlineStr">
+        <is>
+          <t>Tank earn-out base (i): 5%/yr, $300K cap, 5yr FY27–FY31</t>
+        </is>
+      </c>
+      <c r="B14" s="31">
+        <f>MIN(Assumptions!B24*Assumptions!B44,Assumptions!B26)</f>
+        <v/>
+      </c>
+      <c r="C14" s="31">
+        <f>MIN(Assumptions!B24*Assumptions!B44,Assumptions!B26)</f>
+        <v/>
+      </c>
+      <c r="D14" s="31">
+        <f>MIN(Assumptions!B24*Assumptions!B44,Assumptions!B26)</f>
+        <v/>
+      </c>
+      <c r="E14" s="31">
+        <f>MIN(Assumptions!B24*Assumptions!B44,Assumptions!B26)</f>
+        <v/>
+      </c>
+      <c r="F14" s="31">
+        <f>MIN(Assumptions!B24*Assumptions!B44,Assumptions!B26)</f>
+        <v/>
+      </c>
+      <c r="G14" s="31">
+        <f>SUM(B14:F14)</f>
+        <v/>
+      </c>
+      <c r="H14" s="10" t="inlineStr">
+        <is>
+          <t>5% × $5M firm IM ramp × 5 years; $300K/yr cap</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="58" t="inlineStr">
+        <is>
+          <t>Tank earn-out low (i): 3%/yr × 5yr</t>
+        </is>
+      </c>
+      <c r="B15" s="31">
+        <f>MIN(Assumptions!B23*Assumptions!B44,Assumptions!B26)</f>
+        <v/>
+      </c>
+      <c r="C15" s="31">
+        <f>MIN(Assumptions!B23*Assumptions!B44,Assumptions!B26)</f>
+        <v/>
+      </c>
+      <c r="D15" s="31">
+        <f>MIN(Assumptions!B23*Assumptions!B44,Assumptions!B26)</f>
+        <v/>
+      </c>
+      <c r="E15" s="31">
+        <f>MIN(Assumptions!B23*Assumptions!B44,Assumptions!B26)</f>
+        <v/>
+      </c>
+      <c r="F15" s="31">
+        <f>MIN(Assumptions!B23*Assumptions!B44,Assumptions!B26)</f>
+        <v/>
+      </c>
+      <c r="G15" s="31">
+        <f>SUM(B15:F15)</f>
+        <v/>
+      </c>
+      <c r="H15" s="10" t="inlineStr">
+        <is>
+          <t>Low scenario × 5yr</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="58" t="inlineStr">
+        <is>
+          <t>Tank earn-out high (i): 7%/yr × 5yr (cap $300K)</t>
+        </is>
+      </c>
+      <c r="B16" s="31">
+        <f>MIN(Assumptions!B25*Assumptions!B44,Assumptions!B26)</f>
+        <v/>
+      </c>
+      <c r="C16" s="31">
+        <f>MIN(Assumptions!B25*Assumptions!B44,Assumptions!B26)</f>
+        <v/>
+      </c>
+      <c r="D16" s="31">
+        <f>MIN(Assumptions!B25*Assumptions!B44,Assumptions!B26)</f>
+        <v/>
+      </c>
+      <c r="E16" s="31">
+        <f>MIN(Assumptions!B25*Assumptions!B44,Assumptions!B26)</f>
+        <v/>
+      </c>
+      <c r="F16" s="31">
+        <f>MIN(Assumptions!B25*Assumptions!B44,Assumptions!B26)</f>
+        <v/>
+      </c>
+      <c r="G16" s="31">
+        <f>SUM(B16:F16)</f>
+        <v/>
+      </c>
+      <c r="H16" s="10" t="inlineStr">
+        <is>
+          <t>High — capped at $300K/yr × 5yr = $1.5M</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="58" t="inlineStr">
+        <is>
+          <t>Milestone earn-outs base (3 of 5 triggered)</t>
+        </is>
+      </c>
+      <c r="B17" s="31" t="n">
         <v>200000</v>
       </c>
-      <c r="C14" s="111" t="n">
+      <c r="C17" s="31" t="n">
         <v>200000</v>
       </c>
-      <c r="D14" s="111" t="n">
+      <c r="D17" s="31" t="n">
+        <v>250000</v>
+      </c>
+      <c r="E17" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="31">
+        <f>SUM(B17:F17)</f>
+        <v/>
+      </c>
+      <c r="H17" s="10" t="inlineStr">
+        <is>
+          <t>Base: M1 $5.1M rev FY27 + M2 OTV contract + M3 $10M rev (mgmt assumption)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="58" t="inlineStr">
+        <is>
+          <t>Milestone earn-outs low (M1 only)</t>
+        </is>
+      </c>
+      <c r="B18" s="31" t="n">
         <v>200000</v>
       </c>
-      <c r="E14" s="111" t="n">
+      <c r="C18" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="31">
+        <f>SUM(B18:F18)</f>
+        <v/>
+      </c>
+      <c r="H18" s="10" t="inlineStr">
+        <is>
+          <t>Low: only M1 SSLC FY2026-27 revenue ≥$5.1M — $200K</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="58" t="inlineStr">
+        <is>
+          <t>Milestone earn-outs high (all 5 triggered)</t>
+        </is>
+      </c>
+      <c r="B19" s="31" t="n">
         <v>200000</v>
       </c>
-      <c r="F14" s="111" t="n">
+      <c r="C19" s="31" t="n">
         <v>200000</v>
       </c>
-      <c r="G14" s="112">
-        <f>SUM(B14:F14)</f>
-        <v/>
-      </c>
-      <c r="H14" s="113" t="inlineStr">
-        <is>
-          <t>5%×~$4M SSLC/IM rev; cap $250K/yr; FY27-31; total $1,000K</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="110" t="inlineStr">
-        <is>
-          <t>Tank earn-out LOW (IM demand does not materialize)</t>
-        </is>
-      </c>
-      <c r="B15" s="111" t="n">
+      <c r="D19" s="31" t="n">
+        <v>250000</v>
+      </c>
+      <c r="E19" s="31" t="n">
+        <v>250000</v>
+      </c>
+      <c r="F19" s="31" t="n">
+        <v>200000</v>
+      </c>
+      <c r="G19" s="31">
+        <f>SUM(B19:F19)</f>
+        <v/>
+      </c>
+      <c r="H19" s="10" t="inlineStr">
+        <is>
+          <t>High: M1 $200K + M2 $200K + M3 $250K + M4 $250K + M5 $200K = $1.1M</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="58" t="inlineStr">
+        <is>
+          <t>Stock earn-out base (ii): 0.75% FD @ listing</t>
+        </is>
+      </c>
+      <c r="B20" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="C15" s="111" t="n">
+      <c r="C20" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="D15" s="111" t="n">
+      <c r="D20" s="31">
+        <f>Assumptions!B29*Assumptions!B32</f>
+        <v/>
+      </c>
+      <c r="E20" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="E15" s="111" t="n">
+      <c r="F20" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="F15" s="111" t="n">
+      <c r="G20" s="31">
+        <f>SUM(B20:F20)</f>
+        <v/>
+      </c>
+      <c r="H20" s="10" t="inlineStr">
+        <is>
+          <t>At $250M listing; realized FY29 post principals' lockup (modeled ~12 months)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="58" t="inlineStr">
+        <is>
+          <t>Stock earn-out low (ii): 0.5% @ $200M</t>
+        </is>
+      </c>
+      <c r="B21" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="G15" s="112">
-        <f>SUM(B15:F15)</f>
-        <v/>
-      </c>
-      <c r="H15" s="113" t="inlineStr">
-        <is>
-          <t>Low scenario — $0</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="110" t="inlineStr">
-        <is>
-          <t>Tank earn-out HIGH (5%/yr × $5M rev, at $250K/yr cap)</t>
-        </is>
-      </c>
-      <c r="B16" s="111" t="n">
-        <v>250000</v>
-      </c>
-      <c r="C16" s="111" t="n">
-        <v>250000</v>
-      </c>
-      <c r="D16" s="111" t="n">
-        <v>250000</v>
-      </c>
-      <c r="E16" s="111" t="n">
-        <v>250000</v>
-      </c>
-      <c r="F16" s="111" t="n">
-        <v>250000</v>
-      </c>
-      <c r="G16" s="112">
-        <f>SUM(B16:F16)</f>
-        <v/>
-      </c>
-      <c r="H16" s="113" t="inlineStr">
-        <is>
-          <t>5%×$5M/yr; cap $250K; FY27-31; total $1,250K</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="114" t="inlineStr">
-        <is>
-          <t>MILESTONE EARN-OUTS — pays ONLY when trigger is verified (negotiating terms)</t>
-        </is>
-      </c>
-      <c r="B17" s="31" t="n"/>
-      <c r="C17" s="31" t="n"/>
-      <c r="D17" s="31" t="n"/>
-      <c r="E17" s="31" t="n"/>
-      <c r="F17" s="31" t="n"/>
-      <c r="G17" s="31" t="n"/>
-      <c r="H17" s="10" t="n"/>
-    </row>
-    <row r="18" ht="18" customHeight="1">
-      <c r="A18" s="115" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  M1: SSLC FY27 $5M revenue on schedule</t>
-        </is>
-      </c>
-      <c r="B18" s="116" t="n"/>
-      <c r="C18" s="117" t="n">
-        <v>200000</v>
-      </c>
-      <c r="D18" s="116" t="n"/>
-      <c r="E18" s="116" t="n"/>
-      <c r="F18" s="116" t="n"/>
-      <c r="G18" s="116">
-        <f>SUM(B18:F18)</f>
-        <v/>
-      </c>
-      <c r="H18" s="115" t="inlineStr">
-        <is>
-          <t>BASE+HIGH; pays FY28 Q1; $200K</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="115" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  M2: Nebula/OTV production contract signed</t>
-        </is>
-      </c>
-      <c r="B19" s="116" t="n"/>
-      <c r="C19" s="116" t="n"/>
-      <c r="D19" s="117" t="n">
-        <v>300000</v>
-      </c>
-      <c r="E19" s="116" t="n"/>
-      <c r="F19" s="116" t="n"/>
-      <c r="G19" s="116">
-        <f>SUM(B19:F19)</f>
-        <v/>
-      </c>
-      <c r="H19" s="115" t="inlineStr">
-        <is>
-          <t>BASE+HIGH; pays at signing (est. FY29); $300K</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="115" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  M3: SSLC annual revenue ≥$10M</t>
-        </is>
-      </c>
-      <c r="B20" s="116" t="n"/>
-      <c r="C20" s="116" t="n"/>
-      <c r="D20" s="117" t="n">
-        <v>300000</v>
-      </c>
-      <c r="E20" s="116" t="n"/>
-      <c r="F20" s="116" t="n"/>
-      <c r="G20" s="116">
-        <f>SUM(B20:F20)</f>
-        <v/>
-      </c>
-      <c r="H20" s="115" t="inlineStr">
-        <is>
-          <t>HIGH only; est. FY29; $300K</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="115" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  M4: SSLC annual revenue ≥$20M</t>
-        </is>
-      </c>
-      <c r="B21" s="116" t="n"/>
-      <c r="C21" s="116" t="n"/>
-      <c r="D21" s="116" t="n"/>
-      <c r="E21" s="116" t="n"/>
-      <c r="F21" s="117" t="n">
-        <v>400000</v>
-      </c>
-      <c r="G21" s="116">
+      <c r="C21" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="31">
+        <f>Assumptions!B28*Assumptions!B31</f>
+        <v/>
+      </c>
+      <c r="E21" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="31">
         <f>SUM(B21:F21)</f>
         <v/>
       </c>
-      <c r="H21" s="115" t="inlineStr">
-        <is>
-          <t>HIGH only; est. FY31; $400K</t>
+      <c r="H21" s="10" t="inlineStr">
+        <is>
+          <t>Low RTO</t>
         </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="115" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  M5: BLK3 tank qualification complete</t>
-        </is>
-      </c>
-      <c r="B22" s="116" t="n"/>
-      <c r="C22" s="117" t="n">
-        <v>150000</v>
-      </c>
-      <c r="D22" s="116" t="n"/>
-      <c r="E22" s="116" t="n"/>
-      <c r="F22" s="116" t="n"/>
-      <c r="G22" s="116">
+      <c r="A22" s="58" t="inlineStr">
+        <is>
+          <t>Stock earn-out high (ii): 1.0% @ $300M</t>
+        </is>
+      </c>
+      <c r="B22" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="31">
+        <f>Assumptions!B30*Assumptions!B33</f>
+        <v/>
+      </c>
+      <c r="E22" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F22" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="31">
         <f>SUM(B22:F22)</f>
         <v/>
       </c>
-      <c r="H22" s="115" t="inlineStr">
-        <is>
-          <t>BASE+HIGH; est. FY28; $150K</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="113" t="inlineStr">
-        <is>
-          <t>Stock earn-out BASE (0.75% FD × $250M RTO)</t>
-        </is>
-      </c>
-      <c r="B23" s="111" t="n">
-        <v>0</v>
-      </c>
-      <c r="C23" s="111" t="n">
-        <v>0</v>
-      </c>
-      <c r="D23" s="111" t="n">
-        <v>1875000</v>
-      </c>
-      <c r="E23" s="111" t="n">
-        <v>0</v>
-      </c>
-      <c r="F23" s="111" t="n">
-        <v>0</v>
-      </c>
-      <c r="G23" s="113">
-        <f>SUM(B23:F23)</f>
-        <v/>
-      </c>
-      <c r="H23" s="113" t="inlineStr">
-        <is>
-          <t>12-mo lockup after ~FY28 listing; realized FY29</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="113" t="inlineStr">
-        <is>
-          <t>Stock earn-out LOW  (0.5% × $200M)</t>
-        </is>
-      </c>
-      <c r="B24" s="111" t="n">
-        <v>0</v>
-      </c>
-      <c r="C24" s="111" t="n">
-        <v>0</v>
-      </c>
-      <c r="D24" s="111" t="n">
-        <v>1000000</v>
-      </c>
-      <c r="E24" s="111" t="n">
-        <v>0</v>
-      </c>
-      <c r="F24" s="111" t="n">
-        <v>0</v>
-      </c>
-      <c r="G24" s="113">
-        <f>SUM(B24:F24)</f>
-        <v/>
-      </c>
-      <c r="H24" s="113" t="inlineStr">
-        <is>
-          <t>Low RTO</t>
+      <c r="H22" s="10" t="inlineStr">
+        <is>
+          <t>High RTO</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="118" t="inlineStr">
-        <is>
-          <t>Stock earn-out HIGH (1.0% × $300M)</t>
-        </is>
-      </c>
-      <c r="B25" s="111" t="n">
-        <v>0</v>
-      </c>
-      <c r="C25" s="111" t="n">
-        <v>0</v>
-      </c>
-      <c r="D25" s="111" t="n">
-        <v>3000000</v>
-      </c>
-      <c r="E25" s="111" t="n">
-        <v>0</v>
-      </c>
-      <c r="F25" s="111" t="n">
-        <v>0</v>
-      </c>
-      <c r="G25" s="113">
-        <f>SUM(B25:F25)</f>
-        <v/>
-      </c>
-      <c r="H25" s="113" t="inlineStr">
-        <is>
-          <t>High RTO</t>
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>TOTAL CONSIDERATION — 5-yr (base price + earn-outs + milestones) | negotiating terms — management assumptions</t>
         </is>
       </c>
     </row>
     <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="26" t="n"/>
-      <c r="B26" s="62" t="n"/>
-      <c r="C26" s="62" t="n"/>
-      <c r="D26" s="62" t="n"/>
-      <c r="E26" s="62" t="n"/>
-      <c r="F26" s="62" t="n"/>
-      <c r="G26" s="62" t="n"/>
+      <c r="A26" s="26" t="inlineStr">
+        <is>
+          <t>BASE: funding + tank base (5yr) + milestones 1-3 + stock base</t>
+        </is>
+      </c>
+      <c r="B26" s="62">
+        <f>B12+B14+B17+B20</f>
+        <v/>
+      </c>
+      <c r="C26" s="62">
+        <f>C12+C14+C17+C20</f>
+        <v/>
+      </c>
+      <c r="D26" s="62">
+        <f>D12+D14+D17+D20</f>
+        <v/>
+      </c>
+      <c r="E26" s="62">
+        <f>E12+E14+E17+E20</f>
+        <v/>
+      </c>
+      <c r="F26" s="62">
+        <f>F12+F14+F17+F20</f>
+        <v/>
+      </c>
+      <c r="G26" s="62">
+        <f>SUM(B26:F26)</f>
+        <v/>
+      </c>
     </row>
     <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="119" t="inlineStr">
-        <is>
-          <t>TOTAL OFFER VALUE — BASE</t>
-        </is>
-      </c>
-      <c r="B27" s="120">
-        <f>B12+B14+B18+B19+B22+B23</f>
-        <v/>
-      </c>
-      <c r="C27" s="120">
-        <f>C12+C14+C18+C19+C22+C23</f>
-        <v/>
-      </c>
-      <c r="D27" s="120">
-        <f>D12+D14+D18+D19+D22+D23</f>
-        <v/>
-      </c>
-      <c r="E27" s="120">
-        <f>E12+E14+E18+E19+E22+E23</f>
-        <v/>
-      </c>
-      <c r="F27" s="120">
-        <f>F12+F14+F18+F19+F22+F23</f>
-        <v/>
-      </c>
-      <c r="G27" s="120">
+      <c r="A27" s="63" t="inlineStr">
+        <is>
+          <t>LOW:  funding + tank low (5yr) + milestone M1 only + stock low</t>
+        </is>
+      </c>
+      <c r="B27" s="64">
+        <f>B12+B15+B18+B21</f>
+        <v/>
+      </c>
+      <c r="C27" s="64">
+        <f>C12+C15+C18+C21</f>
+        <v/>
+      </c>
+      <c r="D27" s="64">
+        <f>D12+D15+D18+D21</f>
+        <v/>
+      </c>
+      <c r="E27" s="64">
+        <f>E12+E15+E18+E21</f>
+        <v/>
+      </c>
+      <c r="F27" s="64">
+        <f>F12+F15+F18+F21</f>
+        <v/>
+      </c>
+      <c r="G27" s="64">
         <f>SUM(B27:F27)</f>
         <v/>
       </c>
-      <c r="H27" s="119" t="inlineStr">
-        <is>
-          <t>~$7.9M target</t>
-        </is>
-      </c>
     </row>
     <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="121" t="inlineStr">
-        <is>
-          <t>TOTAL OFFER VALUE — LOW  (no WC, no earn-outs, min stock)</t>
-        </is>
-      </c>
-      <c r="B28" s="122">
-        <f>B6+B7+B8+B9+B24</f>
-        <v/>
-      </c>
-      <c r="C28" s="122">
-        <f>C6+C7+C8+C9+C24</f>
-        <v/>
-      </c>
-      <c r="D28" s="122">
-        <f>D6+D7+D8+D9+D24</f>
-        <v/>
-      </c>
-      <c r="E28" s="122">
-        <f>E6+E7+E8+E9+E24</f>
-        <v/>
-      </c>
-      <c r="F28" s="122">
-        <f>F6+F7+F8+F9+F24</f>
-        <v/>
-      </c>
-      <c r="G28" s="122">
+      <c r="A28" s="65" t="inlineStr">
+        <is>
+          <t>HIGH: funding + tank high (5yr) + all milestones + stock high  ≈ $10.0M</t>
+        </is>
+      </c>
+      <c r="B28" s="66">
+        <f>B12+B16+B19+B22</f>
+        <v/>
+      </c>
+      <c r="C28" s="66">
+        <f>C12+C16+C19+C22</f>
+        <v/>
+      </c>
+      <c r="D28" s="66">
+        <f>D12+D16+D19+D22</f>
+        <v/>
+      </c>
+      <c r="E28" s="66">
+        <f>E12+E16+E19+E22</f>
+        <v/>
+      </c>
+      <c r="F28" s="66">
+        <f>F12+F16+F19+F22</f>
+        <v/>
+      </c>
+      <c r="G28" s="66">
         <f>SUM(B28:F28)</f>
         <v/>
       </c>
-      <c r="H28" s="121" t="inlineStr">
-        <is>
-          <t>~$4.9M target</t>
-        </is>
-      </c>
     </row>
     <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="123" t="inlineStr">
-        <is>
-          <t>TOTAL OFFER VALUE — HIGH (all milestones + tank high + stock high)</t>
-        </is>
-      </c>
-      <c r="B29" s="124">
-        <f>B12+B16+B18+B19+B20+B21+B22+B25</f>
-        <v/>
-      </c>
-      <c r="C29" s="124">
-        <f>C12+C16+C18+C19+C20+C21+C22+C25</f>
-        <v/>
-      </c>
-      <c r="D29" s="124">
-        <f>D12+D16+D18+D19+D20+D21+D22+D25</f>
-        <v/>
-      </c>
-      <c r="E29" s="124">
-        <f>E12+E16+E18+E19+E20+E21+E22+E25</f>
-        <v/>
-      </c>
-      <c r="F29" s="124">
-        <f>F12+F16+F18+F19+F20+F21+F22+F25</f>
-        <v/>
-      </c>
-      <c r="G29" s="124">
+      <c r="A29" s="24" t="inlineStr">
+        <is>
+          <t>AA SENSITIVITY BASE (same earn-out structure)</t>
+        </is>
+      </c>
+      <c r="B29" s="67">
+        <f>B12+B14+B17+B20</f>
+        <v/>
+      </c>
+      <c r="C29" s="67">
+        <f>C12+C14+C17+C20</f>
+        <v/>
+      </c>
+      <c r="D29" s="67">
+        <f>D12+D14+D17+D20</f>
+        <v/>
+      </c>
+      <c r="E29" s="67">
+        <f>E12+E14+E17+E20</f>
+        <v/>
+      </c>
+      <c r="F29" s="67">
+        <f>F12+F14+F17+F20</f>
+        <v/>
+      </c>
+      <c r="G29" s="67">
         <f>SUM(B29:F29)</f>
         <v/>
       </c>
-      <c r="H29" s="123" t="inlineStr">
-        <is>
-          <t>~$10.0M target</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="125" t="inlineStr">
-        <is>
-          <t>Memo: Exos stock held to FY31 (NOT additive)</t>
-        </is>
-      </c>
-      <c r="B30" s="125" t="n"/>
-      <c r="C30" s="125" t="n"/>
-      <c r="D30" s="125" t="n"/>
-      <c r="E30" s="125" t="n"/>
-      <c r="F30" s="125" t="n"/>
-      <c r="G30" s="125" t="n"/>
-      <c r="H30" s="125" t="inlineStr">
-        <is>
-          <t>16×EV/EBITDA v12; ~30% dilution; L$5.7M/B$8.5M/H$11.4M — mgmt assumption</t>
-        </is>
-      </c>
     </row>
     <row r="31">
-      <c r="A31" s="10" t="n"/>
-    </row>
-    <row r="32"/>
+      <c r="A31" s="10" t="inlineStr">
+        <is>
+          <t>Chart: see drafts/SSLC_OptionB_Total_Compensation_5yr_2026-10-07.png (incl Y5 hold annotation)</t>
+        </is>
+      </c>
+    </row>
     <row r="33">
-      <c r="A33" s="12" t="n"/>
+      <c r="A33" s="12" t="inlineStr">
+        <is>
+          <t>HOLD TO YEAR 5 — Forward Potential if SSLC Investors Hold Exos Shares to FY31 (John 10/7)</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="32" customHeight="1">
-      <c r="A34" s="68" t="n"/>
+      <c r="A34" s="68" t="inlineStr">
+        <is>
+          <t>Base = Old-Model (v12). Dilution: Series A $25M staged (D1-D4, ~13%) + RTO (~12%) + option pool (~5%) = ~30% flat (MANAGEMENT ASSUMPTION). 0.75% stake at listing → 0.525% post-dilution. AA case EV ~$176M = BELOW $250M listing — stock worth less in AA case by FY31.</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="22" customHeight="1">
-      <c r="A35" s="69" t="n"/>
-      <c r="B35" s="69" t="n"/>
-      <c r="C35" s="69" t="n"/>
-      <c r="D35" s="69" t="n"/>
-      <c r="E35" s="69" t="n"/>
-      <c r="F35" s="69" t="n"/>
-      <c r="G35" s="69" t="n"/>
-      <c r="H35" s="69" t="n"/>
+      <c r="A35" s="69" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="B35" s="69" t="inlineStr">
+        <is>
+          <t>FY31 EV</t>
+        </is>
+      </c>
+      <c r="C35" s="69" t="inlineStr">
+        <is>
+          <t>Post-dil stake</t>
+        </is>
+      </c>
+      <c r="D35" s="69" t="inlineStr">
+        <is>
+          <t>FY31 share value</t>
+        </is>
+      </c>
+      <c r="E35" s="69" t="inlineStr">
+        <is>
+          <t>At-listing value</t>
+        </is>
+      </c>
+      <c r="F35" s="69" t="inlineStr">
+        <is>
+          <t>Multiple vs listing</t>
+        </is>
+      </c>
+      <c r="G35" s="69" t="inlineStr"/>
+      <c r="H35" s="69" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="29" t="inlineStr">
@@ -6718,11 +6541,16 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="9">
     <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A25:H25"/>
     <mergeCell ref="A43:H43"/>
     <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A13:H13"/>
+    <mergeCell ref="A33:H33"/>
     <mergeCell ref="A5:H5"/>
+    <mergeCell ref="A31:H31"/>
+    <mergeCell ref="A34:H34"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7210,36 +7038,9 @@
           <t>KEY FACT:  Reaching $5.1M in FY27 requires averaging $1.46M/quarter for Q2–Q4  ($5,100K − $713K Q1 actual ÷ 3 quarters = $1,462K/qtr)  —  approximately 2.05× the most recent quarter's $713K  —  starting immediately.  Without Exos capital to fund working capital and IM ramp, that doubling is not achievable on SSLC's $198K cash position.</t>
         </is>
       </c>
-      <c r="B4" s="126" t="n"/>
-      <c r="C4" s="126" t="n"/>
-      <c r="D4" s="126" t="n"/>
-      <c r="E4" s="126" t="n"/>
-      <c r="F4" s="126" t="n"/>
-      <c r="G4" s="126" t="n"/>
-      <c r="H4" s="126" t="n"/>
-      <c r="I4" s="126" t="n"/>
-      <c r="J4" s="126" t="n"/>
-      <c r="K4" s="126" t="n"/>
-      <c r="L4" s="127" t="n"/>
-    </row>
-    <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="128" t="n"/>
-      <c r="L5" s="129" t="n"/>
-    </row>
-    <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="130" t="n"/>
-      <c r="B6" s="131" t="n"/>
-      <c r="C6" s="131" t="n"/>
-      <c r="D6" s="131" t="n"/>
-      <c r="E6" s="131" t="n"/>
-      <c r="F6" s="131" t="n"/>
-      <c r="G6" s="131" t="n"/>
-      <c r="H6" s="131" t="n"/>
-      <c r="I6" s="131" t="n"/>
-      <c r="J6" s="131" t="n"/>
-      <c r="K6" s="131" t="n"/>
-      <c r="L6" s="132" t="n"/>
-    </row>
+    </row>
+    <row r="5" ht="22" customHeight="1"/>
+    <row r="6" ht="22" customHeight="1"/>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="80" t="inlineStr">
         <is>
@@ -7296,10 +7097,6 @@
           <t xml:space="preserve">  Cash on hand (10/2/26):  $198K</t>
         </is>
       </c>
-      <c r="I10" s="133" t="n"/>
-      <c r="J10" s="133" t="n"/>
-      <c r="K10" s="133" t="n"/>
-      <c r="L10" s="134" t="n"/>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="86" t="inlineStr">
@@ -7327,10 +7124,6 @@
           <t xml:space="preserve">  Working capital needed to maintain deliveries:  $300K–$700K</t>
         </is>
       </c>
-      <c r="I11" s="133" t="n"/>
-      <c r="J11" s="133" t="n"/>
-      <c r="K11" s="133" t="n"/>
-      <c r="L11" s="134" t="n"/>
     </row>
     <row r="12" ht="16" customHeight="1">
       <c r="A12" s="86" t="inlineStr">
@@ -7356,10 +7149,6 @@
           <t xml:space="preserve">  FY26 operating loss:  −$416K</t>
         </is>
       </c>
-      <c r="I12" s="133" t="n"/>
-      <c r="J12" s="133" t="n"/>
-      <c r="K12" s="133" t="n"/>
-      <c r="L12" s="134" t="n"/>
     </row>
     <row r="13" ht="16" customHeight="1">
       <c r="A13" s="86" t="inlineStr">
@@ -7387,10 +7176,6 @@
           <t xml:space="preserve">  He-tank rework unresolved — no resolution path without new owner</t>
         </is>
       </c>
-      <c r="I13" s="133" t="n"/>
-      <c r="J13" s="133" t="n"/>
-      <c r="K13" s="133" t="n"/>
-      <c r="L13" s="134" t="n"/>
     </row>
     <row r="14" ht="16" customHeight="1">
       <c r="A14" s="86" t="inlineStr">
@@ -7418,10 +7203,6 @@
           <t xml:space="preserve">  No capex capacity → headcount/equipment frozen</t>
         </is>
       </c>
-      <c r="I14" s="133" t="n"/>
-      <c r="J14" s="133" t="n"/>
-      <c r="K14" s="133" t="n"/>
-      <c r="L14" s="134" t="n"/>
     </row>
     <row r="15" ht="16" customHeight="1">
       <c r="A15" s="94" t="inlineStr">
@@ -7434,10 +7215,6 @@
           <t xml:space="preserve">  Growth capped by self-funded working capital</t>
         </is>
       </c>
-      <c r="I15" s="133" t="n"/>
-      <c r="J15" s="133" t="n"/>
-      <c r="K15" s="133" t="n"/>
-      <c r="L15" s="134" t="n"/>
     </row>
     <row r="16" ht="16" customHeight="1">
       <c r="H16" s="85" t="inlineStr">
@@ -7445,10 +7222,6 @@
           <t xml:space="preserve">  FY27 achievable at run-rate:  ~$2.85M</t>
         </is>
       </c>
-      <c r="I16" s="133" t="n"/>
-      <c r="J16" s="133" t="n"/>
-      <c r="K16" s="133" t="n"/>
-      <c r="L16" s="134" t="n"/>
     </row>
     <row r="17" ht="16" customHeight="1">
       <c r="A17" s="95" t="inlineStr">
@@ -7461,10 +7234,6 @@
           <t xml:space="preserve">  FY31 best-case (10% CAGR, no stall):  ~$4.2M</t>
         </is>
       </c>
-      <c r="I17" s="133" t="n"/>
-      <c r="J17" s="133" t="n"/>
-      <c r="K17" s="133" t="n"/>
-      <c r="L17" s="134" t="n"/>
     </row>
     <row r="18" ht="16" customHeight="1">
       <c r="A18" s="96" t="inlineStr">
@@ -7477,10 +7246,6 @@
           <t xml:space="preserve">  5-yr CAGR (status quo):  ~10.0%</t>
         </is>
       </c>
-      <c r="I18" s="133" t="n"/>
-      <c r="J18" s="133" t="n"/>
-      <c r="K18" s="133" t="n"/>
-      <c r="L18" s="134" t="n"/>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="84" t="inlineStr"/>
@@ -7561,10 +7326,6 @@
           <t xml:space="preserve">  Cash at close:  $2.51M</t>
         </is>
       </c>
-      <c r="I21" s="133" t="n"/>
-      <c r="J21" s="133" t="n"/>
-      <c r="K21" s="133" t="n"/>
-      <c r="L21" s="134" t="n"/>
     </row>
     <row r="22" ht="16" customHeight="1">
       <c r="A22" s="86" t="inlineStr">
@@ -7592,10 +7353,6 @@
           <t xml:space="preserve">  SSLC debts paid at face (est. ~$500K TBV)</t>
         </is>
       </c>
-      <c r="I22" s="133" t="n"/>
-      <c r="J22" s="133" t="n"/>
-      <c r="K22" s="133" t="n"/>
-      <c r="L22" s="134" t="n"/>
     </row>
     <row r="23" ht="16" customHeight="1">
       <c r="A23" s="86" t="inlineStr">
@@ -7623,10 +7380,6 @@
           <t xml:space="preserve">  Prepaid-work delivery funded (cost $500K)</t>
         </is>
       </c>
-      <c r="I23" s="133" t="n"/>
-      <c r="J23" s="133" t="n"/>
-      <c r="K23" s="133" t="n"/>
-      <c r="L23" s="134" t="n"/>
     </row>
     <row r="24" ht="16" customHeight="1">
       <c r="H24" s="85" t="inlineStr">
@@ -7634,10 +7387,6 @@
           <t xml:space="preserve">  WC bridge removes Q2–Q3 stall risk</t>
         </is>
       </c>
-      <c r="I24" s="133" t="n"/>
-      <c r="J24" s="133" t="n"/>
-      <c r="K24" s="133" t="n"/>
-      <c r="L24" s="134" t="n"/>
     </row>
     <row r="25" ht="16" customHeight="1">
       <c r="A25" s="81" t="inlineStr">
@@ -7650,10 +7399,6 @@
           <t xml:space="preserve">  Exos procurement channel:  immediate BLK3 tank POs</t>
         </is>
       </c>
-      <c r="I25" s="133" t="n"/>
-      <c r="J25" s="133" t="n"/>
-      <c r="K25" s="133" t="n"/>
-      <c r="L25" s="134" t="n"/>
     </row>
     <row r="26" ht="16" customHeight="1">
       <c r="A26" s="84" t="inlineStr">
@@ -7686,10 +7431,6 @@
           <t xml:space="preserve">  Intuitive Machines ramp:  14–16 tanks firm FY27</t>
         </is>
       </c>
-      <c r="I26" s="133" t="n"/>
-      <c r="J26" s="133" t="n"/>
-      <c r="K26" s="133" t="n"/>
-      <c r="L26" s="134" t="n"/>
     </row>
     <row r="27" ht="16" customHeight="1">
       <c r="A27" s="101" t="inlineStr">
@@ -7708,10 +7449,6 @@
           <t xml:space="preserve">  Capex for production scale-up enabled</t>
         </is>
       </c>
-      <c r="I27" s="133" t="n"/>
-      <c r="J27" s="133" t="n"/>
-      <c r="K27" s="133" t="n"/>
-      <c r="L27" s="134" t="n"/>
     </row>
     <row r="28" ht="16" customHeight="1">
       <c r="A28" s="101" t="inlineStr">
@@ -7730,10 +7467,6 @@
           <t xml:space="preserve">  FY27 target (IM firm + ramp):  $4.1M–$5.5M</t>
         </is>
       </c>
-      <c r="I28" s="133" t="n"/>
-      <c r="J28" s="133" t="n"/>
-      <c r="K28" s="133" t="n"/>
-      <c r="L28" s="134" t="n"/>
     </row>
     <row r="29" ht="16" customHeight="1">
       <c r="A29" s="101" t="inlineStr">
@@ -7752,10 +7485,6 @@
           <t xml:space="preserve">  FY31 (v12 trajectory):  $54.7M</t>
         </is>
       </c>
-      <c r="I29" s="133" t="n"/>
-      <c r="J29" s="133" t="n"/>
-      <c r="K29" s="133" t="n"/>
-      <c r="L29" s="134" t="n"/>
     </row>
     <row r="30" ht="16" customHeight="1">
       <c r="A30" s="101" t="inlineStr">
@@ -7774,10 +7503,6 @@
           <t xml:space="preserve">  5-yr CAGR (with Exos, v12):  ~90.9%</t>
         </is>
       </c>
-      <c r="I30" s="133" t="n"/>
-      <c r="J30" s="133" t="n"/>
-      <c r="K30" s="133" t="n"/>
-      <c r="L30" s="134" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="101" t="inlineStr">
@@ -7812,10 +7537,6 @@
           <t xml:space="preserve">  FY27 $5.1M target − Q1 $713K actual = $4,387K remaining</t>
         </is>
       </c>
-      <c r="I33" s="133" t="n"/>
-      <c r="J33" s="133" t="n"/>
-      <c r="K33" s="133" t="n"/>
-      <c r="L33" s="134" t="n"/>
     </row>
     <row r="34" ht="16" customHeight="1">
       <c r="H34" s="85" t="inlineStr">
@@ -7823,10 +7544,6 @@
           <t xml:space="preserve">  Over 3 quarters (Q2–Q4) = $1,462K/qtr required</t>
         </is>
       </c>
-      <c r="I34" s="133" t="n"/>
-      <c r="J34" s="133" t="n"/>
-      <c r="K34" s="133" t="n"/>
-      <c r="L34" s="134" t="n"/>
     </row>
     <row r="35" ht="16" customHeight="1">
       <c r="H35" s="85" t="inlineStr">
@@ -7834,10 +7551,6 @@
           <t xml:space="preserve">  vs. Q1 $713K actual = 2.05× immediate ramp</t>
         </is>
       </c>
-      <c r="I35" s="133" t="n"/>
-      <c r="J35" s="133" t="n"/>
-      <c r="K35" s="133" t="n"/>
-      <c r="L35" s="134" t="n"/>
     </row>
     <row r="36" ht="16" customHeight="1">
       <c r="H36" s="85" t="inlineStr">
@@ -7845,10 +7558,6 @@
           <t xml:space="preserve">  Only funded if Exos capital bridges the working-capital gap</t>
         </is>
       </c>
-      <c r="I36" s="133" t="n"/>
-      <c r="J36" s="133" t="n"/>
-      <c r="K36" s="133" t="n"/>
-      <c r="L36" s="134" t="n"/>
     </row>
     <row r="37" ht="16" customHeight="1">
       <c r="H37" s="85" t="inlineStr">
@@ -7856,10 +7565,6 @@
           <t xml:space="preserve">  Without capital → Q2–Q4 stays ≈ $713K/qtr = $2.85M FY27</t>
         </is>
       </c>
-      <c r="I37" s="133" t="n"/>
-      <c r="J37" s="133" t="n"/>
-      <c r="K37" s="133" t="n"/>
-      <c r="L37" s="134" t="n"/>
     </row>
     <row r="40" ht="28" customHeight="1">
       <c r="A40" s="108" t="inlineStr">

</xml_diff>

<commit_message>
SSLC v-next offer: 0.5% EAI at close + reduced stock earn-out (10/9)
- Add 0.5% EAI units at close (~$850K at Eqvista 409A $169.7M); subtotal at close → $5.21M
- Stock earn-out: 0.0%/0.25%/0.5% earn-out only (total Exos equity 0.5%/0.75%/1.0%)
- New totals: LOW $6.16M / BASE $7.74M / HIGH $9.31M
- HIGH < $10M target — not rebalanced per John's instruction (10/9)
- Updated: model xlsx, chart PNG, offer summary docx+pdf, v2 draft docx
- All 4 artifacts re-attached to MC #2414
</commit_message>
<xml_diff>
--- a/drafts/EXOS_SSLC_OptionB_Acquisition_Model_2026-10-07.xlsx
+++ b/drafts/EXOS_SSLC_OptionB_Acquisition_Model_2026-10-07.xlsx
@@ -1242,45 +1242,45 @@
     <row r="28" ht="22" customHeight="1">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Earn-out ii — Exos stock % of FD shares (low)</t>
+          <t>Earn-out ii — Exos stock % of FD shares (low, earn-out only)</t>
         </is>
       </c>
       <c r="B28" s="9" t="n">
-        <v>0.005</v>
+        <v>0</v>
       </c>
       <c r="C28" s="10" t="inlineStr">
         <is>
-          <t>Management assumption — unverified</t>
+          <t>0.0% earn-out; total = 0.5% EAI up-front + 0.0% = 0.5%</t>
         </is>
       </c>
     </row>
     <row r="29" ht="22" customHeight="1">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>Earn-out ii — Exos stock % of FD shares (base)</t>
+          <t>Earn-out ii — Exos stock % of FD shares (base, earn-out only)</t>
         </is>
       </c>
       <c r="B29" s="9" t="n">
-        <v>0.0075</v>
+        <v>0.0025</v>
       </c>
       <c r="C29" s="10" t="inlineStr">
         <is>
-          <t>Management assumption — unverified</t>
+          <t>0.25% earn-out; total = 0.5% EAI up-front + 0.25% = 0.75%</t>
         </is>
       </c>
     </row>
     <row r="30" ht="22" customHeight="1">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>Earn-out ii — Exos stock % of FD shares (high)</t>
+          <t>Earn-out ii — Exos stock % of FD shares (high, earn-out only)</t>
         </is>
       </c>
       <c r="B30" s="9" t="n">
-        <v>0.01</v>
+        <v>0.005</v>
       </c>
       <c r="C30" s="10" t="inlineStr">
         <is>
-          <t>Management assumption — unverified</t>
+          <t>0.5% earn-out; total = 0.5% EAI up-front + 0.5% = 1.0%</t>
         </is>
       </c>
     </row>
@@ -1344,6 +1344,21 @@
         </is>
       </c>
     </row>
+    <row r="35" ht="22" customHeight="1">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>EAI up-front equity — % FD shares at close</t>
+        </is>
+      </c>
+      <c r="B35" s="9" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="C35" s="10" t="inlineStr">
+        <is>
+          <t>0.5% EAI units committed at SSLC board acceptance; issued at financing close</t>
+        </is>
+      </c>
+    </row>
     <row r="36" ht="20" customHeight="1">
       <c r="A36" s="11" t="inlineStr">
         <is>
@@ -2289,17 +2304,17 @@
     <row r="111" ht="20" customHeight="1">
       <c r="A111" s="5" t="inlineStr">
         <is>
-          <t>6. Earn-out upside — Exos stock post-RTO</t>
+          <t>6. Up-front EAI equity + stock earn-out upside</t>
         </is>
       </c>
       <c r="B111" s="5" t="inlineStr">
         <is>
-          <t>$1.0M–$3.0M</t>
+          <t>$850K + $0–$1.5M</t>
         </is>
       </c>
       <c r="C111" s="7" t="inlineStr">
         <is>
-          <t>0.5%–1.0% FD at listing ($200M–$300M MEV)</t>
+          <t>0.5% EAI at close; 0.0–0.5% earn-out at listing ($200M–$300M)</t>
         </is>
       </c>
     </row>
@@ -2424,15 +2439,16 @@
     <row r="121" ht="28" customHeight="1">
       <c r="A121" s="13" t="inlineStr">
         <is>
-          <t>SSLC earn-out stock stake at listing (base)</t>
-        </is>
-      </c>
-      <c r="B121" s="20" t="n">
-        <v>0.0075</v>
+          <t>SSLC TOTAL stock stake at listing (base = 0.5% EAI + 0.25% earn-out)</t>
+        </is>
+      </c>
+      <c r="B121" s="20">
+        <f>B35+B29</f>
+        <v/>
       </c>
       <c r="C121" s="19" t="inlineStr">
         <is>
-          <t>Base earn-out grant = 0.75% FD shares at listing</t>
+          <t>Total stake base = 0.5% up-front EAI + 0.25% earn-out = 0.75% FD</t>
         </is>
       </c>
     </row>
@@ -2470,7 +2486,7 @@
     <row r="124" ht="28" customHeight="1">
       <c r="A124" s="13" t="inlineStr">
         <is>
-          <t>SSLC stake FY31 — base post-dilution</t>
+          <t>SSLC stake FY31 — base post-dilution (total 0.75%)</t>
         </is>
       </c>
       <c r="B124" s="20">
@@ -2486,32 +2502,32 @@
     <row r="125" ht="28" customHeight="1">
       <c r="A125" s="13" t="inlineStr">
         <is>
-          <t>SSLC stake FY31 — low post-dilution</t>
+          <t>SSLC stake FY31 — low post-dilution (total 0.5% EAI only)</t>
         </is>
       </c>
       <c r="B125" s="20">
-        <f>Assumptions!B28*(1-B122)</f>
+        <f>(B35+B28)*(1-B122)</f>
         <v/>
       </c>
       <c r="C125" s="19" t="inlineStr">
         <is>
-          <t>0.5% x 0.70 = 0.35%</t>
+          <t>0.5%+0.0% = 0.5% x 0.70 = 0.35%</t>
         </is>
       </c>
     </row>
     <row r="126" ht="28" customHeight="1">
       <c r="A126" s="13" t="inlineStr">
         <is>
-          <t>SSLC stake FY31 — high post-dilution</t>
+          <t>SSLC stake FY31 — high post-dilution (total 1.0%)</t>
         </is>
       </c>
       <c r="B126" s="20">
-        <f>Assumptions!B30*(1-B122)</f>
+        <f>(B35+B30)*(1-B122)</f>
         <v/>
       </c>
       <c r="C126" s="19" t="inlineStr">
         <is>
-          <t>1.0% x 0.70 = 0.70%</t>
+          <t>(0.5%+0.5%) = 1.0% x 0.70 = 0.70%</t>
         </is>
       </c>
     </row>
@@ -2614,7 +2630,7 @@
     <row r="133" ht="28" customHeight="1">
       <c r="A133" s="13" t="inlineStr">
         <is>
-          <t>Multiple v at-listing — Old-Model base</t>
+          <t>Multiple v earn-out at-listing — Old-Model base</t>
         </is>
       </c>
       <c r="B133" s="20">
@@ -2623,14 +2639,14 @@
       </c>
       <c r="C133" s="19" t="inlineStr">
         <is>
-          <t>~4.6x the at-listing stock earn-out value ($1.875M)</t>
+          <t>Compares FY31 hold value to earn-out-only at-listing ($625K); multiple reflects earn-out upside only</t>
         </is>
       </c>
     </row>
     <row r="134" ht="28" customHeight="1">
       <c r="A134" s="13" t="inlineStr">
         <is>
-          <t>Multiple v at-listing — AA base</t>
+          <t>Multiple v earn-out at-listing — AA base</t>
         </is>
       </c>
       <c r="B134" s="20">
@@ -2639,7 +2655,7 @@
       </c>
       <c r="C134" s="19" t="inlineStr">
         <is>
-          <t>~0.49x — AA FY31 EV BELOW listing; stock worth less by FY31 in AA case</t>
+          <t>AA FY31 EV BELOW listing; stock worth less by FY31 in AA case (earn-out portion only)</t>
         </is>
       </c>
     </row>
@@ -3001,7 +3017,7 @@
       </c>
       <c r="E24" s="10" t="inlineStr">
         <is>
-          <t>Low: 3% tank rev (cap $300K) × 5yr + 0.5% of $200M listing + milestone 1 only</t>
+          <t>Low: 3% tank rev (cap $300K) × 5yr + 0.0% earn-out stock (0.5% EAI up-front only) + milestone 1 only</t>
         </is>
       </c>
     </row>
@@ -3025,7 +3041,7 @@
       </c>
       <c r="E25" s="10" t="inlineStr">
         <is>
-          <t>Base: 5% × $5M firm × 5yr + 0.75% of $250M listing + milestones 1-3</t>
+          <t>Base: 5% × $5M firm × 5yr + 0.25% earn-out of $250M listing ($625K) + milestones 1-3</t>
         </is>
       </c>
     </row>
@@ -3049,14 +3065,14 @@
       </c>
       <c r="E26" s="10" t="inlineStr">
         <is>
-          <t>High: 7% × $5M (cap $300K) × 5yr + 1.0% of $300M listing + all 5 milestones → ~$10M</t>
+          <t>High: 7% × $5M (cap $300K) × 5yr + 0.5% earn-out of $300M listing + all 5 milestones → ~$9.3M</t>
         </is>
       </c>
     </row>
     <row r="27" ht="28" customHeight="1">
       <c r="A27" s="29" t="inlineStr">
         <is>
-          <t>Exos dilution (stock, base)</t>
+          <t>Exos dilution (stock earn-out, base)</t>
         </is>
       </c>
       <c r="B27" s="29" t="inlineStr">
@@ -3074,7 +3090,7 @@
       </c>
       <c r="E27" s="10" t="inlineStr">
         <is>
-          <t>0.75% of FD shares; non-material at Series A scale</t>
+          <t>0.25% earn-out FD shares (plus 0.5% EAI up-front = 0.75% total); non-material at Series A scale</t>
         </is>
       </c>
     </row>
@@ -5811,6 +5827,38 @@
         </is>
       </c>
     </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="58" t="inlineStr">
+        <is>
+          <t>Exos equity — 0.5% EAI units at 409A (~$170M)</t>
+        </is>
+      </c>
+      <c r="B11" s="31">
+        <f>Assumptions!B36</f>
+        <v/>
+      </c>
+      <c r="C11" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="31" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="31">
+        <f>SUM(B11:F11)</f>
+        <v/>
+      </c>
+      <c r="H11" s="10" t="inlineStr">
+        <is>
+          <t>~$850K; committed at SSLC board acceptance; issued at financing close</t>
+        </is>
+      </c>
+    </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="59" t="inlineStr">
         <is>
@@ -5818,23 +5866,23 @@
         </is>
       </c>
       <c r="B12" s="60">
-        <f>SUM(B6:B10)</f>
+        <f>SUM(B6:B11)</f>
         <v/>
       </c>
       <c r="C12" s="60">
-        <f>SUM(C6:C10)</f>
+        <f>SUM(C6:C11)</f>
         <v/>
       </c>
       <c r="D12" s="60">
-        <f>SUM(D6:D10)</f>
+        <f>SUM(D6:D11)</f>
         <v/>
       </c>
       <c r="E12" s="60">
-        <f>SUM(E6:E10)</f>
+        <f>SUM(E6:E11)</f>
         <v/>
       </c>
       <c r="F12" s="60">
-        <f>SUM(F6:F10)</f>
+        <f>SUM(F6:F11)</f>
         <v/>
       </c>
       <c r="G12" s="60">
@@ -5843,7 +5891,7 @@
       </c>
       <c r="H12" s="10" t="inlineStr">
         <is>
-          <t>All at close in FY27</t>
+          <t>All at close in FY27; includes EAI equity at 409A</t>
         </is>
       </c>
     </row>
@@ -6058,7 +6106,7 @@
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="58" t="inlineStr">
         <is>
-          <t>Stock earn-out base (ii): 0.75% FD @ listing</t>
+          <t>Stock earn-out base (ii): 0.25% FD @ listing (total 0.75% incl. EAI)</t>
         </is>
       </c>
       <c r="B20" s="31" t="n">
@@ -6083,14 +6131,14 @@
       </c>
       <c r="H20" s="10" t="inlineStr">
         <is>
-          <t>At $250M listing; realized FY29 post principals' lockup (modeled ~12 months)</t>
+          <t>0.25% earn-out at $250M listing = $625K; realized FY29 post principals' lockup. Also = $425K at 409A ($170M).</t>
         </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="58" t="inlineStr">
         <is>
-          <t>Stock earn-out low (ii): 0.5% @ $200M</t>
+          <t>Stock earn-out low (ii): 0.0% earn-out (0.5% EAI up-front only)</t>
         </is>
       </c>
       <c r="B21" s="31" t="n">
@@ -6115,14 +6163,14 @@
       </c>
       <c r="H21" s="10" t="inlineStr">
         <is>
-          <t>Low RTO</t>
+          <t>0.0% earn-out = $0 at listing; total Exos equity = 0.5% EAI only. At 409A = $0.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="58" t="inlineStr">
         <is>
-          <t>Stock earn-out high (ii): 1.0% @ $300M</t>
+          <t>Stock earn-out high (ii): 0.5% @ $300M (total 1.0% incl. EAI)</t>
         </is>
       </c>
       <c r="B22" s="31" t="n">
@@ -6147,7 +6195,7 @@
       </c>
       <c r="H22" s="10" t="inlineStr">
         <is>
-          <t>High RTO</t>
+          <t>0.5% earn-out at $300M = $1.5M; also = $850K at 409A ($170M). Total Exos equity = 1.0%.</t>
         </is>
       </c>
     </row>
@@ -6161,7 +6209,7 @@
     <row r="26" ht="20" customHeight="1">
       <c r="A26" s="26" t="inlineStr">
         <is>
-          <t>BASE: funding + tank base (5yr) + milestones 1-3 + stock base</t>
+          <t>BASE: funding+EAI ($5.21M) + tank base (5yr) + milestones 1-3 + stock earn-out base ≈ $7.74M</t>
         </is>
       </c>
       <c r="B26" s="62">
@@ -6192,7 +6240,7 @@
     <row r="27" ht="20" customHeight="1">
       <c r="A27" s="63" t="inlineStr">
         <is>
-          <t>LOW:  funding + tank low (5yr) + milestone M1 only + stock low</t>
+          <t>LOW:  funding+EAI ($5.21M) + tank low (5yr) + milestone M1 only + 0% earn-out ≈ $6.16M</t>
         </is>
       </c>
       <c r="B27" s="64">
@@ -6223,7 +6271,7 @@
     <row r="28" ht="20" customHeight="1">
       <c r="A28" s="65" t="inlineStr">
         <is>
-          <t>HIGH: funding + tank high (5yr) + all milestones + stock high  ≈ $10.0M</t>
+          <t>HIGH: funding+EAI ($5.21M) + tank high + all milestones + 0.5% earn-out ≈ $9.31M [HIGH &lt; $10M target — not rebalanced per 10/9 instruction]</t>
         </is>
       </c>
       <c r="B28" s="66">
@@ -6299,7 +6347,7 @@
     <row r="34" ht="32" customHeight="1">
       <c r="A34" s="68" t="inlineStr">
         <is>
-          <t>Base = Old-Model (v12). Dilution: Series A $25M staged (D1-D4, ~13%) + RTO (~12%) + option pool (~5%) = ~30% flat (MANAGEMENT ASSUMPTION). 0.75% stake at listing → 0.525% post-dilution. AA case EV ~$176M = BELOW $250M listing — stock worth less in AA case by FY31.</t>
+          <t>Base = Old-Model (v12). Dilution: Series A $25M staged (D1-D4, ~13%) + RTO (~12%) + option pool (~5%) = ~30% flat (MANAGEMENT ASSUMPTION). TOTAL stake at listing: 0.5% EAI up-front + earn-out % = 0.5/0.75/1.0% low/base/high → 0.35/0.525/0.70% post-dilution. AA case EV ~$176M = BELOW $250M listing — stock worth less in AA case by FY31.</t>
         </is>
       </c>
     </row>
@@ -6369,7 +6417,7 @@
       </c>
       <c r="H36" s="71" t="inlineStr">
         <is>
-          <t>0.5% grant x 0.70 = 0.35%; EV $1.626B</t>
+          <t>Total 0.5% (EAI only, 0% earn-out) x 0.70 = 0.35%; EV $1.626B; multiple vs earn-out at listing ($0)</t>
         </is>
       </c>
     </row>
@@ -6401,7 +6449,7 @@
       </c>
       <c r="H37" s="71" t="inlineStr">
         <is>
-          <t>0.75% grant x 0.70 = 0.525%; EV $1.626B (~4.6x listing)</t>
+          <t>Total 0.75% (0.5% EAI + 0.25% earn-out) x 0.70 = 0.525%; EV $1.626B; vs earn-out at listing $625K</t>
         </is>
       </c>
     </row>
@@ -6433,7 +6481,7 @@
       </c>
       <c r="H38" s="71" t="inlineStr">
         <is>
-          <t>1.0% grant x 0.70 = 0.70%; EV $1.626B</t>
+          <t>Total 1.0% (0.5% EAI + 0.5% earn-out) x 0.70 = 0.70%; EV $1.626B; vs earn-out at listing $1.5M</t>
         </is>
       </c>
     </row>
@@ -6465,7 +6513,7 @@
       </c>
       <c r="H39" s="71" t="inlineStr">
         <is>
-          <t>BELOW listing value — AA FY31 EV ~$176M &lt; $250M MEV</t>
+          <t>BELOW listing value — AA FY31 EV ~$176M &lt; $250M MEV; earn-out = $0</t>
         </is>
       </c>
     </row>
@@ -6497,7 +6545,7 @@
       </c>
       <c r="H40" s="71" t="inlineStr">
         <is>
-          <t>BELOW listing — ~$924K vs $1.875M at listing (~0.49x)</t>
+          <t>BELOW listing — ~$924K vs earn-out at listing $625K</t>
         </is>
       </c>
     </row>
@@ -6529,7 +6577,7 @@
       </c>
       <c r="H41" s="71" t="inlineStr">
         <is>
-          <t>BELOW listing — ~$1.23M vs $3.0M at listing (~0.41x)</t>
+          <t>BELOW listing — ~$1.23M vs earn-out at listing $1.5M</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SSLC Option B: 1.0% EAI up-front equity (Rule 504), re-verify totals — task #2414
John change 2026-10-09 14:12:
- Up-front equity: 0.5% → 1.0% EAI units (Rule 504, at 409A $169.7M = ~$1.697M)
- Subtotal at close: ~$5.21M → ~$6.06M
- Stock earn-out unchanged: 0.0%/0.25%/0.5%; total equity: 1.0%/1.25%/1.5%
- Expected totals: ~$7.0M / $8.58M / $10.16M (HIGH back above $10M)
- Offer summary: equity described as 'EAI units issued as part of Exos's Rule 504 offering'
- Model notes: Rule 504 $10M cap reminder + sec.gov reference; Rule 504 U.S.-only vs Japan Reg S flag

Files rebuilt: XLSX model, PNG chart, DOCX/PDF offer summary (re-attached to MC #2414 as v3/v4)
</commit_message>
<xml_diff>
--- a/drafts/EXOS_SSLC_OptionB_Acquisition_Model_2026-10-07.xlsx
+++ b/drafts/EXOS_SSLC_OptionB_Acquisition_Model_2026-10-07.xlsx
@@ -14,7 +14,6 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Total Compensation" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reconciliation" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="With vs Without Exos Capital" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -30,7 +29,7 @@
     <numFmt numFmtId="167" formatCode="0.0x"/>
     <numFmt numFmtId="168" formatCode="0.00x"/>
   </numFmts>
-  <fonts count="31">
+  <fonts count="22">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -131,49 +130,8 @@
       <color rgb="00C00000"/>
       <sz val="8"/>
     </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="00555555"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00000000"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="009B1C1C"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <color rgb="00000000"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <color rgb="009B1C1C"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="00375623"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="00000000"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <sz val="9.5"/>
-    </font>
   </fonts>
-  <fills count="19">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -245,28 +203,8 @@
         <fgColor rgb="00E26A21"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="009B1C1C"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00375623"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00BF8F00"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="3">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -274,39 +212,11 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color rgb="00BF8F00"/>
-      </left>
-      <right style="medium">
-        <color rgb="00BF8F00"/>
-      </right>
-      <top style="medium">
-        <color rgb="00BF8F00"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="00BF8F00"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="00CCCCCC"/>
-      </left>
-      <right style="thin">
-        <color rgb="00CCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="00CCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00CCCCCC"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="109">
+  <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -421,100 +331,6 @@
     <xf numFmtId="166" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="26" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="165" fontId="26" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="165" fontId="26" fillId="16" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="27" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="27" fillId="16" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="26" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="26" fillId="16" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="29" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="17" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="165" fontId="6" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1250,7 +1066,7 @@
       </c>
       <c r="C28" s="10" t="inlineStr">
         <is>
-          <t>0.0% earn-out; total = 0.5% EAI up-front + 0.0% = 0.5%</t>
+          <t>0.0% earn-out; total = 1.0% EAI up-front + 0.0% = 1.0%</t>
         </is>
       </c>
     </row>
@@ -1265,7 +1081,7 @@
       </c>
       <c r="C29" s="10" t="inlineStr">
         <is>
-          <t>0.25% earn-out; total = 0.5% EAI up-front + 0.25% = 0.75%</t>
+          <t>0.25% earn-out; total = 1.0% EAI up-front + 0.25% = 1.25%</t>
         </is>
       </c>
     </row>
@@ -1280,7 +1096,7 @@
       </c>
       <c r="C30" s="10" t="inlineStr">
         <is>
-          <t>0.5% earn-out; total = 0.5% EAI up-front + 0.5% = 1.0%</t>
+          <t>0.5% earn-out; total = 1.0% EAI up-front + 0.5% = 1.5%</t>
         </is>
       </c>
     </row>
@@ -1351,11 +1167,11 @@
         </is>
       </c>
       <c r="B35" s="9" t="n">
-        <v>0.005</v>
+        <v>0.01</v>
       </c>
       <c r="C35" s="10" t="inlineStr">
         <is>
-          <t>0.5% EAI units committed at SSLC board acceptance; issued at financing close</t>
+          <t>1.0% EAI units (Rule 504); committed at SSLC board acceptance; issued at financing close</t>
         </is>
       </c>
     </row>
@@ -2309,12 +2125,12 @@
       </c>
       <c r="B111" s="5" t="inlineStr">
         <is>
-          <t>$850K + $0–$1.5M</t>
+          <t>$1,697K + $0–$848K</t>
         </is>
       </c>
       <c r="C111" s="7" t="inlineStr">
         <is>
-          <t>0.5% EAI at close; 0.0–0.5% earn-out at listing ($200M–$300M)</t>
+          <t>1.0% EAI (Rule 504) at close; 0.0–0.5% earn-out at listing ($200M–$300M)</t>
         </is>
       </c>
     </row>
@@ -2439,7 +2255,7 @@
     <row r="121" ht="28" customHeight="1">
       <c r="A121" s="13" t="inlineStr">
         <is>
-          <t>SSLC TOTAL stock stake at listing (base = 0.5% EAI + 0.25% earn-out)</t>
+          <t>SSLC TOTAL stock stake at listing (base = 1.0% EAI + 0.25% earn-out)</t>
         </is>
       </c>
       <c r="B121" s="20">
@@ -2448,7 +2264,7 @@
       </c>
       <c r="C121" s="19" t="inlineStr">
         <is>
-          <t>Total stake base = 0.5% up-front EAI + 0.25% earn-out = 0.75% FD</t>
+          <t>Total stake base = 1.0% up-front EAI (Rule 504) + 0.25% earn-out = 1.25% FD</t>
         </is>
       </c>
     </row>
@@ -2502,7 +2318,7 @@
     <row r="125" ht="28" customHeight="1">
       <c r="A125" s="13" t="inlineStr">
         <is>
-          <t>SSLC stake FY31 — low post-dilution (total 0.5% EAI only)</t>
+          <t>SSLC stake FY31 — low post-dilution (total 1.0% EAI only)</t>
         </is>
       </c>
       <c r="B125" s="20">
@@ -2511,14 +2327,14 @@
       </c>
       <c r="C125" s="19" t="inlineStr">
         <is>
-          <t>0.5%+0.0% = 0.5% x 0.70 = 0.35%</t>
+          <t>1.0%+0.0% = 1.0% x 0.70 = 0.70%</t>
         </is>
       </c>
     </row>
     <row r="126" ht="28" customHeight="1">
       <c r="A126" s="13" t="inlineStr">
         <is>
-          <t>SSLC stake FY31 — high post-dilution (total 1.0%)</t>
+          <t>SSLC stake FY31 — high post-dilution (total 1.5%)</t>
         </is>
       </c>
       <c r="B126" s="20">
@@ -2527,7 +2343,7 @@
       </c>
       <c r="C126" s="19" t="inlineStr">
         <is>
-          <t>(0.5%+0.5%) = 1.0% x 0.70 = 0.70%</t>
+          <t>(1.0%+0.5%) = 1.5% x 0.70 = 1.05%</t>
         </is>
       </c>
     </row>
@@ -2863,6 +2679,7 @@
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
+      <c r="A14" t="inlineStr"/>
       <c r="E14" s="10" t="inlineStr"/>
     </row>
     <row r="15" ht="18" customHeight="1">
@@ -3017,7 +2834,7 @@
       </c>
       <c r="E24" s="10" t="inlineStr">
         <is>
-          <t>Low: 3% tank rev (cap $300K) × 5yr + 0.0% earn-out stock (0.5% EAI up-front only) + milestone 1 only</t>
+          <t>Low: 3% tank rev (cap $300K) × 5yr + 0.0% earn-out stock (1.0% EAI up-front only, Rule 504) + milestone 1 only</t>
         </is>
       </c>
     </row>
@@ -3090,7 +2907,7 @@
       </c>
       <c r="E27" s="10" t="inlineStr">
         <is>
-          <t>0.25% earn-out FD shares (plus 0.5% EAI up-front = 0.75% total); non-material at Series A scale</t>
+          <t>0.25% earn-out FD shares (plus 1.0% EAI up-front = 1.25% total); non-material at Series A scale</t>
         </is>
       </c>
     </row>
@@ -5830,7 +5647,7 @@
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="58" t="inlineStr">
         <is>
-          <t>Exos equity — 0.5% EAI units at 409A (~$170M)</t>
+          <t>Exos equity — 1.0% EAI units at 409A (~$170M, Rule 504)</t>
         </is>
       </c>
       <c r="B11" s="31">
@@ -5855,7 +5672,7 @@
       </c>
       <c r="H11" s="10" t="inlineStr">
         <is>
-          <t>~$850K; committed at SSLC board acceptance; issued at financing close</t>
+          <t>~$1,697K; committed at SSLC board acceptance; issued at financing close (Rule 504)</t>
         </is>
       </c>
     </row>
@@ -6106,7 +5923,7 @@
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="58" t="inlineStr">
         <is>
-          <t>Stock earn-out base (ii): 0.25% FD @ listing (total 0.75% incl. EAI)</t>
+          <t>Stock earn-out base (ii): 0.25% FD @ listing (total 1.25% incl. EAI)</t>
         </is>
       </c>
       <c r="B20" s="31" t="n">
@@ -6131,14 +5948,14 @@
       </c>
       <c r="H20" s="10" t="inlineStr">
         <is>
-          <t>0.25% earn-out at $250M listing = $625K; realized FY29 post principals' lockup. Also = $425K at 409A ($170M).</t>
+          <t>0.25% earn-out at $250M listing = $625K; realized FY29 post principals' lockup. Also = $424K at 409A ($170M).</t>
         </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="58" t="inlineStr">
         <is>
-          <t>Stock earn-out low (ii): 0.0% earn-out (0.5% EAI up-front only)</t>
+          <t>Stock earn-out low (ii): 0.0% earn-out (1.0% EAI up-front only)</t>
         </is>
       </c>
       <c r="B21" s="31" t="n">
@@ -6163,14 +5980,14 @@
       </c>
       <c r="H21" s="10" t="inlineStr">
         <is>
-          <t>0.0% earn-out = $0 at listing; total Exos equity = 0.5% EAI only. At 409A = $0.</t>
+          <t>0.0% earn-out = $0 at listing; total Exos equity = 1.0% EAI (Rule 504) only. At 409A = $0.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="58" t="inlineStr">
         <is>
-          <t>Stock earn-out high (ii): 0.5% @ $300M (total 1.0% incl. EAI)</t>
+          <t>Stock earn-out high (ii): 0.5% @ $300M (total 1.5% incl. EAI)</t>
         </is>
       </c>
       <c r="B22" s="31" t="n">
@@ -6195,7 +6012,7 @@
       </c>
       <c r="H22" s="10" t="inlineStr">
         <is>
-          <t>0.5% earn-out at $300M = $1.5M; also = $850K at 409A ($170M). Total Exos equity = 1.0%.</t>
+          <t>0.5% earn-out at $300M = $1.5M; also = $848K at 409A ($170M). Total Exos equity = 1.5%.</t>
         </is>
       </c>
     </row>
@@ -6347,7 +6164,7 @@
     <row r="34" ht="32" customHeight="1">
       <c r="A34" s="68" t="inlineStr">
         <is>
-          <t>Base = Old-Model (v12). Dilution: Series A $25M staged (D1-D4, ~13%) + RTO (~12%) + option pool (~5%) = ~30% flat (MANAGEMENT ASSUMPTION). TOTAL stake at listing: 0.5% EAI up-front + earn-out % = 0.5/0.75/1.0% low/base/high → 0.35/0.525/0.70% post-dilution. AA case EV ~$176M = BELOW $250M listing — stock worth less in AA case by FY31.</t>
+          <t>Base = Old-Model (v12). Dilution: Series A $25M staged (D1-D4, ~13%) + RTO (~12%) + option pool (~5%) = ~30% flat (MANAGEMENT ASSUMPTION). TOTAL stake at listing: 1.0% EAI up-front (Rule 504) + earn-out % = 1.0/1.25/1.5% low/base/high → 0.70/0.875/1.05% post-dilution. AA case EV ~$176M = BELOW $250M listing — stock worth less in AA case by FY31.</t>
         </is>
       </c>
     </row>
@@ -6417,7 +6234,7 @@
       </c>
       <c r="H36" s="71" t="inlineStr">
         <is>
-          <t>Total 0.5% (EAI only, 0% earn-out) x 0.70 = 0.35%; EV $1.626B; multiple vs earn-out at listing ($0)</t>
+          <t>Total 1.0% (EAI only, 0% earn-out) x 0.70 = 0.70%; EV $1.626B; multiple vs earn-out at listing ($0)</t>
         </is>
       </c>
     </row>
@@ -6449,7 +6266,7 @@
       </c>
       <c r="H37" s="71" t="inlineStr">
         <is>
-          <t>Total 0.75% (0.5% EAI + 0.25% earn-out) x 0.70 = 0.525%; EV $1.626B; vs earn-out at listing $625K</t>
+          <t>Total 1.25% (1.0% EAI + 0.25% earn-out) x 0.70 = 0.875%; EV $1.626B; vs earn-out at listing $625K</t>
         </is>
       </c>
     </row>
@@ -6481,7 +6298,7 @@
       </c>
       <c r="H38" s="71" t="inlineStr">
         <is>
-          <t>Total 1.0% (0.5% EAI + 0.5% earn-out) x 0.70 = 0.70%; EV $1.626B; vs earn-out at listing $1.5M</t>
+          <t>Total 1.5% (1.0% EAI + 0.5% earn-out) x 0.70 = 1.05%; EV $1.626B; vs earn-out at listing $1.5M</t>
         </is>
       </c>
     </row>
@@ -6584,7 +6401,7 @@
     <row r="43" ht="42" customHeight="1">
       <c r="A43" s="73" t="inlineStr">
         <is>
-          <t>NOTE: Y5 hold values are NOT additive to at-listing earn-out. Investors choose to hold OR sell at listing. Old-Model base: hold to FY31 = ~$8.54M vs sell at listing = $1.875M (4.6x). AA base: hold to FY31 = ~$0.92M vs sell at listing = $1.875M (0.49x) — AA case penalizes holding.</t>
+          <t>NOTE: Y5 hold values are NOT additive to at-listing earn-out. Investors choose to hold OR sell at listing. Old-Model base: hold to FY31 = ~$8.54M vs sell at listing = $1.875M (4.6x). AA base: hold to FY31 = ~$0.92M vs sell at listing = $1.875M (0.49x) — AA case penalizes holding. Model notes: Up-front 1.0% EAI equity (~$1.7M) counts toward Rule 504 $10M rolling 12-month cap; confirm remaining 504 capacity before issuance. Rule 504 reference: https://www.sec.gov/resources-small-businesses/exempt-offerings/exemption-limited-offerings-not-exceeding-10-million-rule-504-regulation-d. Rule 504 is U.S.-only; EAI units used in the separate Reg S Japan round must be tracked under a distinct exemption.</t>
         </is>
       </c>
     </row>
@@ -7041,627 +6858,4 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:L40"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="2" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="77" t="inlineStr">
-        <is>
-          <t>SSLC: WITH vs WITHOUT EXOS CAPITAL — 5-Year Growth Comparison</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="28" customHeight="1">
-      <c r="A2" s="78" t="inlineStr">
-        <is>
-          <t>Prepared 2026-10-07  |  DRAFT — MANAGEMENT ASSUMPTIONS  |  INTERNAL — Exo/CEO only  |  Without-Exos trajectory derived from FY27 Q1 actual $713K run-rate; With-Exos uses v12 SSLC revenue drivers. All figures management assumptions unless labeled 'Actual'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="79" t="inlineStr">
-        <is>
-          <t>KEY FACT:  Reaching $5.1M in FY27 requires averaging $1.46M/quarter for Q2–Q4  ($5,100K − $713K Q1 actual ÷ 3 quarters = $1,462K/qtr)  —  approximately 2.05× the most recent quarter's $713K  —  starting immediately.  Without Exos capital to fund working capital and IM ramp, that doubling is not achievable on SSLC's $198K cash position.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="22" customHeight="1"/>
-    <row r="6" ht="22" customHeight="1"/>
-    <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="80" t="inlineStr">
-        <is>
-          <t>WITHOUT EXOS CAPITAL — Status-Quo Standalone Trajectory</t>
-        </is>
-      </c>
-      <c r="H8" s="81" t="inlineStr">
-        <is>
-          <t>NARRATIVE — The Capital Gap Story</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="82" t="inlineStr">
-        <is>
-          <t>Constraints: Cash $198K | ~1 month burn | WC bridge $300–700K needed | FY26 op loss −$416K | He-tank rework unresolved | No capex | No IM ramp capital → growth capped by self-funded working capital</t>
-        </is>
-      </c>
-      <c r="H9" s="83" t="inlineStr">
-        <is>
-          <t>Without Exos: Status-Quo Constraints</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="16" customHeight="1">
-      <c r="A10" s="84" t="inlineStr"/>
-      <c r="B10" s="84" t="inlineStr">
-        <is>
-          <t>FY27</t>
-        </is>
-      </c>
-      <c r="C10" s="84" t="inlineStr">
-        <is>
-          <t>FY28</t>
-        </is>
-      </c>
-      <c r="D10" s="84" t="inlineStr">
-        <is>
-          <t>FY29</t>
-        </is>
-      </c>
-      <c r="E10" s="84" t="inlineStr">
-        <is>
-          <t>FY30</t>
-        </is>
-      </c>
-      <c r="F10" s="84" t="inlineStr">
-        <is>
-          <t>FY31</t>
-        </is>
-      </c>
-      <c r="H10" s="85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Cash on hand (10/2/26):  $198K</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="16" customHeight="1">
-      <c r="A11" s="86" t="inlineStr">
-        <is>
-          <t>SSLC Revenue (standalone)</t>
-        </is>
-      </c>
-      <c r="B11" s="87" t="n">
-        <v>2850000</v>
-      </c>
-      <c r="C11" s="87" t="n">
-        <v>3136000</v>
-      </c>
-      <c r="D11" s="87" t="n">
-        <v>3449000</v>
-      </c>
-      <c r="E11" s="87" t="n">
-        <v>3794000</v>
-      </c>
-      <c r="F11" s="87" t="n">
-        <v>4174000</v>
-      </c>
-      <c r="H11" s="85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Working capital needed to maintain deliveries:  $300K–$700K</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="86" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  YoY Revenue Growth</t>
-        </is>
-      </c>
-      <c r="B12" s="88" t="n"/>
-      <c r="C12" s="89" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="D12" s="88" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="E12" s="89" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F12" s="88" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="H12" s="85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  FY26 operating loss:  −$416K</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="16" customHeight="1">
-      <c r="A13" s="86" t="inlineStr">
-        <is>
-          <t>SSLC Est. EBITDA (standalone)</t>
-        </is>
-      </c>
-      <c r="B13" s="90" t="n">
-        <v>-416000</v>
-      </c>
-      <c r="C13" s="91" t="n">
-        <v>-200000</v>
-      </c>
-      <c r="D13" s="92" t="n">
-        <v>50000</v>
-      </c>
-      <c r="E13" s="93" t="n">
-        <v>200000</v>
-      </c>
-      <c r="F13" s="92" t="n">
-        <v>350000</v>
-      </c>
-      <c r="H13" s="85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  He-tank rework unresolved — no resolution path without new owner</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="16" customHeight="1">
-      <c r="A14" s="86" t="inlineStr">
-        <is>
-          <t>Cumulative Revenue (FY27–year)</t>
-        </is>
-      </c>
-      <c r="B14" s="92" t="n">
-        <v>2850000</v>
-      </c>
-      <c r="C14" s="93" t="n">
-        <v>5986000</v>
-      </c>
-      <c r="D14" s="92" t="n">
-        <v>9435000</v>
-      </c>
-      <c r="E14" s="93" t="n">
-        <v>13229000</v>
-      </c>
-      <c r="F14" s="92" t="n">
-        <v>17403000</v>
-      </c>
-      <c r="H14" s="85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  No capex capacity → headcount/equipment frozen</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="16" customHeight="1">
-      <c r="A15" s="94" t="inlineStr">
-        <is>
-          <t>⚠  Stall Risk: SSLC needs $300–700K in working capital to maintain delivery commitments. On $198K cash, a working-capital crunch could interrupt deliveries in Q2–Q3 FY27, reducing FY27 below the $2.85M run-rate. The 10% CAGR assumes the crunch is survived.</t>
-        </is>
-      </c>
-      <c r="H15" s="85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Growth capped by self-funded working capital</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="16" customHeight="1">
-      <c r="H16" s="85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  FY27 achievable at run-rate:  ~$2.85M</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="95" t="inlineStr">
-        <is>
-          <t>WITH EXOS CAPITAL — v12 SSLC Revenue Trajectory (→ $54.7M by FY31)</t>
-        </is>
-      </c>
-      <c r="H17" s="85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  FY31 best-case (10% CAGR, no stall):  ~$4.2M</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="16" customHeight="1">
-      <c r="A18" s="96" t="inlineStr">
-        <is>
-          <t>Exos offer provides: Cash at close $2.51M | Debts paid at face | WC bridge ($300–700K) | Exos channel + IM ramp capex | v12 tank-unit/ASP ramp model. Figures: v12 Annual P&amp;L, recalculated 2026-10-07.</t>
-        </is>
-      </c>
-      <c r="H18" s="85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  5-yr CAGR (status quo):  ~10.0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="84" t="inlineStr"/>
-      <c r="B19" s="84" t="inlineStr">
-        <is>
-          <t>FY27</t>
-        </is>
-      </c>
-      <c r="C19" s="84" t="inlineStr">
-        <is>
-          <t>FY28</t>
-        </is>
-      </c>
-      <c r="D19" s="84" t="inlineStr">
-        <is>
-          <t>FY29</t>
-        </is>
-      </c>
-      <c r="E19" s="84" t="inlineStr">
-        <is>
-          <t>FY30</t>
-        </is>
-      </c>
-      <c r="F19" s="84" t="inlineStr">
-        <is>
-          <t>FY31</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="86" t="inlineStr">
-        <is>
-          <t>SSLC Revenue (with Exos, v12)</t>
-        </is>
-      </c>
-      <c r="B20" s="97" t="n">
-        <v>4120000</v>
-      </c>
-      <c r="C20" s="97" t="n">
-        <v>8680000</v>
-      </c>
-      <c r="D20" s="97" t="n">
-        <v>19220000</v>
-      </c>
-      <c r="E20" s="97" t="n">
-        <v>33880000</v>
-      </c>
-      <c r="F20" s="97" t="n">
-        <v>54690000</v>
-      </c>
-      <c r="H20" s="98" t="inlineStr">
-        <is>
-          <t>With Exos: What Capital Unlocks</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="16" customHeight="1">
-      <c r="A21" s="86" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  YoY Revenue Growth</t>
-        </is>
-      </c>
-      <c r="B21" s="88" t="n"/>
-      <c r="C21" s="89" t="n">
-        <v>1.108</v>
-      </c>
-      <c r="D21" s="88" t="n">
-        <v>1.214</v>
-      </c>
-      <c r="E21" s="89" t="n">
-        <v>0.763</v>
-      </c>
-      <c r="F21" s="88" t="n">
-        <v>0.614</v>
-      </c>
-      <c r="H21" s="85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Cash at close:  $2.51M</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="16" customHeight="1">
-      <c r="A22" s="86" t="inlineStr">
-        <is>
-          <t>SSLC Est. EBITDA (v12 drivers)</t>
-        </is>
-      </c>
-      <c r="B22" s="92" t="n">
-        <v>1278000</v>
-      </c>
-      <c r="C22" s="93" t="n">
-        <v>4130000</v>
-      </c>
-      <c r="D22" s="92" t="n">
-        <v>11821000</v>
-      </c>
-      <c r="E22" s="93" t="n">
-        <v>21953000</v>
-      </c>
-      <c r="F22" s="92" t="n">
-        <v>36379000</v>
-      </c>
-      <c r="H22" s="85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  SSLC debts paid at face (est. ~$500K TBV)</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="16" customHeight="1">
-      <c r="A23" s="86" t="inlineStr">
-        <is>
-          <t>Cumulative Revenue (FY27–year)</t>
-        </is>
-      </c>
-      <c r="B23" s="92" t="n">
-        <v>4120000</v>
-      </c>
-      <c r="C23" s="93" t="n">
-        <v>12800000</v>
-      </c>
-      <c r="D23" s="92" t="n">
-        <v>32020000</v>
-      </c>
-      <c r="E23" s="93" t="n">
-        <v>65900000</v>
-      </c>
-      <c r="F23" s="92" t="n">
-        <v>120590000</v>
-      </c>
-      <c r="H23" s="85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Prepaid-work delivery funded (cost $500K)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="16" customHeight="1">
-      <c r="H24" s="85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  WC bridge removes Q2–Q3 stall risk</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="16" customHeight="1">
-      <c r="A25" s="81" t="inlineStr">
-        <is>
-          <t>GROWTH-RATE (CAGR) AND CUMULATIVE-GAP COMPARISON — FY27 to FY31</t>
-        </is>
-      </c>
-      <c r="H25" s="85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Exos procurement channel:  immediate BLK3 tank POs</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="16" customHeight="1">
-      <c r="A26" s="84" t="inlineStr">
-        <is>
-          <t>Metric</t>
-        </is>
-      </c>
-      <c r="B26" s="99" t="inlineStr">
-        <is>
-          <t>Without Exos Capital</t>
-        </is>
-      </c>
-      <c r="C26" s="100" t="inlineStr">
-        <is>
-          <t>With Exos Capital</t>
-        </is>
-      </c>
-      <c r="D26" s="99" t="inlineStr">
-        <is>
-          <t>Without Exos Capital</t>
-        </is>
-      </c>
-      <c r="E26" s="100" t="inlineStr">
-        <is>
-          <t>With Exos Capital</t>
-        </is>
-      </c>
-      <c r="H26" s="85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Intuitive Machines ramp:  14–16 tanks firm FY27</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="16" customHeight="1">
-      <c r="A27" s="101" t="inlineStr">
-        <is>
-          <t>FY27 SSLC Revenue</t>
-        </is>
-      </c>
-      <c r="B27" s="102" t="n">
-        <v>2850000</v>
-      </c>
-      <c r="C27" s="103" t="n">
-        <v>4120000</v>
-      </c>
-      <c r="H27" s="85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Capex for production scale-up enabled</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="16" customHeight="1">
-      <c r="A28" s="101" t="inlineStr">
-        <is>
-          <t>FY31 SSLC Revenue</t>
-        </is>
-      </c>
-      <c r="B28" s="102" t="n">
-        <v>4174000</v>
-      </c>
-      <c r="C28" s="103" t="n">
-        <v>54690000</v>
-      </c>
-      <c r="H28" s="85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  FY27 target (IM firm + ramp):  $4.1M–$5.5M</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="16" customHeight="1">
-      <c r="A29" s="101" t="inlineStr">
-        <is>
-          <t>FY27–FY31 CAGR (SSLC Revenue)</t>
-        </is>
-      </c>
-      <c r="B29" s="104" t="n">
-        <v>0.1000866545812265</v>
-      </c>
-      <c r="C29" s="105" t="n">
-        <v>0.9087659399397092</v>
-      </c>
-      <c r="H29" s="85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  FY31 (v12 trajectory):  $54.7M</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="16" customHeight="1">
-      <c r="A30" s="101" t="inlineStr">
-        <is>
-          <t>Cumulative 5-yr SSLC Revenue</t>
-        </is>
-      </c>
-      <c r="B30" s="102" t="n">
-        <v>17403000</v>
-      </c>
-      <c r="C30" s="103" t="n">
-        <v>120590000</v>
-      </c>
-      <c r="H30" s="85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  5-yr CAGR (with Exos, v12):  ~90.9%</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="101" t="inlineStr">
-        <is>
-          <t>Y5 Annual Revenue Gap (With − W/O)</t>
-        </is>
-      </c>
-      <c r="B31" s="106" t="n"/>
-      <c r="C31" s="103" t="n">
-        <v>50516000</v>
-      </c>
-    </row>
-    <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="101" t="inlineStr">
-        <is>
-          <t>Cumulative 5-yr Gap (With − W/O)</t>
-        </is>
-      </c>
-      <c r="B32" s="106" t="n"/>
-      <c r="C32" s="103" t="n">
-        <v>103187000</v>
-      </c>
-      <c r="H32" s="107" t="inlineStr">
-        <is>
-          <t>The Doubling Requirement</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="16" customHeight="1">
-      <c r="H33" s="85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  FY27 $5.1M target − Q1 $713K actual = $4,387K remaining</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="16" customHeight="1">
-      <c r="H34" s="85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Over 3 quarters (Q2–Q4) = $1,462K/qtr required</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="16" customHeight="1">
-      <c r="H35" s="85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  vs. Q1 $713K actual = 2.05× immediate ramp</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="16" customHeight="1">
-      <c r="H36" s="85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Only funded if Exos capital bridges the working-capital gap</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="16" customHeight="1">
-      <c r="H37" s="85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Without capital → Q2–Q4 stays ≈ $713K/qtr = $2.85M FY27</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="28" customHeight="1">
-      <c r="A40" s="108" t="inlineStr">
-        <is>
-          <t>Management Assumptions — all projections forward of FY27 Q1 actual ($713K) are management estimates, not independently audited. Without-Exos CAGR assumes no working-capital stall; stall scenarios produce lower figures. With-Exos CAGR uses v12 SSLC tank-unit/ASP/COGS drivers, not independently audited. DRAFT, 2026-10-07.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="38">
-    <mergeCell ref="H30:L30"/>
-    <mergeCell ref="H26:L26"/>
-    <mergeCell ref="H29:L29"/>
-    <mergeCell ref="H35:L35"/>
-    <mergeCell ref="H20:L20"/>
-    <mergeCell ref="H10:L10"/>
-    <mergeCell ref="A18:F18"/>
-    <mergeCell ref="H34:L34"/>
-    <mergeCell ref="H9:L9"/>
-    <mergeCell ref="A2:L2"/>
-    <mergeCell ref="H25:L25"/>
-    <mergeCell ref="H21:L21"/>
-    <mergeCell ref="A8:F8"/>
-    <mergeCell ref="H36:L36"/>
-    <mergeCell ref="A17:F17"/>
-    <mergeCell ref="H17:L17"/>
-    <mergeCell ref="H11:L11"/>
-    <mergeCell ref="H16:L16"/>
-    <mergeCell ref="A9:F9"/>
-    <mergeCell ref="H32:L32"/>
-    <mergeCell ref="H28:L28"/>
-    <mergeCell ref="A4:L6"/>
-    <mergeCell ref="A40:L40"/>
-    <mergeCell ref="H13:L13"/>
-    <mergeCell ref="H37:L37"/>
-    <mergeCell ref="H22:L22"/>
-    <mergeCell ref="A15:F15"/>
-    <mergeCell ref="H27:L27"/>
-    <mergeCell ref="H12:L12"/>
-    <mergeCell ref="H15:L15"/>
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="H24:L24"/>
-    <mergeCell ref="H18:L18"/>
-    <mergeCell ref="H33:L33"/>
-    <mergeCell ref="H14:L14"/>
-    <mergeCell ref="H23:L23"/>
-    <mergeCell ref="H8:L8"/>
-    <mergeCell ref="A25:F25"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
SSLC Option B: lockup + projected post-RTO value; offer summary ≤2 pages — task #2414
- EAI Lockup & Liquidity: Rule 504 restricted/legended; lockup=Exos principals;
  Rule 144 6-mo (reporting) / 1-yr (non-reporting); 6-mo path only after RTO;
  RTO preferred→common after shareholder vote + resale reg (S-1/S-3)
  [Board Brief 2026-09-04:16; Board Questions 2026-09-08:36,44]
- Lockup timeline table (6 rows) in offer summary; full detail in XLSX Sheet 9
- Projected post-RTO value (1.0% EAI alone, ~30% dil):
  Low $200M→$1.40M / Base $250M→$1.75M / High $300M→$2.10M post-dil
  vs 409A issuance ~$1.70M; Rule 10b-5 cautionary statement
- Removed Section 2 (With vs Without) from offer summary → model reference only
- Offer summary trimmed to 2 pages (pdfinfo verified)
</commit_message>
<xml_diff>
--- a/drafts/EXOS_SSLC_OptionB_Acquisition_Model_2026-10-07.xlsx
+++ b/drafts/EXOS_SSLC_OptionB_Acquisition_Model_2026-10-07.xlsx
@@ -14,6 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Funding" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Total Compensation" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reconciliation" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="EAI Lockup &amp; Liquidity" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -29,7 +30,7 @@
     <numFmt numFmtId="167" formatCode="0.0x"/>
     <numFmt numFmtId="168" formatCode="0.00x"/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="25">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -130,8 +131,23 @@
       <color rgb="00C00000"/>
       <sz val="8"/>
     </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00C00000"/>
+      <sz val="8.5"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F3864"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00444444"/>
+      <sz val="8.5"/>
+    </font>
   </fonts>
-  <fills count="15">
+  <fills count="17">
     <fill>
       <patternFill/>
     </fill>
@@ -203,6 +219,16 @@
         <fgColor rgb="00E26A21"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00375623"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D1FAE5"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -216,7 +242,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="94">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -330,6 +356,49 @@
     <xf numFmtId="0" fontId="5" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -6858,4 +6927,615 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G41"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="77" t="inlineStr">
+        <is>
+          <t>EAI UNIT LOCKUP &amp; LIQUIDITY — DETAIL</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="78" t="inlineStr">
+        <is>
+          <t>INTERNAL — NEGOTIATING TERMS — Not a final or binding offer. 2026-10-09 update (John Quinn). Sources: Ainigma_RTO_Board_Brief_2026-09-04.md:16; Ainigma_RTO_Anticipated_Board_Questions_2026-09-08.md:36,44.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="79" t="inlineStr">
+        <is>
+          <t>A.  Legal Status of EAI Units at Issuance</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="80" t="inlineStr">
+        <is>
+          <t>Instrument type</t>
+        </is>
+      </c>
+      <c r="B5" s="81" t="inlineStr">
+        <is>
+          <t>Exos Aerospace Investments LLC (EAI) units.</t>
+        </is>
+      </c>
+      <c r="C5" s="82" t="inlineStr"/>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="80" t="inlineStr">
+        <is>
+          <t>Securities law status</t>
+        </is>
+      </c>
+      <c r="B6" s="81" t="inlineStr">
+        <is>
+          <t>Restricted securities issued under Rule 504, Regulation D. Bear a restrictive legend. Not freely tradeable at issuance.</t>
+        </is>
+      </c>
+      <c r="C6" s="82" t="inlineStr">
+        <is>
+          <t>Rule 504: https://www.sec.gov/resources-small-businesses/exempt-offerings/exemption-limited-offerings-not-exceeding-10-million-rule-504-regulation-d</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="80" t="inlineStr">
+        <is>
+          <t>Offering type</t>
+        </is>
+      </c>
+      <c r="B7" s="81" t="inlineStr">
+        <is>
+          <t>Rule 504 / Regulation D (U.S. domestic offering). NOT covered by the Reg S exemption used for the Japan round.</t>
+        </is>
+      </c>
+      <c r="C7" s="82" t="inlineStr">
+        <is>
+          <t>The two offerings must be tracked under distinct exemptions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="80" t="inlineStr">
+        <is>
+          <t>409A value at issuance</t>
+        </is>
+      </c>
+      <c r="B8" s="81" t="inlineStr">
+        <is>
+          <t>1.0% × $169.7M (Eqvista 409A, valuation date 3/31/2026) = $1,697,000 (~$1.7M)</t>
+        </is>
+      </c>
+      <c r="C8" s="82" t="inlineStr">
+        <is>
+          <t>Issued at financing close, committed at SSLC board acceptance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="80" t="inlineStr">
+        <is>
+          <t>Lockup — mirrors principals</t>
+        </is>
+      </c>
+      <c r="B9" s="81" t="inlineStr">
+        <is>
+          <t>Same lockup terms as Exos Aerospace principals under the RTO transaction documents. Specific lock periods in the RTO definitive agreement govern.</t>
+        </is>
+      </c>
+      <c r="C9" s="82" t="inlineStr">
+        <is>
+          <t>Ainigma mandate per Board Brief 2026-09-04.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="79" t="inlineStr">
+        <is>
+          <t>B.  Rule 144 Resale Requirements  (17 CFR 230.144(d))</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="42" customHeight="1">
+      <c r="A12" s="80" t="inlineStr">
+        <is>
+          <t>Rule 144 reference</t>
+        </is>
+      </c>
+      <c r="B12" s="81" t="inlineStr">
+        <is>
+          <t>17 CFR 230.144(d) — Holding period requirement. URL: https://www.ecfr.gov/current/title-17/chapter-II/part-230/section-230.144</t>
+        </is>
+      </c>
+      <c r="C12" s="82" t="inlineStr">
+        <is>
+          <t>Verified 2026-10-09.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="42" customHeight="1">
+      <c r="A13" s="80" t="inlineStr">
+        <is>
+          <t>Holding period — reporting issuer</t>
+        </is>
+      </c>
+      <c r="B13" s="81" t="inlineStr">
+        <is>
+          <t>6 months from issuance date. Applies ONLY after the issuer (or successor) is an SEC-reporting company with current public information available.</t>
+        </is>
+      </c>
+      <c r="C13" s="82" t="inlineStr">
+        <is>
+          <t>17 CFR 230.144(d)(1)(i).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="42" customHeight="1">
+      <c r="A14" s="80" t="inlineStr">
+        <is>
+          <t>Holding period — non-reporting issuer</t>
+        </is>
+      </c>
+      <c r="B14" s="81" t="inlineStr">
+        <is>
+          <t>1 year from issuance date. Exos Aerospace Systems &amp; Technologies, Inc. is NOT currently an SEC reporting company. Until the RTO makes the successor entity reporting, the 1-year path applies.</t>
+        </is>
+      </c>
+      <c r="C14" s="82" t="inlineStr">
+        <is>
+          <t>17 CFR 230.144(d)(1)(ii).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="42" customHeight="1">
+      <c r="A15" s="80" t="inlineStr">
+        <is>
+          <t>6-month clock start</t>
+        </is>
+      </c>
+      <c r="B15" s="81" t="inlineStr">
+        <is>
+          <t>The 6-month clock begins only AFTER the RTO close makes the issuer/successor a reporting company. With a targeted RTO close ~6 months after financing close, the earliest Rule 144 window under the 6-month path is ~12 months post-issuance (close + 6 months). Actual timing depends on RTO completion and the conversion/resale registration schedule.</t>
+        </is>
+      </c>
+      <c r="C15" s="82" t="inlineStr">
+        <is>
+          <t>Targeted, not assured.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="79" t="inlineStr">
+        <is>
+          <t>C.  RTO Structure — Preferred-at-Close / Conversion Path</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="48" customHeight="1">
+      <c r="A18" s="80" t="inlineStr">
+        <is>
+          <t>RTO mechanics</t>
+        </is>
+      </c>
+      <c r="B18" s="81" t="inlineStr">
+        <is>
+          <t>Merger closes BEFORE the public stockholder vote using non-voting, non-convertible preferred stock (avoids NASDAQ Rule 5635 early-stage trigger). A proxy is filed within ~30 days of RTO close.</t>
+        </is>
+      </c>
+      <c r="C18" s="82" t="inlineStr">
+        <is>
+          <t>Source: Ainigma_RTO_Board_Brief_2026-09-04.md:16.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="48" customHeight="1">
+      <c r="A19" s="80" t="inlineStr">
+        <is>
+          <t>Preferred → common</t>
+        </is>
+      </c>
+      <c r="B19" s="81" t="inlineStr">
+        <is>
+          <t>Preferred converts to common and becomes liquid ONLY after: (i) post-close public-shareholder vote (that founders do not control at the moment of close), AND (ii) effective resale registration (S-1/S-3).</t>
+        </is>
+      </c>
+      <c r="C19" s="82" t="inlineStr">
+        <is>
+          <t>Sources: Board Brief 2026-09-04.md:16; Board Questions 2026-09-08.md:36,44.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="48" customHeight="1">
+      <c r="A20" s="80" t="inlineStr">
+        <is>
+          <t>EAI units follow same path</t>
+        </is>
+      </c>
+      <c r="B20" s="81" t="inlineStr">
+        <is>
+          <t>The EAI units' liquidity follows the identical path: committed at board acceptance → issued at financing close → held as restricted/non-trading until RTO close → preferred conversion vote → resale registration effective → Rule 144 / free-trading eligibility.</t>
+        </is>
+      </c>
+      <c r="C20" s="82" t="inlineStr">
+        <is>
+          <t>See timeline table below.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="48" customHeight="1">
+      <c r="A21" s="80" t="inlineStr">
+        <is>
+          <t>Risk if vote fails / reg stalls</t>
+        </is>
+      </c>
+      <c r="B21" s="81" t="inlineStr">
+        <is>
+          <t>If the conversion vote fails or the resale registration stalls, holders of the EAI units (like founders) hold restricted, non-voting paper with no near-term liquidity. This is a known RTO structure, not disqualifying, but must be understood.</t>
+        </is>
+      </c>
+      <c r="C21" s="82" t="inlineStr">
+        <is>
+          <t>Source: Board Brief:44; Board Questions:62.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="79" t="inlineStr">
+        <is>
+          <t>D.  Liquidity Timeline  (Targeted — Not Assured)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="83" t="inlineStr">
+        <is>
+          <t>Milestone</t>
+        </is>
+      </c>
+      <c r="B24" s="83" t="inlineStr">
+        <is>
+          <t>Target / Detail</t>
+        </is>
+      </c>
+      <c r="C24" s="83" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="36" customHeight="1">
+      <c r="A25" s="80" t="inlineStr">
+        <is>
+          <t>Board acceptance</t>
+        </is>
+      </c>
+      <c r="B25" s="81" t="inlineStr">
+        <is>
+          <t>D+0. EAI units committed; not yet issued. SSLC board confirms Option B.</t>
+        </is>
+      </c>
+      <c r="C25" s="84" t="inlineStr">
+        <is>
+          <t>Targeted</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="36" customHeight="1">
+      <c r="A26" s="80" t="inlineStr">
+        <is>
+          <t>Financing close — units issued</t>
+        </is>
+      </c>
+      <c r="B26" s="81" t="inlineStr">
+        <is>
+          <t>Targeted Q1 FY27 (~2026-Q4/Q1 2027). EAI units formally issued. Rule 144 holding period (1-year, non-reporting) clock starts.</t>
+        </is>
+      </c>
+      <c r="C26" s="84" t="inlineStr">
+        <is>
+          <t>Targeted, not assured</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="36" customHeight="1">
+      <c r="A27" s="80" t="inlineStr">
+        <is>
+          <t>Targeted RTO close</t>
+        </is>
+      </c>
+      <c r="B27" s="81" t="inlineStr">
+        <is>
+          <t>~6 months post-financing close. Exos/NewCo merger closes using non-voting preferred. NOT the liquidity event — preferred not yet tradeable.</t>
+        </is>
+      </c>
+      <c r="C27" s="84" t="inlineStr">
+        <is>
+          <t>Targeted, not assured</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="36" customHeight="1">
+      <c r="A28" s="80" t="inlineStr">
+        <is>
+          <t>Proxy filed / shareholder vote</t>
+        </is>
+      </c>
+      <c r="B28" s="81" t="inlineStr">
+        <is>
+          <t>~30 days post-RTO close. Public stockholder vote on preferred → common conversion.</t>
+        </is>
+      </c>
+      <c r="C28" s="84" t="inlineStr">
+        <is>
+          <t>Targeted, not assured</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="36" customHeight="1">
+      <c r="A29" s="80" t="inlineStr">
+        <is>
+          <t>Resale registration effective (S-1/S-3)</t>
+        </is>
+      </c>
+      <c r="B29" s="81" t="inlineStr">
+        <is>
+          <t>~30–90 days post-RTO close (concurrent with or following vote). Registration must go effective before preferred converts to tradeable common.</t>
+        </is>
+      </c>
+      <c r="C29" s="84" t="inlineStr">
+        <is>
+          <t>Targeted, not assured</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="36" customHeight="1">
+      <c r="A30" s="80" t="inlineStr">
+        <is>
+          <t>Rule 144 eligibility — 6-month path</t>
+        </is>
+      </c>
+      <c r="B30" s="81" t="inlineStr">
+        <is>
+          <t>AFTER reporting status is established AND ≥6 months from issuance date. Earliest: ~12 months post-issuance (close + RTO ~6 mo + holding). Requires current public information available.</t>
+        </is>
+      </c>
+      <c r="C30" s="84" t="inlineStr">
+        <is>
+          <t>Targeted, not assured</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="36" customHeight="1">
+      <c r="A31" s="80" t="inlineStr">
+        <is>
+          <t>Rule 144 eligibility — 1-year path</t>
+        </is>
+      </c>
+      <c r="B31" s="81" t="inlineStr">
+        <is>
+          <t>1 year from issuance date (non-reporting issuer path). If RTO does not close by 1-year mark, this is the available resale window.</t>
+        </is>
+      </c>
+      <c r="C31" s="84" t="inlineStr">
+        <is>
+          <t>Fallback if 6-mo path unavailable</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="36" customHeight="1">
+      <c r="A32" s="85" t="inlineStr">
+        <is>
+          <t>ALL DATES</t>
+        </is>
+      </c>
+      <c r="B32" s="86" t="inlineStr">
+        <is>
+          <t>TARGETED, NOT ASSURED. The RTO may not close.</t>
+        </is>
+      </c>
+      <c r="C32" s="87" t="inlineStr">
+        <is>
+          <t>Risk</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="18" customHeight="1">
+      <c r="A34" s="88" t="inlineStr">
+        <is>
+          <t>E.  Projected Post-RTO Value  —  PROJECTION, NOT A PROMISE</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="60" customHeight="1">
+      <c r="A35" s="89" t="inlineStr">
+        <is>
+          <t>CAUTIONARY STATEMENT: Forward-looking projection based on management assumptions (RTO completion, listing valuation, ~30% dilution). Not a guarantee or promise of value; actual results may differ materially. The RTO may not close. SEC Rule 10b-5 (17 CFR 240.10b-5; https://www.ecfr.gov/current/title-17/chapter-II/part-240/section-240.10b-5) antifraud rules apply to projections. Projections must have a reasonable basis; do not rely on this section as an offer to sell or inducement beyond the framing above.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="28" customHeight="1">
+      <c r="A36" s="69" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="B36" s="69" t="inlineStr">
+        <is>
+          <t>RTO MEV</t>
+        </is>
+      </c>
+      <c r="C36" s="69" t="inlineStr">
+        <is>
+          <t>1.0% pre-dilution</t>
+        </is>
+      </c>
+      <c r="D36" s="69" t="inlineStr">
+        <is>
+          <t>~30% dilution</t>
+        </is>
+      </c>
+      <c r="E36" s="69" t="inlineStr">
+        <is>
+          <t>1.0% post-dilution (up-front only)</t>
+        </is>
+      </c>
+      <c r="F36" s="69" t="inlineStr">
+        <is>
+          <t>409A at issuance</t>
+        </is>
+      </c>
+      <c r="G36" s="69" t="inlineStr">
+        <is>
+          <t>Additional: earn-out at listing</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="22" customHeight="1">
+      <c r="A37" s="90" t="inlineStr">
+        <is>
+          <t>Low (floor)</t>
+        </is>
+      </c>
+      <c r="B37" s="90" t="inlineStr">
+        <is>
+          <t>$200M</t>
+        </is>
+      </c>
+      <c r="C37" s="90" t="inlineStr">
+        <is>
+          <t>$2.00M</t>
+        </is>
+      </c>
+      <c r="D37" s="90" t="inlineStr">
+        <is>
+          <t>−$0.60M</t>
+        </is>
+      </c>
+      <c r="E37" s="90" t="inlineStr">
+        <is>
+          <t>$1.40M</t>
+        </is>
+      </c>
+      <c r="F37" s="90" t="inlineStr">
+        <is>
+          <t>~$1.70M (409A)</t>
+        </is>
+      </c>
+      <c r="G37" s="90" t="inlineStr">
+        <is>
+          <t>$0  (0.0% earn-out)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="22" customHeight="1">
+      <c r="A38" s="91" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="B38" s="91" t="inlineStr">
+        <is>
+          <t>$250M</t>
+        </is>
+      </c>
+      <c r="C38" s="91" t="inlineStr">
+        <is>
+          <t>$2.50M</t>
+        </is>
+      </c>
+      <c r="D38" s="91" t="inlineStr">
+        <is>
+          <t>−$0.75M</t>
+        </is>
+      </c>
+      <c r="E38" s="91" t="inlineStr">
+        <is>
+          <t>$1.75M</t>
+        </is>
+      </c>
+      <c r="F38" s="91" t="inlineStr">
+        <is>
+          <t>~$1.70M (409A)</t>
+        </is>
+      </c>
+      <c r="G38" s="91" t="inlineStr">
+        <is>
+          <t>+$424K  (0.25%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="22" customHeight="1">
+      <c r="A39" s="92" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B39" s="92" t="inlineStr">
+        <is>
+          <t>$300M</t>
+        </is>
+      </c>
+      <c r="C39" s="92" t="inlineStr">
+        <is>
+          <t>$3.00M</t>
+        </is>
+      </c>
+      <c r="D39" s="92" t="inlineStr">
+        <is>
+          <t>−$0.90M</t>
+        </is>
+      </c>
+      <c r="E39" s="92" t="inlineStr">
+        <is>
+          <t>$2.10M</t>
+        </is>
+      </c>
+      <c r="F39" s="92" t="inlineStr">
+        <is>
+          <t>~$1.70M (409A)</t>
+        </is>
+      </c>
+      <c r="G39" s="92" t="inlineStr">
+        <is>
+          <t>+$848K  (0.50%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="60" customHeight="1">
+      <c r="A41" s="93" t="inlineStr">
+        <is>
+          <t>Notes: MEV per Ainigma mandate ($250M min, $300M stretch). Dilution ~30% (Series A D1–D4 ~13% + RTO ~12% + option pool ~5%) — management assumption. Post-dil = (1.0%) × (1 − 0.30) × MEV. Earn-out column is ADDITIONAL at listing price; not additive to 409A value. Full Y5 hold analysis (16× EV/EBITDA): model 'Total Compensation' sheet. Rule 10b-5 reference: https://www.ecfr.gov/current/title-17/chapter-II/part-240/section-240.10b-5. Rule 144 reference: https://www.ecfr.gov/current/title-17/chapter-II/part-230/section-230.144. Rule 504 reference: https://www.sec.gov/resources-small-businesses/exempt-offerings/exemption-limited-offerings-not-exceeding-10-million-rule-504-regulation-d.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="A41:C41"/>
+    <mergeCell ref="A11:C11"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="A34:C34"/>
+    <mergeCell ref="A35:C35"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A2:C2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
SSLC offer: float/tradeable-at-going-public lockup, orange IF-HELD rows, DIV/0 fix
</commit_message>
<xml_diff>
--- a/drafts/EXOS_SSLC_OptionB_Acquisition_Model_2026-10-07.xlsx
+++ b/drafts/EXOS_SSLC_OptionB_Acquisition_Model_2026-10-07.xlsx
@@ -31,7 +31,7 @@
     <numFmt numFmtId="167" formatCode="0.0x"/>
     <numFmt numFmtId="168" formatCode="0.00x"/>
   </numFmts>
-  <fonts count="34">
+  <fonts count="40">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -188,8 +188,36 @@
     <font>
       <sz val="9.5"/>
     </font>
+    <font/>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="001F3A68"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00606060"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="20">
+  <fills count="22">
     <fill>
       <patternFill/>
     </fill>
@@ -286,8 +314,18 @@
         <fgColor rgb="00BF8F00"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3A68"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FEF3C7"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="3">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -323,11 +361,124 @@
         <color rgb="00CCCCCC"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="00BF8F00"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00BF8F00"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="00BF8F00"/>
+      </right>
+      <top style="medium">
+        <color rgb="00BF8F00"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="00BF8F00"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00BF8F00"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="00BF8F00"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="00BF8F00"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="00BF8F00"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="00BF8F00"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="127">
+  <cellXfs count="144">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -581,6 +732,37 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -6476,7 +6658,7 @@
         <v/>
       </c>
       <c r="F36" s="71">
-        <f>D36/E36</f>
+        <f>IFERROR(D36/E36,"n/a")</f>
         <v/>
       </c>
       <c r="H36" s="72" t="inlineStr">
@@ -6572,7 +6754,7 @@
         <v/>
       </c>
       <c r="F39" s="71">
-        <f>D39/E39</f>
+        <f>IFERROR(D39/E39,"n/a")</f>
         <v/>
       </c>
       <c r="H39" s="72" t="inlineStr">
@@ -7116,604 +7298,649 @@
   <dimension ref="A1:G41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="72" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
     <col width="32" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="78" t="inlineStr">
+      <c r="A1" s="127" t="inlineStr">
         <is>
           <t>EAI UNIT LOCKUP &amp; LIQUIDITY — DETAIL</t>
         </is>
       </c>
+      <c r="B1" s="128" t="n"/>
+      <c r="C1" s="128" t="n"/>
+      <c r="D1" s="128" t="n"/>
+      <c r="E1" s="128" t="n"/>
+      <c r="F1" s="128" t="n"/>
+      <c r="G1" s="128" t="n"/>
     </row>
     <row r="2" ht="28" customHeight="1">
-      <c r="A2" s="79" t="inlineStr">
-        <is>
-          <t>INTERNAL — NEGOTIATING TERMS — Not a final or binding offer. 2026-10-09 update (John Quinn). Sources: Ainigma_RTO_Board_Brief_2026-09-04.md:16; Ainigma_RTO_Anticipated_Board_Questions_2026-09-08.md:36,44.</t>
-        </is>
-      </c>
+      <c r="A2" s="129" t="inlineStr">
+        <is>
+          <t>INTERNAL — NEGOTIATING TERMS — Not a final or binding offer. 2026-10-09 update (John Quinn).</t>
+        </is>
+      </c>
+      <c r="B2" s="128" t="n"/>
+      <c r="C2" s="128" t="n"/>
+      <c r="D2" s="128" t="n"/>
+      <c r="E2" s="128" t="n"/>
+      <c r="F2" s="128" t="n"/>
+      <c r="G2" s="128" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="128" t="n"/>
+      <c r="B3" s="128" t="n"/>
+      <c r="C3" s="128" t="n"/>
+      <c r="D3" s="128" t="n"/>
+      <c r="E3" s="128" t="n"/>
+      <c r="F3" s="128" t="n"/>
+      <c r="G3" s="128" t="n"/>
     </row>
     <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="80" t="inlineStr">
+      <c r="A4" s="127" t="inlineStr">
         <is>
           <t>A.  Legal Status of EAI Units at Issuance</t>
         </is>
       </c>
+      <c r="B4" s="128" t="n"/>
+      <c r="C4" s="128" t="n"/>
+      <c r="D4" s="128" t="n"/>
+      <c r="E4" s="128" t="n"/>
+      <c r="F4" s="128" t="n"/>
+      <c r="G4" s="128" t="n"/>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="81" t="inlineStr">
+      <c r="A5" s="130" t="inlineStr">
         <is>
           <t>Instrument type</t>
         </is>
       </c>
-      <c r="B5" s="82" t="inlineStr">
+      <c r="B5" s="131" t="inlineStr">
         <is>
           <t>Exos Aerospace Investments LLC (EAI) units.</t>
         </is>
       </c>
-      <c r="C5" s="83" t="inlineStr"/>
+      <c r="C5" s="128" t="n"/>
+      <c r="D5" s="128" t="n"/>
+      <c r="E5" s="128" t="n"/>
+      <c r="F5" s="128" t="n"/>
+      <c r="G5" s="128" t="n"/>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="81" t="inlineStr">
+      <c r="A6" s="130" t="inlineStr">
         <is>
           <t>Securities law status</t>
         </is>
       </c>
-      <c r="B6" s="82" t="inlineStr">
+      <c r="B6" s="131" t="inlineStr">
         <is>
           <t>Restricted securities issued under Rule 504, Regulation D. Bear a restrictive legend. Not freely tradeable at issuance.</t>
         </is>
       </c>
-      <c r="C6" s="83" t="inlineStr">
+      <c r="C6" s="129" t="inlineStr">
         <is>
           <t>Rule 504: https://www.sec.gov/resources-small-businesses/exempt-offerings/exemption-limited-offerings-not-exceeding-10-million-rule-504-regulation-d</t>
         </is>
       </c>
+      <c r="D6" s="128" t="n"/>
+      <c r="E6" s="128" t="n"/>
+      <c r="F6" s="128" t="n"/>
+      <c r="G6" s="128" t="n"/>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="81" t="inlineStr">
+      <c r="A7" s="130" t="inlineStr">
         <is>
           <t>Offering type</t>
         </is>
       </c>
-      <c r="B7" s="82" t="inlineStr">
+      <c r="B7" s="131" t="inlineStr">
         <is>
           <t>Rule 504 / Regulation D (U.S. domestic offering). NOT covered by the Reg S exemption used for the Japan round.</t>
         </is>
       </c>
-      <c r="C7" s="83" t="inlineStr">
+      <c r="C7" s="129" t="inlineStr">
         <is>
           <t>The two offerings must be tracked under distinct exemptions.</t>
         </is>
       </c>
+      <c r="D7" s="128" t="n"/>
+      <c r="E7" s="128" t="n"/>
+      <c r="F7" s="128" t="n"/>
+      <c r="G7" s="128" t="n"/>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="81" t="inlineStr">
+      <c r="A8" s="130" t="inlineStr">
         <is>
           <t>409A value at issuance</t>
         </is>
       </c>
-      <c r="B8" s="82" t="inlineStr">
+      <c r="B8" s="131" t="inlineStr">
         <is>
           <t>$1,000,000 fixed (= ~0.589% × $169.7M Eqvista 409A, valuation date 3/31/2026). ~0.59% of FD shares at close.</t>
         </is>
       </c>
-      <c r="C8" s="83" t="inlineStr">
+      <c r="C8" s="129" t="inlineStr">
         <is>
           <t>Issued at financing close, committed at SSLC board acceptance.</t>
         </is>
       </c>
+      <c r="D8" s="128" t="n"/>
+      <c r="E8" s="128" t="n"/>
+      <c r="F8" s="128" t="n"/>
+      <c r="G8" s="128" t="n"/>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="81" t="inlineStr">
+      <c r="A9" s="130" t="inlineStr">
         <is>
           <t>Lockup — mirrors principals</t>
         </is>
       </c>
-      <c r="B9" s="82" t="inlineStr">
+      <c r="B9" s="131" t="inlineStr">
         <is>
           <t>Same lockup terms as Exos Aerospace principals under the RTO transaction documents. Specific lock periods in the RTO definitive agreement govern.</t>
         </is>
       </c>
-      <c r="C9" s="83" t="inlineStr">
+      <c r="C9" s="129" t="inlineStr">
         <is>
           <t>Ainigma mandate per Board Brief 2026-09-04.</t>
         </is>
       </c>
+      <c r="D9" s="128" t="n"/>
+      <c r="E9" s="128" t="n"/>
+      <c r="F9" s="128" t="n"/>
+      <c r="G9" s="128" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="130" t="inlineStr">
+        <is>
+          <t>Float at RTO listing</t>
+        </is>
+      </c>
+      <c r="B10" s="131" t="inlineStr">
+        <is>
+          <t>The EAI units are structured to provide part of the public float for the Exos RTO and become tradeable at going public (the RTO listing), subject to the same lockup as Exos principals. Resale at listing assumes the units are included in the RTO's resale registration.</t>
+        </is>
+      </c>
+      <c r="C10" s="128" t="n"/>
+      <c r="D10" s="128" t="n"/>
+      <c r="E10" s="128" t="n"/>
+      <c r="F10" s="128" t="n"/>
+      <c r="G10" s="128" t="n"/>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="80" t="inlineStr">
-        <is>
-          <t>B.  Rule 144 Resale Requirements  (17 CFR 230.144(d))</t>
-        </is>
-      </c>
+      <c r="A11" s="128" t="n"/>
+      <c r="B11" s="128" t="n"/>
+      <c r="C11" s="128" t="n"/>
+      <c r="D11" s="128" t="n"/>
+      <c r="E11" s="128" t="n"/>
+      <c r="F11" s="128" t="n"/>
+      <c r="G11" s="128" t="n"/>
     </row>
     <row r="12" ht="42" customHeight="1">
-      <c r="A12" s="81" t="inlineStr">
-        <is>
-          <t>Rule 144 reference</t>
-        </is>
-      </c>
-      <c r="B12" s="82" t="inlineStr">
-        <is>
-          <t>17 CFR 230.144(d) — Holding period requirement. URL: https://www.ecfr.gov/current/title-17/chapter-II/part-230/section-230.144</t>
-        </is>
-      </c>
-      <c r="C12" s="83" t="inlineStr">
-        <is>
-          <t>Verified 2026-10-09.</t>
-        </is>
-      </c>
+      <c r="A12" s="127" t="inlineStr">
+        <is>
+          <t>B.  Liquidity Timeline  (Targeted — Not Assured)</t>
+        </is>
+      </c>
+      <c r="B12" s="128" t="n"/>
+      <c r="C12" s="128" t="n"/>
+      <c r="D12" s="128" t="n"/>
+      <c r="E12" s="128" t="n"/>
+      <c r="F12" s="128" t="n"/>
+      <c r="G12" s="128" t="n"/>
     </row>
     <row r="13" ht="42" customHeight="1">
-      <c r="A13" s="81" t="inlineStr">
-        <is>
-          <t>Holding period — reporting issuer</t>
-        </is>
-      </c>
-      <c r="B13" s="82" t="inlineStr">
-        <is>
-          <t>6 months from issuance date. Applies ONLY after the issuer (or successor) is an SEC-reporting company with current public information available.</t>
-        </is>
-      </c>
-      <c r="C13" s="83" t="inlineStr">
-        <is>
-          <t>17 CFR 230.144(d)(1)(i).</t>
-        </is>
-      </c>
+      <c r="A13" s="132" t="inlineStr">
+        <is>
+          <t>Milestone</t>
+        </is>
+      </c>
+      <c r="B13" s="132" t="inlineStr">
+        <is>
+          <t>Target / Detail</t>
+        </is>
+      </c>
+      <c r="C13" s="132" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="D13" s="128" t="n"/>
+      <c r="E13" s="128" t="n"/>
+      <c r="F13" s="128" t="n"/>
+      <c r="G13" s="128" t="n"/>
     </row>
     <row r="14" ht="42" customHeight="1">
-      <c r="A14" s="81" t="inlineStr">
-        <is>
-          <t>Holding period — non-reporting issuer</t>
-        </is>
-      </c>
-      <c r="B14" s="82" t="inlineStr">
-        <is>
-          <t>1 year from issuance date. Exos Aerospace Systems &amp; Technologies, Inc. is NOT currently an SEC reporting company. Until the RTO makes the successor entity reporting, the 1-year path applies.</t>
-        </is>
-      </c>
-      <c r="C14" s="83" t="inlineStr">
-        <is>
-          <t>17 CFR 230.144(d)(1)(ii).</t>
-        </is>
-      </c>
+      <c r="A14" s="131" t="inlineStr">
+        <is>
+          <t>Board acceptance</t>
+        </is>
+      </c>
+      <c r="B14" s="131" t="inlineStr">
+        <is>
+          <t>D+0. EAI units committed; not yet issued. SSLC board confirms Option B.</t>
+        </is>
+      </c>
+      <c r="C14" s="131" t="inlineStr">
+        <is>
+          <t>Targeted</t>
+        </is>
+      </c>
+      <c r="D14" s="128" t="n"/>
+      <c r="E14" s="128" t="n"/>
+      <c r="F14" s="128" t="n"/>
+      <c r="G14" s="128" t="n"/>
     </row>
     <row r="15" ht="42" customHeight="1">
-      <c r="A15" s="81" t="inlineStr">
-        <is>
-          <t>6-month clock start</t>
-        </is>
-      </c>
-      <c r="B15" s="82" t="inlineStr">
-        <is>
-          <t>The 6-month clock begins only AFTER the RTO close makes the issuer/successor a reporting company. With a targeted RTO close ~6 months after financing close, the earliest Rule 144 window under the 6-month path is ~12 months post-issuance (close + 6 months). Actual timing depends on RTO completion and the conversion/resale registration schedule.</t>
-        </is>
-      </c>
-      <c r="C15" s="83" t="inlineStr">
-        <is>
-          <t>Targeted, not assured.</t>
-        </is>
-      </c>
+      <c r="A15" s="131" t="inlineStr">
+        <is>
+          <t>Financing close — units issued</t>
+        </is>
+      </c>
+      <c r="B15" s="131" t="inlineStr">
+        <is>
+          <t>Targeted Q1 FY27. EAI units formally issued as restricted/legended securities (Rule 504 Reg D).</t>
+        </is>
+      </c>
+      <c r="C15" s="131" t="inlineStr">
+        <is>
+          <t>Targeted, not assured</t>
+        </is>
+      </c>
+      <c r="D15" s="128" t="n"/>
+      <c r="E15" s="128" t="n"/>
+      <c r="F15" s="128" t="n"/>
+      <c r="G15" s="128" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="131" t="inlineStr">
+        <is>
+          <t>Targeted RTO close</t>
+        </is>
+      </c>
+      <c r="B16" s="131" t="inlineStr">
+        <is>
+          <t>~6 months post-financing close. RTO listing occurs; EAI units become part of the public float and are tradeable at going public, subject to the principals' lockup.</t>
+        </is>
+      </c>
+      <c r="C16" s="131" t="inlineStr">
+        <is>
+          <t>Targeted, not assured</t>
+        </is>
+      </c>
+      <c r="D16" s="128" t="n"/>
+      <c r="E16" s="128" t="n"/>
+      <c r="F16" s="128" t="n"/>
+      <c r="G16" s="128" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="80" t="inlineStr">
-        <is>
-          <t>C.  RTO Structure — Preferred-at-Close / Conversion Path</t>
-        </is>
-      </c>
+      <c r="A17" s="133" t="inlineStr">
+        <is>
+          <t>ALL DATES</t>
+        </is>
+      </c>
+      <c r="B17" s="133" t="inlineStr">
+        <is>
+          <t>TARGETED, NOT ASSURED. The RTO may not close.</t>
+        </is>
+      </c>
+      <c r="C17" s="133" t="inlineStr">
+        <is>
+          <t>Risk</t>
+        </is>
+      </c>
+      <c r="D17" s="128" t="n"/>
+      <c r="E17" s="128" t="n"/>
+      <c r="F17" s="128" t="n"/>
+      <c r="G17" s="128" t="n"/>
     </row>
     <row r="18" ht="48" customHeight="1">
-      <c r="A18" s="81" t="inlineStr">
-        <is>
-          <t>RTO mechanics</t>
-        </is>
-      </c>
-      <c r="B18" s="82" t="inlineStr">
-        <is>
-          <t>Merger closes BEFORE the public stockholder vote using non-voting, non-convertible preferred stock (avoids NASDAQ Rule 5635 early-stage trigger). A proxy is filed within ~30 days of RTO close.</t>
-        </is>
-      </c>
-      <c r="C18" s="83" t="inlineStr">
-        <is>
-          <t>Source: Ainigma_RTO_Board_Brief_2026-09-04.md:16.</t>
-        </is>
-      </c>
+      <c r="A18" s="128" t="n"/>
+      <c r="B18" s="128" t="n"/>
+      <c r="C18" s="128" t="n"/>
+      <c r="D18" s="128" t="n"/>
+      <c r="E18" s="128" t="n"/>
+      <c r="F18" s="128" t="n"/>
+      <c r="G18" s="128" t="n"/>
     </row>
     <row r="19" ht="48" customHeight="1">
-      <c r="A19" s="81" t="inlineStr">
-        <is>
-          <t>Preferred → common</t>
-        </is>
-      </c>
-      <c r="B19" s="82" t="inlineStr">
-        <is>
-          <t>Preferred converts to common and becomes liquid ONLY after: (i) post-close public-shareholder vote (that founders do not control at the moment of close), AND (ii) effective resale registration (S-1/S-3).</t>
-        </is>
-      </c>
-      <c r="C19" s="83" t="inlineStr">
-        <is>
-          <t>Sources: Board Brief 2026-09-04.md:16; Board Questions 2026-09-08.md:36,44.</t>
-        </is>
-      </c>
+      <c r="A19" s="127" t="inlineStr">
+        <is>
+          <t>C.  Projected Post-RTO Value  —  PROJECTION, NOT A PROMISE</t>
+        </is>
+      </c>
+      <c r="B19" s="128" t="n"/>
+      <c r="C19" s="128" t="n"/>
+      <c r="D19" s="128" t="n"/>
+      <c r="E19" s="128" t="n"/>
+      <c r="F19" s="128" t="n"/>
+      <c r="G19" s="128" t="n"/>
     </row>
     <row r="20" ht="48" customHeight="1">
-      <c r="A20" s="81" t="inlineStr">
-        <is>
-          <t>EAI units follow same path</t>
-        </is>
-      </c>
-      <c r="B20" s="82" t="inlineStr">
-        <is>
-          <t>The EAI units' liquidity follows the identical path: committed at board acceptance → issued at financing close → held as restricted/non-trading until RTO close → preferred conversion vote → resale registration effective → Rule 144 / free-trading eligibility.</t>
-        </is>
-      </c>
-      <c r="C20" s="83" t="inlineStr">
-        <is>
-          <t>See timeline table below.</t>
-        </is>
-      </c>
+      <c r="A20" s="129" t="inlineStr">
+        <is>
+          <t>CAUTIONARY STATEMENT: Forward-looking projection — management assumptions (RTO completion, listing valuation, ~30% dilution). Not a guarantee; actual results may differ. RTO may not close. SEC Rule 10b-5 (https://www.ecfr.gov/current/title-17/chapter-II/part-240/section-240.10b-5) antifraud rules apply.</t>
+        </is>
+      </c>
+      <c r="B20" s="128" t="n"/>
+      <c r="C20" s="128" t="n"/>
+      <c r="D20" s="128" t="n"/>
+      <c r="E20" s="128" t="n"/>
+      <c r="F20" s="128" t="n"/>
+      <c r="G20" s="128" t="n"/>
     </row>
     <row r="21" ht="48" customHeight="1">
-      <c r="A21" s="81" t="inlineStr">
-        <is>
-          <t>Risk if vote fails / reg stalls</t>
-        </is>
-      </c>
-      <c r="B21" s="82" t="inlineStr">
-        <is>
-          <t>If the conversion vote fails or the resale registration stalls, holders of the EAI units (like founders) hold restricted, non-voting paper with no near-term liquidity. This is a known RTO structure, not disqualifying, but must be understood.</t>
-        </is>
-      </c>
-      <c r="C21" s="83" t="inlineStr">
-        <is>
-          <t>Source: Board Brief:44; Board Questions:62.</t>
+      <c r="A21" s="134" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="B21" s="134" t="inlineStr">
+        <is>
+          <t>RTO MEV</t>
+        </is>
+      </c>
+      <c r="C21" s="134" t="inlineStr">
+        <is>
+          <t>~0.59% pre-dil</t>
+        </is>
+      </c>
+      <c r="D21" s="134" t="inlineStr">
+        <is>
+          <t>~30% dilution</t>
+        </is>
+      </c>
+      <c r="E21" s="134" t="inlineStr">
+        <is>
+          <t>~0.59% post-dil</t>
+        </is>
+      </c>
+      <c r="F21" s="134" t="inlineStr">
+        <is>
+          <t>409A at issuance</t>
+        </is>
+      </c>
+      <c r="G21" s="134" t="inlineStr">
+        <is>
+          <t>+ earn-out at listing</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="131" t="inlineStr">
+        <is>
+          <t>Low (floor)</t>
+        </is>
+      </c>
+      <c r="B22" s="131" t="inlineStr">
+        <is>
+          <t>$200M</t>
+        </is>
+      </c>
+      <c r="C22" s="131" t="inlineStr">
+        <is>
+          <t>$1.18M</t>
+        </is>
+      </c>
+      <c r="D22" s="131" t="inlineStr">
+        <is>
+          <t>−$0.35M</t>
+        </is>
+      </c>
+      <c r="E22" s="131" t="inlineStr">
+        <is>
+          <t>$0.83M</t>
+        </is>
+      </c>
+      <c r="F22" s="131" t="inlineStr">
+        <is>
+          <t>$1.0M (409A)</t>
+        </is>
+      </c>
+      <c r="G22" s="131" t="inlineStr">
+        <is>
+          <t>$0  (0.0%)</t>
         </is>
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="80" t="inlineStr">
-        <is>
-          <t>D.  Liquidity Timeline  (Targeted — Not Assured)</t>
+      <c r="A23" s="131" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="B23" s="131" t="inlineStr">
+        <is>
+          <t>$250M</t>
+        </is>
+      </c>
+      <c r="C23" s="131" t="inlineStr">
+        <is>
+          <t>$1.47M</t>
+        </is>
+      </c>
+      <c r="D23" s="131" t="inlineStr">
+        <is>
+          <t>−$0.44M</t>
+        </is>
+      </c>
+      <c r="E23" s="131" t="inlineStr">
+        <is>
+          <t>$1.03M</t>
+        </is>
+      </c>
+      <c r="F23" s="131" t="inlineStr">
+        <is>
+          <t>$1.0M (409A)</t>
+        </is>
+      </c>
+      <c r="G23" s="131" t="inlineStr">
+        <is>
+          <t>+$625K  (0.25%)</t>
         </is>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="84" t="inlineStr">
-        <is>
-          <t>Milestone</t>
-        </is>
-      </c>
-      <c r="B24" s="84" t="inlineStr">
-        <is>
-          <t>Target / Detail</t>
-        </is>
-      </c>
-      <c r="C24" s="84" t="inlineStr">
-        <is>
-          <t>Status</t>
+      <c r="A24" s="131" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B24" s="131" t="inlineStr">
+        <is>
+          <t>$300M</t>
+        </is>
+      </c>
+      <c r="C24" s="131" t="inlineStr">
+        <is>
+          <t>$1.77M</t>
+        </is>
+      </c>
+      <c r="D24" s="131" t="inlineStr">
+        <is>
+          <t>−$0.53M</t>
+        </is>
+      </c>
+      <c r="E24" s="131" t="inlineStr">
+        <is>
+          <t>$1.24M</t>
+        </is>
+      </c>
+      <c r="F24" s="131" t="inlineStr">
+        <is>
+          <t>$1.0M (409A)</t>
+        </is>
+      </c>
+      <c r="G24" s="131" t="inlineStr">
+        <is>
+          <t>+$1,500K  (0.50%)</t>
         </is>
       </c>
     </row>
     <row r="25" ht="36" customHeight="1">
-      <c r="A25" s="81" t="inlineStr">
-        <is>
-          <t>Board acceptance</t>
-        </is>
-      </c>
-      <c r="B25" s="82" t="inlineStr">
-        <is>
-          <t>D+0. EAI units committed; not yet issued. SSLC board confirms Option B.</t>
-        </is>
-      </c>
-      <c r="C25" s="85" t="inlineStr">
-        <is>
-          <t>Targeted</t>
-        </is>
-      </c>
+      <c r="A25" s="129" t="inlineStr">
+        <is>
+          <t>Notes: MEV per Ainigma mandate. Dilution ~30% (Series A D1–D4 ~13% + RTO ~12% + pool ~5%). Post-dil = (~0.589%) × (1−0.30) × MEV. $1.0M counts toward Rule 504 $10M rolling cap. Earn-out column is ADDITIONAL at listing. Full Y5 hold: 'Total Compensation' sheet. Rule 10b-5: https://www.ecfr.gov/current/title-17/chapter-II/part-240/section-240.10b-5. Rule 504: https://www.sec.gov/resources-small-businesses/exempt-offerings/exemption-limited-offerings-not-exceeding-10-million-rule-504-regulation-d.</t>
+        </is>
+      </c>
+      <c r="B25" s="128" t="n"/>
+      <c r="C25" s="128" t="n"/>
+      <c r="D25" s="128" t="n"/>
+      <c r="E25" s="128" t="n"/>
+      <c r="F25" s="128" t="n"/>
+      <c r="G25" s="128" t="n"/>
     </row>
     <row r="26" ht="36" customHeight="1">
-      <c r="A26" s="81" t="inlineStr">
-        <is>
-          <t>Financing close — units issued</t>
-        </is>
-      </c>
-      <c r="B26" s="82" t="inlineStr">
-        <is>
-          <t>Targeted Q1 FY27 (~2026-Q4/Q1 2027). EAI units formally issued. Rule 144 holding period (1-year, non-reporting) clock starts.</t>
-        </is>
-      </c>
-      <c r="C26" s="85" t="inlineStr">
-        <is>
-          <t>Targeted, not assured</t>
-        </is>
-      </c>
+      <c r="A26" s="128" t="n"/>
+      <c r="B26" s="128" t="n"/>
+      <c r="C26" s="128" t="n"/>
+      <c r="D26" s="128" t="n"/>
+      <c r="E26" s="128" t="n"/>
+      <c r="F26" s="128" t="n"/>
+      <c r="G26" s="128" t="n"/>
     </row>
     <row r="27" ht="36" customHeight="1">
-      <c r="A27" s="81" t="inlineStr">
-        <is>
-          <t>Targeted RTO close</t>
-        </is>
-      </c>
-      <c r="B27" s="82" t="inlineStr">
-        <is>
-          <t>~6 months post-financing close. Exos/NewCo merger closes using non-voting preferred. NOT the liquidity event — preferred not yet tradeable.</t>
-        </is>
-      </c>
-      <c r="C27" s="85" t="inlineStr">
-        <is>
-          <t>Targeted, not assured</t>
-        </is>
-      </c>
+      <c r="A27" s="128" t="n"/>
+      <c r="B27" s="128" t="n"/>
+      <c r="C27" s="128" t="n"/>
+      <c r="D27" s="128" t="n"/>
+      <c r="E27" s="128" t="n"/>
+      <c r="F27" s="128" t="n"/>
+      <c r="G27" s="128" t="n"/>
     </row>
     <row r="28" ht="36" customHeight="1">
-      <c r="A28" s="81" t="inlineStr">
-        <is>
-          <t>Proxy filed / shareholder vote</t>
-        </is>
-      </c>
-      <c r="B28" s="82" t="inlineStr">
-        <is>
-          <t>~30 days post-RTO close. Public stockholder vote on preferred → common conversion.</t>
-        </is>
-      </c>
-      <c r="C28" s="85" t="inlineStr">
-        <is>
-          <t>Targeted, not assured</t>
-        </is>
-      </c>
+      <c r="A28" s="128" t="n"/>
+      <c r="B28" s="128" t="n"/>
+      <c r="C28" s="128" t="n"/>
+      <c r="D28" s="128" t="n"/>
+      <c r="E28" s="128" t="n"/>
+      <c r="F28" s="128" t="n"/>
+      <c r="G28" s="128" t="n"/>
     </row>
     <row r="29" ht="36" customHeight="1">
-      <c r="A29" s="81" t="inlineStr">
-        <is>
-          <t>Resale registration effective (S-1/S-3)</t>
-        </is>
-      </c>
-      <c r="B29" s="82" t="inlineStr">
-        <is>
-          <t>~30–90 days post-RTO close (concurrent with or following vote). Registration must go effective before preferred converts to tradeable common.</t>
-        </is>
-      </c>
-      <c r="C29" s="85" t="inlineStr">
-        <is>
-          <t>Targeted, not assured</t>
-        </is>
-      </c>
+      <c r="A29" s="128" t="n"/>
+      <c r="B29" s="128" t="n"/>
+      <c r="C29" s="128" t="n"/>
+      <c r="D29" s="128" t="n"/>
+      <c r="E29" s="128" t="n"/>
+      <c r="F29" s="128" t="n"/>
+      <c r="G29" s="128" t="n"/>
     </row>
     <row r="30" ht="36" customHeight="1">
-      <c r="A30" s="81" t="inlineStr">
-        <is>
-          <t>Rule 144 eligibility — 6-month path</t>
-        </is>
-      </c>
-      <c r="B30" s="82" t="inlineStr">
-        <is>
-          <t>AFTER reporting status is established AND ≥6 months from issuance date. Earliest: ~12 months post-issuance (close + RTO ~6 mo + holding). Requires current public information available.</t>
-        </is>
-      </c>
-      <c r="C30" s="85" t="inlineStr">
-        <is>
-          <t>Targeted, not assured</t>
-        </is>
-      </c>
+      <c r="A30" s="128" t="n"/>
+      <c r="B30" s="128" t="n"/>
+      <c r="C30" s="128" t="n"/>
+      <c r="D30" s="128" t="n"/>
+      <c r="E30" s="128" t="n"/>
+      <c r="F30" s="128" t="n"/>
+      <c r="G30" s="128" t="n"/>
     </row>
     <row r="31" ht="36" customHeight="1">
-      <c r="A31" s="81" t="inlineStr">
-        <is>
-          <t>Rule 144 eligibility — 1-year path</t>
-        </is>
-      </c>
-      <c r="B31" s="82" t="inlineStr">
-        <is>
-          <t>1 year from issuance date (non-reporting issuer path). If RTO does not close by 1-year mark, this is the available resale window.</t>
-        </is>
-      </c>
-      <c r="C31" s="85" t="inlineStr">
-        <is>
-          <t>Fallback if 6-mo path unavailable</t>
-        </is>
-      </c>
+      <c r="A31" s="128" t="n"/>
+      <c r="B31" s="128" t="n"/>
+      <c r="C31" s="128" t="n"/>
+      <c r="D31" s="128" t="n"/>
+      <c r="E31" s="128" t="n"/>
+      <c r="F31" s="128" t="n"/>
+      <c r="G31" s="128" t="n"/>
     </row>
     <row r="32" ht="36" customHeight="1">
-      <c r="A32" s="86" t="inlineStr">
-        <is>
-          <t>ALL DATES</t>
-        </is>
-      </c>
-      <c r="B32" s="87" t="inlineStr">
-        <is>
-          <t>TARGETED, NOT ASSURED. The RTO may not close.</t>
-        </is>
-      </c>
-      <c r="C32" s="88" t="inlineStr">
-        <is>
-          <t>Risk</t>
-        </is>
-      </c>
+      <c r="A32" s="128" t="n"/>
+      <c r="B32" s="128" t="n"/>
+      <c r="C32" s="128" t="n"/>
+      <c r="D32" s="128" t="n"/>
+      <c r="E32" s="128" t="n"/>
+      <c r="F32" s="128" t="n"/>
+      <c r="G32" s="128" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="128" t="n"/>
+      <c r="B33" s="128" t="n"/>
+      <c r="C33" s="128" t="n"/>
+      <c r="D33" s="128" t="n"/>
+      <c r="E33" s="128" t="n"/>
+      <c r="F33" s="128" t="n"/>
+      <c r="G33" s="128" t="n"/>
     </row>
     <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="89" t="inlineStr">
-        <is>
-          <t>E.  Projected Post-RTO Value  —  PROJECTION, NOT A PROMISE</t>
-        </is>
-      </c>
+      <c r="A34" s="128" t="n"/>
+      <c r="B34" s="128" t="n"/>
+      <c r="C34" s="128" t="n"/>
+      <c r="D34" s="128" t="n"/>
+      <c r="E34" s="128" t="n"/>
+      <c r="F34" s="128" t="n"/>
+      <c r="G34" s="128" t="n"/>
     </row>
     <row r="35" ht="60" customHeight="1">
-      <c r="A35" s="90" t="inlineStr">
-        <is>
-          <t>CAUTIONARY STATEMENT: Forward-looking projection based on management assumptions (RTO completion, listing valuation, ~30% dilution). Not a guarantee or promise of value; actual results may differ materially. The RTO may not close. SEC Rule 10b-5 (17 CFR 240.10b-5; https://www.ecfr.gov/current/title-17/chapter-II/part-240/section-240.10b-5) antifraud rules apply to projections. Projections must have a reasonable basis; do not rely on this section as an offer to sell or inducement beyond the framing above.</t>
-        </is>
-      </c>
+      <c r="A35" s="128" t="n"/>
+      <c r="B35" s="128" t="n"/>
+      <c r="C35" s="128" t="n"/>
+      <c r="D35" s="128" t="n"/>
+      <c r="E35" s="128" t="n"/>
+      <c r="F35" s="128" t="n"/>
+      <c r="G35" s="128" t="n"/>
     </row>
     <row r="36" ht="28" customHeight="1">
-      <c r="A36" s="70" t="inlineStr">
-        <is>
-          <t>Scenario</t>
-        </is>
-      </c>
-      <c r="B36" s="70" t="inlineStr">
-        <is>
-          <t>RTO MEV</t>
-        </is>
-      </c>
-      <c r="C36" s="70" t="inlineStr">
-        <is>
-          <t>~0.59% pre-dilution</t>
-        </is>
-      </c>
-      <c r="D36" s="70" t="inlineStr">
-        <is>
-          <t>~30% dilution</t>
-        </is>
-      </c>
-      <c r="E36" s="70" t="inlineStr">
-        <is>
-          <t>~0.59% post-dilution (up-front only)</t>
-        </is>
-      </c>
-      <c r="F36" s="70" t="inlineStr">
-        <is>
-          <t>409A at issuance</t>
-        </is>
-      </c>
-      <c r="G36" s="70" t="inlineStr">
-        <is>
-          <t>Additional: earn-out at listing</t>
-        </is>
-      </c>
+      <c r="A36" s="128" t="n"/>
+      <c r="B36" s="128" t="n"/>
+      <c r="C36" s="128" t="n"/>
+      <c r="D36" s="128" t="n"/>
+      <c r="E36" s="128" t="n"/>
+      <c r="F36" s="128" t="n"/>
+      <c r="G36" s="128" t="n"/>
     </row>
     <row r="37" ht="22" customHeight="1">
-      <c r="A37" s="91" t="inlineStr">
-        <is>
-          <t>Low (floor)</t>
-        </is>
-      </c>
-      <c r="B37" s="91" t="inlineStr">
-        <is>
-          <t>$200M</t>
-        </is>
-      </c>
-      <c r="C37" s="91" t="inlineStr">
-        <is>
-          <t>$1.18M</t>
-        </is>
-      </c>
-      <c r="D37" s="91" t="inlineStr">
-        <is>
-          <t>−$0.35M</t>
-        </is>
-      </c>
-      <c r="E37" s="91" t="inlineStr">
-        <is>
-          <t>$0.83M</t>
-        </is>
-      </c>
-      <c r="F37" s="91" t="inlineStr">
-        <is>
-          <t>$1.0M (409A)</t>
-        </is>
-      </c>
-      <c r="G37" s="91" t="inlineStr">
-        <is>
-          <t>$0  (0.0% earn-out)</t>
-        </is>
-      </c>
+      <c r="A37" s="128" t="n"/>
+      <c r="B37" s="128" t="n"/>
+      <c r="C37" s="128" t="n"/>
+      <c r="D37" s="128" t="n"/>
+      <c r="E37" s="128" t="n"/>
+      <c r="F37" s="128" t="n"/>
+      <c r="G37" s="128" t="n"/>
     </row>
     <row r="38" ht="22" customHeight="1">
-      <c r="A38" s="92" t="inlineStr">
-        <is>
-          <t>Base</t>
-        </is>
-      </c>
-      <c r="B38" s="92" t="inlineStr">
-        <is>
-          <t>$250M</t>
-        </is>
-      </c>
-      <c r="C38" s="92" t="inlineStr">
-        <is>
-          <t>$1.47M</t>
-        </is>
-      </c>
-      <c r="D38" s="92" t="inlineStr">
-        <is>
-          <t>−$0.44M</t>
-        </is>
-      </c>
-      <c r="E38" s="92" t="inlineStr">
-        <is>
-          <t>$1.03M</t>
-        </is>
-      </c>
-      <c r="F38" s="92" t="inlineStr">
-        <is>
-          <t>$1.0M (409A)</t>
-        </is>
-      </c>
-      <c r="G38" s="92" t="inlineStr">
-        <is>
-          <t>+$625K  (0.25%)</t>
-        </is>
-      </c>
+      <c r="A38" s="128" t="n"/>
+      <c r="B38" s="128" t="n"/>
+      <c r="C38" s="128" t="n"/>
+      <c r="D38" s="128" t="n"/>
+      <c r="E38" s="128" t="n"/>
+      <c r="F38" s="128" t="n"/>
+      <c r="G38" s="128" t="n"/>
     </row>
     <row r="39" ht="22" customHeight="1">
-      <c r="A39" s="93" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="B39" s="93" t="inlineStr">
-        <is>
-          <t>$300M</t>
-        </is>
-      </c>
-      <c r="C39" s="93" t="inlineStr">
-        <is>
-          <t>$1.77M</t>
-        </is>
-      </c>
-      <c r="D39" s="93" t="inlineStr">
-        <is>
-          <t>−$0.53M</t>
-        </is>
-      </c>
-      <c r="E39" s="93" t="inlineStr">
-        <is>
-          <t>$1.24M</t>
-        </is>
-      </c>
-      <c r="F39" s="93" t="inlineStr">
-        <is>
-          <t>$1.0M (409A)</t>
-        </is>
-      </c>
-      <c r="G39" s="93" t="inlineStr">
-        <is>
-          <t>+$1,500K  (0.50%)</t>
-        </is>
-      </c>
+      <c r="A39" s="128" t="n"/>
+      <c r="B39" s="128" t="n"/>
+      <c r="C39" s="128" t="n"/>
+      <c r="D39" s="128" t="n"/>
+      <c r="E39" s="128" t="n"/>
+      <c r="F39" s="128" t="n"/>
+      <c r="G39" s="128" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="128" t="n"/>
+      <c r="B40" s="128" t="n"/>
+      <c r="C40" s="128" t="n"/>
+      <c r="D40" s="128" t="n"/>
+      <c r="E40" s="128" t="n"/>
+      <c r="F40" s="128" t="n"/>
+      <c r="G40" s="128" t="n"/>
     </row>
     <row r="41" ht="60" customHeight="1">
-      <c r="A41" s="94" t="inlineStr">
-        <is>
-          <t>Notes: MEV per Ainigma mandate ($250M min, $300M stretch). Dilution ~30% (Series A D1–D4 ~13% + RTO ~12% + option pool ~5%) — management assumption. Post-dil = (~0.589%) × (1 − 0.30) × MEV. $1.0M counts toward the Rule 504 $10M rolling cap. Earn-out column is ADDITIONAL at listing price; not additive to 409A value. Full Y5 hold analysis (16× EV/EBITDA): model 'Total Compensation' sheet. Rule 10b-5 reference: https://www.ecfr.gov/current/title-17/chapter-II/part-240/section-240.10b-5. Rule 144 reference: https://www.ecfr.gov/current/title-17/chapter-II/part-230/section-230.144. Rule 504 reference: https://www.sec.gov/resources-small-businesses/exempt-offerings/exemption-limited-offerings-not-exceeding-10-million-rule-504-regulation-d.</t>
-        </is>
-      </c>
+      <c r="A41" s="128" t="n"/>
+      <c r="B41" s="128" t="n"/>
+      <c r="C41" s="128" t="n"/>
+      <c r="D41" s="128" t="n"/>
+      <c r="E41" s="128" t="n"/>
+      <c r="F41" s="128" t="n"/>
+      <c r="G41" s="128" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="A41:C41"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A23:C23"/>
-    <mergeCell ref="A17:C17"/>
-    <mergeCell ref="A34:C34"/>
-    <mergeCell ref="A35:C35"/>
-    <mergeCell ref="A4:C4"/>
-    <mergeCell ref="A2:C2"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -7761,9 +7988,36 @@
           <t>KEY FACT:  Reaching $5.1M in FY27 requires averaging $1.46M/quarter for Q2–Q4  ($5,100K − $713K Q1 actual ÷ 3 quarters = $1,462K/qtr)  —  approximately 2.05× the most recent quarter's $713K  —  starting immediately.  Without Exos capital to fund working capital and IM ramp, that doubling is not achievable on SSLC's $198K cash position.</t>
         </is>
       </c>
-    </row>
-    <row r="5" ht="22" customHeight="1"/>
-    <row r="6" ht="22" customHeight="1"/>
+      <c r="B4" s="135" t="n"/>
+      <c r="C4" s="135" t="n"/>
+      <c r="D4" s="135" t="n"/>
+      <c r="E4" s="135" t="n"/>
+      <c r="F4" s="135" t="n"/>
+      <c r="G4" s="135" t="n"/>
+      <c r="H4" s="135" t="n"/>
+      <c r="I4" s="135" t="n"/>
+      <c r="J4" s="135" t="n"/>
+      <c r="K4" s="135" t="n"/>
+      <c r="L4" s="136" t="n"/>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="137" t="n"/>
+      <c r="L5" s="138" t="n"/>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="139" t="n"/>
+      <c r="B6" s="140" t="n"/>
+      <c r="C6" s="140" t="n"/>
+      <c r="D6" s="140" t="n"/>
+      <c r="E6" s="140" t="n"/>
+      <c r="F6" s="140" t="n"/>
+      <c r="G6" s="140" t="n"/>
+      <c r="H6" s="140" t="n"/>
+      <c r="I6" s="140" t="n"/>
+      <c r="J6" s="140" t="n"/>
+      <c r="K6" s="140" t="n"/>
+      <c r="L6" s="141" t="n"/>
+    </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="98" t="inlineStr">
         <is>
@@ -7820,6 +8074,10 @@
           <t xml:space="preserve">  Cash on hand (10/2/26):  $198K</t>
         </is>
       </c>
+      <c r="I10" s="142" t="n"/>
+      <c r="J10" s="142" t="n"/>
+      <c r="K10" s="142" t="n"/>
+      <c r="L10" s="143" t="n"/>
     </row>
     <row r="11" ht="16" customHeight="1">
       <c r="A11" s="104" t="inlineStr">
@@ -7847,6 +8105,10 @@
           <t xml:space="preserve">  Working capital needed to maintain deliveries:  $300K–$700K</t>
         </is>
       </c>
+      <c r="I11" s="142" t="n"/>
+      <c r="J11" s="142" t="n"/>
+      <c r="K11" s="142" t="n"/>
+      <c r="L11" s="143" t="n"/>
     </row>
     <row r="12" ht="16" customHeight="1">
       <c r="A12" s="104" t="inlineStr">
@@ -7872,6 +8134,10 @@
           <t xml:space="preserve">  FY26 operating loss:  −$416K</t>
         </is>
       </c>
+      <c r="I12" s="142" t="n"/>
+      <c r="J12" s="142" t="n"/>
+      <c r="K12" s="142" t="n"/>
+      <c r="L12" s="143" t="n"/>
     </row>
     <row r="13" ht="16" customHeight="1">
       <c r="A13" s="104" t="inlineStr">
@@ -7899,6 +8165,10 @@
           <t xml:space="preserve">  He-tank rework unresolved — no resolution path without new owner</t>
         </is>
       </c>
+      <c r="I13" s="142" t="n"/>
+      <c r="J13" s="142" t="n"/>
+      <c r="K13" s="142" t="n"/>
+      <c r="L13" s="143" t="n"/>
     </row>
     <row r="14" ht="16" customHeight="1">
       <c r="A14" s="104" t="inlineStr">
@@ -7926,6 +8196,10 @@
           <t xml:space="preserve">  No capex capacity → headcount/equipment frozen</t>
         </is>
       </c>
+      <c r="I14" s="142" t="n"/>
+      <c r="J14" s="142" t="n"/>
+      <c r="K14" s="142" t="n"/>
+      <c r="L14" s="143" t="n"/>
     </row>
     <row r="15" ht="16" customHeight="1">
       <c r="A15" s="112" t="inlineStr">
@@ -7938,6 +8212,10 @@
           <t xml:space="preserve">  Growth capped by self-funded working capital</t>
         </is>
       </c>
+      <c r="I15" s="142" t="n"/>
+      <c r="J15" s="142" t="n"/>
+      <c r="K15" s="142" t="n"/>
+      <c r="L15" s="143" t="n"/>
     </row>
     <row r="16" ht="16" customHeight="1">
       <c r="H16" s="103" t="inlineStr">
@@ -7945,6 +8223,10 @@
           <t xml:space="preserve">  FY27 achievable at run-rate:  ~$2.85M</t>
         </is>
       </c>
+      <c r="I16" s="142" t="n"/>
+      <c r="J16" s="142" t="n"/>
+      <c r="K16" s="142" t="n"/>
+      <c r="L16" s="143" t="n"/>
     </row>
     <row r="17" ht="16" customHeight="1">
       <c r="A17" s="113" t="inlineStr">
@@ -7957,6 +8239,10 @@
           <t xml:space="preserve">  FY31 best-case (10% CAGR, no stall):  ~$4.2M</t>
         </is>
       </c>
+      <c r="I17" s="142" t="n"/>
+      <c r="J17" s="142" t="n"/>
+      <c r="K17" s="142" t="n"/>
+      <c r="L17" s="143" t="n"/>
     </row>
     <row r="18" ht="16" customHeight="1">
       <c r="A18" s="114" t="inlineStr">
@@ -7969,6 +8255,10 @@
           <t xml:space="preserve">  5-yr CAGR (status quo):  ~10.0%</t>
         </is>
       </c>
+      <c r="I18" s="142" t="n"/>
+      <c r="J18" s="142" t="n"/>
+      <c r="K18" s="142" t="n"/>
+      <c r="L18" s="143" t="n"/>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="102" t="inlineStr"/>
@@ -8049,6 +8339,10 @@
           <t xml:space="preserve">  Cash at close:  $2.51M</t>
         </is>
       </c>
+      <c r="I21" s="142" t="n"/>
+      <c r="J21" s="142" t="n"/>
+      <c r="K21" s="142" t="n"/>
+      <c r="L21" s="143" t="n"/>
     </row>
     <row r="22" ht="16" customHeight="1">
       <c r="A22" s="104" t="inlineStr">
@@ -8076,6 +8370,10 @@
           <t xml:space="preserve">  SSLC debts paid at face (est. ~$500K TBV)</t>
         </is>
       </c>
+      <c r="I22" s="142" t="n"/>
+      <c r="J22" s="142" t="n"/>
+      <c r="K22" s="142" t="n"/>
+      <c r="L22" s="143" t="n"/>
     </row>
     <row r="23" ht="16" customHeight="1">
       <c r="A23" s="104" t="inlineStr">
@@ -8103,6 +8401,10 @@
           <t xml:space="preserve">  Prepaid-work delivery funded (cost $500K)</t>
         </is>
       </c>
+      <c r="I23" s="142" t="n"/>
+      <c r="J23" s="142" t="n"/>
+      <c r="K23" s="142" t="n"/>
+      <c r="L23" s="143" t="n"/>
     </row>
     <row r="24" ht="16" customHeight="1">
       <c r="H24" s="103" t="inlineStr">
@@ -8110,6 +8412,10 @@
           <t xml:space="preserve">  WC bridge removes Q2–Q3 stall risk</t>
         </is>
       </c>
+      <c r="I24" s="142" t="n"/>
+      <c r="J24" s="142" t="n"/>
+      <c r="K24" s="142" t="n"/>
+      <c r="L24" s="143" t="n"/>
     </row>
     <row r="25" ht="16" customHeight="1">
       <c r="A25" s="99" t="inlineStr">
@@ -8122,6 +8428,10 @@
           <t xml:space="preserve">  Exos procurement channel:  immediate BLK3 tank POs</t>
         </is>
       </c>
+      <c r="I25" s="142" t="n"/>
+      <c r="J25" s="142" t="n"/>
+      <c r="K25" s="142" t="n"/>
+      <c r="L25" s="143" t="n"/>
     </row>
     <row r="26" ht="16" customHeight="1">
       <c r="A26" s="102" t="inlineStr">
@@ -8154,6 +8464,10 @@
           <t xml:space="preserve">  Intuitive Machines ramp:  14–16 tanks firm FY27</t>
         </is>
       </c>
+      <c r="I26" s="142" t="n"/>
+      <c r="J26" s="142" t="n"/>
+      <c r="K26" s="142" t="n"/>
+      <c r="L26" s="143" t="n"/>
     </row>
     <row r="27" ht="16" customHeight="1">
       <c r="A27" s="119" t="inlineStr">
@@ -8172,6 +8486,10 @@
           <t xml:space="preserve">  Capex for production scale-up enabled</t>
         </is>
       </c>
+      <c r="I27" s="142" t="n"/>
+      <c r="J27" s="142" t="n"/>
+      <c r="K27" s="142" t="n"/>
+      <c r="L27" s="143" t="n"/>
     </row>
     <row r="28" ht="16" customHeight="1">
       <c r="A28" s="119" t="inlineStr">
@@ -8190,6 +8508,10 @@
           <t xml:space="preserve">  FY27 target (IM firm + ramp):  $4.1M–$5.5M</t>
         </is>
       </c>
+      <c r="I28" s="142" t="n"/>
+      <c r="J28" s="142" t="n"/>
+      <c r="K28" s="142" t="n"/>
+      <c r="L28" s="143" t="n"/>
     </row>
     <row r="29" ht="16" customHeight="1">
       <c r="A29" s="119" t="inlineStr">
@@ -8208,6 +8530,10 @@
           <t xml:space="preserve">  FY31 (v12 trajectory):  $54.7M</t>
         </is>
       </c>
+      <c r="I29" s="142" t="n"/>
+      <c r="J29" s="142" t="n"/>
+      <c r="K29" s="142" t="n"/>
+      <c r="L29" s="143" t="n"/>
     </row>
     <row r="30" ht="16" customHeight="1">
       <c r="A30" s="119" t="inlineStr">
@@ -8226,6 +8552,10 @@
           <t xml:space="preserve">  5-yr CAGR (with Exos, v12):  ~90.9%</t>
         </is>
       </c>
+      <c r="I30" s="142" t="n"/>
+      <c r="J30" s="142" t="n"/>
+      <c r="K30" s="142" t="n"/>
+      <c r="L30" s="143" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="119" t="inlineStr">
@@ -8260,6 +8590,10 @@
           <t xml:space="preserve">  FY27 $5.1M target − Q1 $713K actual = $4,387K remaining</t>
         </is>
       </c>
+      <c r="I33" s="142" t="n"/>
+      <c r="J33" s="142" t="n"/>
+      <c r="K33" s="142" t="n"/>
+      <c r="L33" s="143" t="n"/>
     </row>
     <row r="34" ht="16" customHeight="1">
       <c r="H34" s="103" t="inlineStr">
@@ -8267,6 +8601,10 @@
           <t xml:space="preserve">  Over 3 quarters (Q2–Q4) = $1,462K/qtr required</t>
         </is>
       </c>
+      <c r="I34" s="142" t="n"/>
+      <c r="J34" s="142" t="n"/>
+      <c r="K34" s="142" t="n"/>
+      <c r="L34" s="143" t="n"/>
     </row>
     <row r="35" ht="16" customHeight="1">
       <c r="H35" s="103" t="inlineStr">
@@ -8274,6 +8612,10 @@
           <t xml:space="preserve">  vs. Q1 $713K actual = 2.05× immediate ramp</t>
         </is>
       </c>
+      <c r="I35" s="142" t="n"/>
+      <c r="J35" s="142" t="n"/>
+      <c r="K35" s="142" t="n"/>
+      <c r="L35" s="143" t="n"/>
     </row>
     <row r="36" ht="16" customHeight="1">
       <c r="H36" s="103" t="inlineStr">
@@ -8281,6 +8623,10 @@
           <t xml:space="preserve">  Only funded if Exos capital bridges the working-capital gap</t>
         </is>
       </c>
+      <c r="I36" s="142" t="n"/>
+      <c r="J36" s="142" t="n"/>
+      <c r="K36" s="142" t="n"/>
+      <c r="L36" s="143" t="n"/>
     </row>
     <row r="37" ht="16" customHeight="1">
       <c r="H37" s="103" t="inlineStr">
@@ -8288,6 +8634,10 @@
           <t xml:space="preserve">  Without capital → Q2–Q4 stays ≈ $713K/qtr = $2.85M FY27</t>
         </is>
       </c>
+      <c r="I37" s="142" t="n"/>
+      <c r="J37" s="142" t="n"/>
+      <c r="K37" s="142" t="n"/>
+      <c r="L37" s="143" t="n"/>
     </row>
     <row r="40" ht="28" customHeight="1">
       <c r="A40" s="126" t="inlineStr">

</xml_diff>

<commit_message>
SSLC offer: EAI up-front units = float, no lockup at listing (John opt 2); employee term in summary
</commit_message>
<xml_diff>
--- a/drafts/EXOS_SSLC_OptionB_Acquisition_Model_2026-10-07.xlsx
+++ b/drafts/EXOS_SSLC_OptionB_Acquisition_Model_2026-10-07.xlsx
@@ -7438,12 +7438,12 @@
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="130" t="inlineStr">
         <is>
-          <t>Lockup — mirrors principals</t>
+          <t>No lockup at listing (float)</t>
         </is>
       </c>
       <c r="B9" s="131" t="inlineStr">
         <is>
-          <t>Same lockup terms as Exos Aerospace principals under the RTO transaction documents. Specific lock periods in the RTO definitive agreement govern.</t>
+          <t>John 10/9 (option 2): NO principals' lockup on the up-front EAI units. Locked-up shares are 'Restricted Securities' and do not count toward public float (Nasdaq Rule 5005(a)(38),(46); https://listingcenter.nasdaq.com/rulebook/nasdaq/rules/nasdaq-5000-series). Earn-out stock issued post-listing keeps principals' lockup terms.</t>
         </is>
       </c>
       <c r="C9" s="129" t="inlineStr">
@@ -7464,7 +7464,7 @@
       </c>
       <c r="B10" s="131" t="inlineStr">
         <is>
-          <t>The EAI units are structured to provide part of the public float for the Exos RTO and become tradeable at going public (the RTO listing), subject to the same lockup as Exos principals. Resale at listing assumes the units are included in the RTO's resale registration.</t>
+          <t>The EAI units are structured to provide part of the public float for the Exos RTO and become freely tradeable at going public (the RTO listing). Resale at listing assumes the units are included in the RTO's resale registration.</t>
         </is>
       </c>
       <c r="C10" s="128" t="n"/>
@@ -7566,7 +7566,7 @@
       </c>
       <c r="B16" s="131" t="inlineStr">
         <is>
-          <t>~6 months post-financing close. RTO listing occurs; EAI units become part of the public float and are tradeable at going public, subject to the principals' lockup.</t>
+          <t>~6 months post-financing close. RTO listing occurs; EAI units become part of the public float and are freely tradeable (no lockup), covered by the RTO resale registration.</t>
         </is>
       </c>
       <c r="C16" s="131" t="inlineStr">

</xml_diff>

<commit_message>
SSLC earn-out: reframe as single 5% rate + performance targets (Low $3M/Base $5M/High $6M+)
- Offer summary: replace 3%/5%/7% wording with target framing; add Earn-Out
  Targets FY27-31 table (tank + M1-M5 + stock + totals with check/dash marks);
  tighten to 2 pages
- Board deck slide 5: rebuild around 6-column targets table (Earn-out | Target |
  Low | Base | High | Pays) with per-year revenue targets and check/dash marks
- xlsx model Assumptions rows 23-25: change from rate inputs (0.03/0.05/0.07) to
  revenue target inputs ($3M/$5M/$6M); Total Compensation formulas updated to
  MIN(0.05*revTarget, cap); verified Low $150K/Base $250K/High $300K per yr
- build_sslc_option_b_model.py: same input changes applied (no regression)
- Totals verified: Low $950K / Base $2,525K / High $4,100K = III minus II
</commit_message>
<xml_diff>
--- a/drafts/EXOS_SSLC_OptionB_Acquisition_Model_2026-10-07.xlsx
+++ b/drafts/EXOS_SSLC_OptionB_Acquisition_Model_2026-10-07.xlsx
@@ -1414,45 +1414,45 @@
     <row r="23" ht="22" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>Earn-out i — IM tank revenue % (low)</t>
+          <t>Earn-out i — IM tank revenue target, LOW ($/yr)</t>
         </is>
       </c>
       <c r="B23" s="9" t="n">
-        <v>0.03</v>
+        <v>3000000</v>
       </c>
       <c r="C23" s="10" t="inlineStr">
         <is>
-          <t>Management assumption — unverified</t>
+          <t>Single rate 5%; MIN(5%×$3.0M, $300K cap) = $150K/yr → $750K over 5 yrs</t>
         </is>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>Earn-out i — IM tank revenue % (base)</t>
+          <t>Earn-out i — IM tank revenue target, BASE ($/yr)</t>
         </is>
       </c>
       <c r="B24" s="9" t="n">
-        <v>0.05</v>
+        <v>5000000</v>
       </c>
       <c r="C24" s="10" t="inlineStr">
         <is>
-          <t>Management assumption — unverified</t>
+          <t>Single rate 5%; MIN(5%×$5.0M, $300K cap) = $250K/yr → $1.25M over 5 yrs</t>
         </is>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>Earn-out i — IM tank revenue % (high)</t>
+          <t>Earn-out i — IM tank revenue target, HIGH ($/yr)</t>
         </is>
       </c>
       <c r="B25" s="9" t="n">
-        <v>0.07000000000000001</v>
+        <v>6000000</v>
       </c>
       <c r="C25" s="10" t="inlineStr">
         <is>
-          <t>Management assumption — unverified</t>
+          <t>Single rate 5%; MIN(5%×$6.0M, $300K cap) = $300K/yr (cap) → $1.5M over 5 yrs</t>
         </is>
       </c>
     </row>
@@ -6151,27 +6151,27 @@
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="59" t="inlineStr">
         <is>
-          <t>Tank earn-out base (i): 5%/yr, $300K cap, 5yr FY27–FY31</t>
+          <t>Tank earn-out base (i): 5%/yr × $5M/yr target, $300K cap, 5yr FY27–FY31</t>
         </is>
       </c>
       <c r="B14" s="32">
-        <f>MIN(Assumptions!B24*Assumptions!B44,Assumptions!B26)</f>
+        <f>MIN(0.05*Assumptions!B24,Assumptions!B26)</f>
         <v/>
       </c>
       <c r="C14" s="32">
-        <f>MIN(Assumptions!B24*Assumptions!B44,Assumptions!B26)</f>
+        <f>MIN(0.05*Assumptions!B24,Assumptions!B26)</f>
         <v/>
       </c>
       <c r="D14" s="32">
-        <f>MIN(Assumptions!B24*Assumptions!B44,Assumptions!B26)</f>
+        <f>MIN(0.05*Assumptions!B24,Assumptions!B26)</f>
         <v/>
       </c>
       <c r="E14" s="32">
-        <f>MIN(Assumptions!B24*Assumptions!B44,Assumptions!B26)</f>
+        <f>MIN(0.05*Assumptions!B24,Assumptions!B26)</f>
         <v/>
       </c>
       <c r="F14" s="32">
-        <f>MIN(Assumptions!B24*Assumptions!B44,Assumptions!B26)</f>
+        <f>MIN(0.05*Assumptions!B24,Assumptions!B26)</f>
         <v/>
       </c>
       <c r="G14" s="32">
@@ -6180,34 +6180,34 @@
       </c>
       <c r="H14" s="10" t="inlineStr">
         <is>
-          <t>5% × $5M firm IM ramp × 5 years; $300K/yr cap</t>
+          <t>5% × $5M revenue target × 5 yrs; $300K/yr cap → $250K/yr → $1.25M total</t>
         </is>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="59" t="inlineStr">
         <is>
-          <t>Tank earn-out low (i): 3%/yr × 5yr</t>
+          <t>Tank earn-out low (i): 5%/yr × $3M/yr target × 5yr</t>
         </is>
       </c>
       <c r="B15" s="32">
-        <f>MIN(Assumptions!B23*Assumptions!B44,Assumptions!B26)</f>
+        <f>MIN(0.05*Assumptions!B23,Assumptions!B26)</f>
         <v/>
       </c>
       <c r="C15" s="32">
-        <f>MIN(Assumptions!B23*Assumptions!B44,Assumptions!B26)</f>
+        <f>MIN(0.05*Assumptions!B23,Assumptions!B26)</f>
         <v/>
       </c>
       <c r="D15" s="32">
-        <f>MIN(Assumptions!B23*Assumptions!B44,Assumptions!B26)</f>
+        <f>MIN(0.05*Assumptions!B23,Assumptions!B26)</f>
         <v/>
       </c>
       <c r="E15" s="32">
-        <f>MIN(Assumptions!B23*Assumptions!B44,Assumptions!B26)</f>
+        <f>MIN(0.05*Assumptions!B23,Assumptions!B26)</f>
         <v/>
       </c>
       <c r="F15" s="32">
-        <f>MIN(Assumptions!B23*Assumptions!B44,Assumptions!B26)</f>
+        <f>MIN(0.05*Assumptions!B23,Assumptions!B26)</f>
         <v/>
       </c>
       <c r="G15" s="32">
@@ -6216,34 +6216,34 @@
       </c>
       <c r="H15" s="10" t="inlineStr">
         <is>
-          <t>Low scenario × 5yr</t>
+          <t>5% × $3M revenue target × 5 yrs; $300K/yr cap → $150K/yr → $750K total</t>
         </is>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="59" t="inlineStr">
         <is>
-          <t>Tank earn-out high (i): 7%/yr × 5yr (cap $300K)</t>
+          <t>Tank earn-out high (i): 5%/yr × $6M+/yr target × 5yr (cap $300K)</t>
         </is>
       </c>
       <c r="B16" s="32">
-        <f>MIN(Assumptions!B25*Assumptions!B44,Assumptions!B26)</f>
+        <f>MIN(0.05*Assumptions!B25,Assumptions!B26)</f>
         <v/>
       </c>
       <c r="C16" s="32">
-        <f>MIN(Assumptions!B25*Assumptions!B44,Assumptions!B26)</f>
+        <f>MIN(0.05*Assumptions!B25,Assumptions!B26)</f>
         <v/>
       </c>
       <c r="D16" s="32">
-        <f>MIN(Assumptions!B25*Assumptions!B44,Assumptions!B26)</f>
+        <f>MIN(0.05*Assumptions!B25,Assumptions!B26)</f>
         <v/>
       </c>
       <c r="E16" s="32">
-        <f>MIN(Assumptions!B25*Assumptions!B44,Assumptions!B26)</f>
+        <f>MIN(0.05*Assumptions!B25,Assumptions!B26)</f>
         <v/>
       </c>
       <c r="F16" s="32">
-        <f>MIN(Assumptions!B25*Assumptions!B44,Assumptions!B26)</f>
+        <f>MIN(0.05*Assumptions!B25,Assumptions!B26)</f>
         <v/>
       </c>
       <c r="G16" s="32">
@@ -6252,7 +6252,7 @@
       </c>
       <c r="H16" s="10" t="inlineStr">
         <is>
-          <t>High — capped at $300K/yr × 5yr = $1.5M</t>
+          <t>5% × $6M revenue target × 5 yrs; $300K/yr cap → $300K/yr (capped) → $1.5M total</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
SSLC r2: remove SSLC debts at face ($500K) from all outputs
Per John 10/10: SSLC debts NOT assumed by Exos at close.

Changes:
- Assumptions!B14 = 0 (was $500K)
- ① $4.36M → $3.86M | ② $5.36M → $4.86M
- ③ LOW/BASE/HIGH: $6.31M/$7.885M/$9.46M → $5.81M/$7.385M/$8.96M
- ④ hold to 2031: $12.0M/$15.8M/$19.4M → $11.5M/$15.3M/$18.9M
- Earn-out totals unchanged ($950K/$2,525K/$4,100K = ③ - ②)

Artifacts updated: xlsx model, r2 pptx deck, offer summary docx,
briefing email docx. Scripts updated in parallel (do NOT re-run model script).
</commit_message>
<xml_diff>
--- a/drafts/EXOS_SSLC_OptionB_Acquisition_Model_2026-10-07.xlsx
+++ b/drafts/EXOS_SSLC_OptionB_Acquisition_Model_2026-10-07.xlsx
@@ -1306,11 +1306,11 @@
         </is>
       </c>
       <c r="B14" s="8" t="n">
-        <v>500000</v>
+        <v>0</v>
       </c>
       <c r="C14" s="7" t="inlineStr">
         <is>
-          <t>MANAGEMENT ASSUMPTION — UNVERIFIED. QB session expired 10/7. Microcosm loan + Wertz notes + AP.</t>
+          <t>REMOVED per John 10/10: SSLC debts NOT assumed at close. Was $500K TBV — debt payoff is SSLC's responsibility, not part of Exos offer.</t>
         </is>
       </c>
     </row>
@@ -2471,12 +2471,12 @@
       </c>
       <c r="B106" s="5" t="inlineStr">
         <is>
-          <t>~$500K TBV</t>
+          <t>$0 — Exos not assuming SSLC debts</t>
         </is>
       </c>
       <c r="C106" s="7" t="inlineStr">
         <is>
-          <t>Microcosm/Wertz notes + AP paid; personal path for Jim</t>
+          <t>Removed 10/10: SSLC debts at face excluded from Exos offer.</t>
         </is>
       </c>
     </row>
@@ -2958,10 +2958,11 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t>Option B: invoke §3 exclusivity at $3.36M base + earn-out (IM tank revenue and/or Exos stock post-listing). SSLC debts paid at face. DRAFT — negotiation-stage terms.</t>
-        </is>
-      </c>
-    </row>
+          <t>Option B: invoke §3 exclusivity at $3.36M base + earn-out (IM tank revenue and/or Exos stock post-listing). DRAFT — negotiation-stage terms.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="23" t="inlineStr">
         <is>
@@ -3039,7 +3040,7 @@
       </c>
       <c r="E9" s="10" t="inlineStr">
         <is>
-          <t>Microcosm/Wertz notes + AP — TO VERIFY IN SSLC QB</t>
+          <t>Removed 10/10: Exos NOT assuming SSLC debts. Verify remains as SSLC's own responsibility.</t>
         </is>
       </c>
     </row>
@@ -3183,6 +3184,7 @@
         </is>
       </c>
     </row>
+    <row r="20"/>
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="23" t="inlineStr">
         <is>
@@ -3368,6 +3370,7 @@
         </is>
       </c>
     </row>
+    <row r="29"/>
     <row r="30">
       <c r="A30" s="23" t="inlineStr">
         <is>
@@ -5775,7 +5778,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>~$500K est. — TO VERIFY</t>
+          <t>~$500K est. — Exos NOT assuming at close. SSLC's own liability.</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
@@ -5792,7 +5795,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>TO VERIFY IN SSLC QB</t>
+          <t>N/A — Exos not assuming SSLC debts (removed 10/10)</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
@@ -5865,6 +5868,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="54" t="inlineStr">
         <is>
@@ -6137,7 +6141,7 @@
       </c>
       <c r="H12" s="10" t="inlineStr">
         <is>
-          <t>All at close in FY27; includes $1.0M EAI equity at 409A (Rule 504); total ②=$5,360K</t>
+          <t>All at close in FY27; includes $1.0M EAI equity at 409A (Rule 504); total ②=$4,860K</t>
         </is>
       </c>
     </row>
@@ -6445,6 +6449,8 @@
         </is>
       </c>
     </row>
+    <row r="23"/>
+    <row r="24"/>
     <row r="25">
       <c r="A25" s="13" t="inlineStr">
         <is>
@@ -6455,7 +6461,7 @@
     <row r="26" ht="20" customHeight="1">
       <c r="A26" s="27" t="inlineStr">
         <is>
-          <t>BASE: funding+$1M EAI ($5.36M) + tank base (5yr) + milestones 1-3 + stock earn-out base ≈ $7.885M</t>
+          <t>BASE: funding+$1M EAI ($4.86M) + tank base (5yr) + milestones 1-3 + stock earn-out base ≈ $7.385M</t>
         </is>
       </c>
       <c r="B26" s="63">
@@ -6486,7 +6492,7 @@
     <row r="27" ht="20" customHeight="1">
       <c r="A27" s="64" t="inlineStr">
         <is>
-          <t>LOW:  funding+$1M EAI ($5.36M) + tank low (5yr) + milestone M1 only + 0% earn-out ≈ $6.31M</t>
+          <t>LOW:  funding+$1M EAI ($4.86M) + tank low (5yr) + milestone M1 only + 0% earn-out ≈ $5.81M</t>
         </is>
       </c>
       <c r="B27" s="65">
@@ -6517,7 +6523,7 @@
     <row r="28" ht="20" customHeight="1">
       <c r="A28" s="66" t="inlineStr">
         <is>
-          <t>HIGH: funding+$1M EAI ($5.36M) + tank high + all milestones + 0.5% earn-out ≈ $9.46M [HIGH &lt; $10M target — not rebalanced per 10/9 instruction]</t>
+          <t>HIGH: funding+$1M EAI ($4.86M) + tank high + all milestones + 0.5% earn-out ≈ $8.96M [HIGH &lt; $10M target — not rebalanced per 10/10 instruction]</t>
         </is>
       </c>
       <c r="B28" s="67">
@@ -6576,6 +6582,7 @@
         <v/>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="10" t="inlineStr">
         <is>
@@ -6583,6 +6590,7 @@
         </is>
       </c>
     </row>
+    <row r="32"/>
     <row r="33">
       <c r="A33" s="13" t="inlineStr">
         <is>
@@ -6827,6 +6835,7 @@
         </is>
       </c>
     </row>
+    <row r="42"/>
     <row r="43" ht="42" customHeight="1">
       <c r="A43" s="74" t="inlineStr">
         <is>
@@ -8247,7 +8256,7 @@
     <row r="18" ht="16" customHeight="1">
       <c r="A18" s="114" t="inlineStr">
         <is>
-          <t>Exos offer provides: Cash at close $2.51M | Debts paid at face | WC bridge ($300–700K) | Exos channel + IM ramp capex | v12 tank-unit/ASP ramp model. Figures: v12 Annual P&amp;L, recalculated 2026-10-07.</t>
+          <t>Exos offer provides: Cash at close $2.51M | WC bridge ($300–700K) | Exos channel + IM ramp capex | v12 tank-unit/ASP ramp model. Figures: v12 Annual P&amp;L, recalculated 2026-10-07.</t>
         </is>
       </c>
       <c r="H18" s="103" t="inlineStr">
@@ -8367,7 +8376,7 @@
       </c>
       <c r="H22" s="103" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SSLC debts paid at face (est. ~$500K TBV)</t>
+          <t xml:space="preserve">  Prepaid-work delivery funded (cost $500K)</t>
         </is>
       </c>
       <c r="I22" s="142" t="n"/>
@@ -8398,7 +8407,7 @@
       </c>
       <c r="H23" s="103" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Prepaid-work delivery funded (cost $500K)</t>
+          <t xml:space="preserve">  Exos channel access + IM ramp capex + Series A backing</t>
         </is>
       </c>
       <c r="I23" s="142" t="n"/>

</xml_diff>